<commit_message>
LED Glass pipe link added
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/eSpark BOM_Top (20 Boards).xlsx
+++ b/Deliverables/SM_Top Board/_BOM/eSpark BOM_Top (20 Boards).xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="471">
   <si>
     <t>Component list</t>
   </si>
@@ -1558,6 +1558,24 @@
       </rPr>
       <t xml:space="preserve"> Cx1, Cx2</t>
     </r>
+  </si>
+  <si>
+    <t>LED Glass Pipe</t>
+  </si>
+  <si>
+    <t>LED Light Pipes PCB Mount</t>
+  </si>
+  <si>
+    <t>3mm .5 inch</t>
+  </si>
+  <si>
+    <t>VBL3D0500C</t>
+  </si>
+  <si>
+    <t>VCC</t>
+  </si>
+  <si>
+    <t>Mounting Holes required in design</t>
   </si>
 </sst>
 </file>
@@ -2064,7 +2082,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -2376,9 +2394,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2738,7 +2753,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AB89"/>
+  <dimension ref="A1:R90"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="3.109375" style="25" customWidth="1"/>
@@ -2769,14 +2784,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
+      <c r="K1" s="115"/>
+      <c r="L1" s="115"/>
+      <c r="M1" s="115"/>
+      <c r="N1" s="115"/>
+      <c r="O1" s="115"/>
+      <c r="P1" s="115"/>
+      <c r="Q1" s="115"/>
+      <c r="R1" s="115"/>
     </row>
     <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -2824,7 +2839,7 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="117"/>
+      <c r="R3" s="116"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -2848,7 +2863,7 @@
       <c r="O4" s="61"/>
       <c r="P4" s="61"/>
       <c r="Q4" s="61"/>
-      <c r="R4" s="118"/>
+      <c r="R4" s="117"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
@@ -2870,7 +2885,7 @@
       <c r="O5" s="61"/>
       <c r="P5" s="61"/>
       <c r="Q5" s="61"/>
-      <c r="R5" s="118"/>
+      <c r="R5" s="117"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -2890,7 +2905,7 @@
       <c r="O6" s="61"/>
       <c r="P6" s="61"/>
       <c r="Q6" s="61"/>
-      <c r="R6" s="118"/>
+      <c r="R6" s="117"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -2910,7 +2925,7 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="118"/>
+      <c r="R7" s="117"/>
     </row>
     <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
@@ -2930,7 +2945,7 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="118"/>
+      <c r="R8" s="117"/>
     </row>
     <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
@@ -3044,7 +3059,7 @@
     <row r="11" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="53">
-        <f t="shared" ref="B11:B87" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B88" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="81" t="s">
@@ -3135,7 +3150,7 @@
         <v>2</v>
       </c>
       <c r="M12" s="41">
-        <f t="shared" ref="M12:M69" si="1">L12*20</f>
+        <f t="shared" ref="M12:M70" si="1">L12*20</f>
         <v>40</v>
       </c>
       <c r="N12" s="41">
@@ -4965,2700 +4980,2402 @@
         <v>0.08</v>
       </c>
       <c r="Q45" s="109">
-        <f t="shared" ref="Q45" si="34">P45*N45</f>
+        <f t="shared" ref="Q45:Q46" si="34">P45*N45</f>
         <v>2.4</v>
       </c>
       <c r="R45" s="109"/>
     </row>
     <row r="46" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
-      <c r="B46" s="113">
-        <f t="shared" si="0"/>
+      <c r="B46" s="53">
         <v>37</v>
       </c>
-      <c r="C46" s="102" t="s">
-        <v>320</v>
-      </c>
-      <c r="D46" s="103" t="s">
-        <v>33</v>
-      </c>
-      <c r="E46" s="104" t="s">
-        <v>101</v>
-      </c>
-      <c r="F46" s="103" t="s">
-        <v>308</v>
-      </c>
-      <c r="G46" s="104" t="s">
-        <v>162</v>
-      </c>
-      <c r="H46" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="I46" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J46" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="K46" s="104" t="s">
-        <v>314</v>
-      </c>
-      <c r="L46" s="103">
-        <v>2</v>
-      </c>
-      <c r="M46" s="96">
+      <c r="C46" s="106" t="s">
+        <v>465</v>
+      </c>
+      <c r="D46" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="E46" s="108" t="s">
+        <v>466</v>
+      </c>
+      <c r="F46" s="107" t="s">
+        <v>467</v>
+      </c>
+      <c r="G46" s="108" t="s">
+        <v>468</v>
+      </c>
+      <c r="H46" s="107" t="s">
+        <v>469</v>
+      </c>
+      <c r="I46" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J46" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="K46" s="108" t="s">
+        <v>314</v>
+      </c>
+      <c r="L46" s="107">
+        <v>1</v>
+      </c>
+      <c r="M46" s="109">
         <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="N46" s="96">
-        <v>50</v>
-      </c>
-      <c r="O46" s="105" t="s">
+        <v>20</v>
+      </c>
+      <c r="N46" s="109">
+        <v>20</v>
+      </c>
+      <c r="O46" s="110" t="s">
         <v>379</v>
       </c>
-      <c r="P46" s="96">
-        <v>1.5</v>
-      </c>
-      <c r="Q46" s="96">
-        <f t="shared" ref="Q46" si="35">N46*P46</f>
-        <v>75</v>
-      </c>
-      <c r="R46" s="96"/>
+      <c r="P46" s="109">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="Q46" s="109">
+        <f t="shared" si="34"/>
+        <v>9.24</v>
+      </c>
+      <c r="R46" s="109" t="s">
+        <v>470</v>
+      </c>
     </row>
     <row r="47" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1"/>
       <c r="B47" s="53">
-        <f>ROW(B47) - ROW($B$9)</f>
+        <f t="shared" ref="B47:B88" si="35">ROW(B47) - ROW($B$9)</f>
         <v>38</v>
       </c>
-      <c r="C47" s="97" t="s">
-        <v>283</v>
-      </c>
-      <c r="D47" s="98" t="s">
-        <v>34</v>
-      </c>
-      <c r="E47" s="99" t="s">
-        <v>102</v>
-      </c>
-      <c r="F47" s="98" t="s">
-        <v>163</v>
-      </c>
-      <c r="G47" s="99" t="s">
-        <v>314</v>
-      </c>
-      <c r="H47" s="98" t="s">
-        <v>314</v>
-      </c>
-      <c r="I47" s="98"/>
-      <c r="J47" s="98"/>
-      <c r="K47" s="99" t="s">
-        <v>314</v>
-      </c>
-      <c r="L47" s="98">
-        <v>4</v>
-      </c>
-      <c r="M47" s="66">
+      <c r="C47" s="102" t="s">
+        <v>320</v>
+      </c>
+      <c r="D47" s="103" t="s">
+        <v>33</v>
+      </c>
+      <c r="E47" s="104" t="s">
+        <v>101</v>
+      </c>
+      <c r="F47" s="103" t="s">
+        <v>308</v>
+      </c>
+      <c r="G47" s="104" t="s">
+        <v>162</v>
+      </c>
+      <c r="H47" s="103" t="s">
+        <v>247</v>
+      </c>
+      <c r="I47" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J47" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="K47" s="104" t="s">
+        <v>314</v>
+      </c>
+      <c r="L47" s="103">
+        <v>2</v>
+      </c>
+      <c r="M47" s="96">
         <f t="shared" si="1"/>
-        <v>80</v>
-      </c>
-      <c r="N47" s="66">
-        <f t="shared" ref="N47" si="36">M47+(M47*0.1)</f>
-        <v>88</v>
-      </c>
-      <c r="O47" s="66"/>
-      <c r="P47" s="66"/>
-      <c r="Q47" s="66">
-        <f t="shared" ref="Q47" si="37">P47*N47</f>
-        <v>0</v>
-      </c>
-      <c r="R47" s="66" t="s">
-        <v>384</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="N47" s="96">
+        <v>50</v>
+      </c>
+      <c r="O47" s="105" t="s">
+        <v>379</v>
+      </c>
+      <c r="P47" s="96">
+        <v>1.5</v>
+      </c>
+      <c r="Q47" s="96">
+        <f t="shared" ref="Q47" si="36">N47*P47</f>
+        <v>75</v>
+      </c>
+      <c r="R47" s="96"/>
     </row>
     <row r="48" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1"/>
       <c r="B48" s="53">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-      <c r="C48" s="102" t="s">
-        <v>321</v>
-      </c>
-      <c r="D48" s="103" t="s">
-        <v>35</v>
-      </c>
-      <c r="E48" s="104" t="s">
-        <v>103</v>
-      </c>
-      <c r="F48" s="103" t="s">
-        <v>164</v>
-      </c>
-      <c r="G48" s="104">
-        <v>61300211121</v>
-      </c>
-      <c r="H48" s="103" t="s">
-        <v>235</v>
-      </c>
-      <c r="I48" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J48" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="K48" s="104" t="s">
-        <v>314</v>
-      </c>
-      <c r="L48" s="103">
+        <v>38</v>
+      </c>
+      <c r="C48" s="97" t="s">
+        <v>283</v>
+      </c>
+      <c r="D48" s="98" t="s">
+        <v>34</v>
+      </c>
+      <c r="E48" s="99" t="s">
+        <v>102</v>
+      </c>
+      <c r="F48" s="98" t="s">
+        <v>163</v>
+      </c>
+      <c r="G48" s="99" t="s">
+        <v>314</v>
+      </c>
+      <c r="H48" s="98" t="s">
+        <v>314</v>
+      </c>
+      <c r="I48" s="98"/>
+      <c r="J48" s="98"/>
+      <c r="K48" s="99" t="s">
+        <v>314</v>
+      </c>
+      <c r="L48" s="98">
         <v>4</v>
       </c>
-      <c r="M48" s="96">
+      <c r="M48" s="66">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="N48" s="96">
-        <v>90</v>
-      </c>
-      <c r="O48" s="105" t="s">
-        <v>379</v>
-      </c>
-      <c r="P48" s="96">
-        <v>0.13</v>
-      </c>
-      <c r="Q48" s="96">
-        <f t="shared" ref="Q48" si="38">N48*P48</f>
-        <v>11.700000000000001</v>
-      </c>
-      <c r="R48" s="96"/>
+      <c r="N48" s="66">
+        <f t="shared" ref="N48" si="37">M48+(M48*0.1)</f>
+        <v>88</v>
+      </c>
+      <c r="O48" s="66"/>
+      <c r="P48" s="66"/>
+      <c r="Q48" s="66">
+        <f t="shared" ref="Q48" si="38">P48*N48</f>
+        <v>0</v>
+      </c>
+      <c r="R48" s="66" t="s">
+        <v>384</v>
+      </c>
     </row>
     <row r="49" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1"/>
       <c r="B49" s="53">
-        <f>ROW(B49) - ROW($B$9)</f>
+        <f t="shared" ref="B49:B88" si="39">ROW(B49) - ROW($B$9)</f>
         <v>40</v>
       </c>
-      <c r="C49" s="106" t="s">
-        <v>323</v>
-      </c>
-      <c r="D49" s="107" t="s">
-        <v>439</v>
-      </c>
-      <c r="E49" s="108" t="s">
-        <v>104</v>
-      </c>
-      <c r="F49" s="107" t="s">
-        <v>165</v>
-      </c>
-      <c r="G49" s="108" t="s">
-        <v>200</v>
-      </c>
-      <c r="H49" s="107" t="s">
-        <v>248</v>
-      </c>
-      <c r="I49" s="107" t="s">
-        <v>385</v>
-      </c>
-      <c r="J49" s="107" t="s">
-        <v>386</v>
-      </c>
-      <c r="K49" s="108" t="s">
-        <v>314</v>
-      </c>
-      <c r="L49" s="107">
+      <c r="C49" s="102" t="s">
+        <v>321</v>
+      </c>
+      <c r="D49" s="103" t="s">
+        <v>35</v>
+      </c>
+      <c r="E49" s="104" t="s">
+        <v>103</v>
+      </c>
+      <c r="F49" s="103" t="s">
+        <v>164</v>
+      </c>
+      <c r="G49" s="104">
+        <v>61300211121</v>
+      </c>
+      <c r="H49" s="103" t="s">
+        <v>235</v>
+      </c>
+      <c r="I49" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J49" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="K49" s="104" t="s">
+        <v>314</v>
+      </c>
+      <c r="L49" s="103">
         <v>4</v>
       </c>
-      <c r="M49" s="109">
+      <c r="M49" s="96">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="N49" s="109">
-        <v>85</v>
-      </c>
-      <c r="O49" s="110" t="s">
-        <v>343</v>
-      </c>
-      <c r="P49" s="109">
-        <v>0.21740000000000001</v>
-      </c>
-      <c r="Q49" s="109">
-        <f t="shared" ref="Q49" si="39">P49*N49</f>
-        <v>18.478999999999999</v>
-      </c>
-      <c r="R49" s="109"/>
+      <c r="N49" s="96">
+        <v>90</v>
+      </c>
+      <c r="O49" s="105" t="s">
+        <v>379</v>
+      </c>
+      <c r="P49" s="96">
+        <v>0.13</v>
+      </c>
+      <c r="Q49" s="96">
+        <f t="shared" ref="Q49" si="40">N49*P49</f>
+        <v>11.700000000000001</v>
+      </c>
+      <c r="R49" s="96"/>
     </row>
     <row r="50" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1"/>
       <c r="B50" s="53">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-      <c r="C50" s="102" t="s">
+        <v>39</v>
+      </c>
+      <c r="C50" s="106" t="s">
+        <v>323</v>
+      </c>
+      <c r="D50" s="107" t="s">
+        <v>439</v>
+      </c>
+      <c r="E50" s="108" t="s">
+        <v>104</v>
+      </c>
+      <c r="F50" s="107" t="s">
+        <v>165</v>
+      </c>
+      <c r="G50" s="108" t="s">
+        <v>200</v>
+      </c>
+      <c r="H50" s="107" t="s">
+        <v>248</v>
+      </c>
+      <c r="I50" s="107" t="s">
+        <v>385</v>
+      </c>
+      <c r="J50" s="107" t="s">
+        <v>386</v>
+      </c>
+      <c r="K50" s="108" t="s">
+        <v>314</v>
+      </c>
+      <c r="L50" s="107">
+        <v>4</v>
+      </c>
+      <c r="M50" s="109">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+      <c r="N50" s="109">
+        <v>85</v>
+      </c>
+      <c r="O50" s="110" t="s">
+        <v>343</v>
+      </c>
+      <c r="P50" s="109">
+        <v>0.21740000000000001</v>
+      </c>
+      <c r="Q50" s="109">
+        <f t="shared" ref="Q50" si="41">P50*N50</f>
+        <v>18.478999999999999</v>
+      </c>
+      <c r="R50" s="109"/>
+    </row>
+    <row r="51" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="1"/>
+      <c r="B51" s="53">
+        <f t="shared" ref="B51:B88" si="42">ROW(B51) - ROW($B$9)</f>
+        <v>42</v>
+      </c>
+      <c r="C51" s="102" t="s">
         <v>324</v>
       </c>
-      <c r="D50" s="103" t="s">
+      <c r="D51" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="E50" s="104" t="s">
+      <c r="E51" s="104" t="s">
         <v>105</v>
       </c>
-      <c r="F50" s="103" t="s">
+      <c r="F51" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="G50" s="104" t="s">
+      <c r="G51" s="104" t="s">
         <v>201</v>
       </c>
-      <c r="H50" s="103" t="s">
+      <c r="H51" s="103" t="s">
         <v>229</v>
       </c>
-      <c r="I50" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J50" s="103" t="s">
+      <c r="I51" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J51" s="103" t="s">
         <v>387</v>
       </c>
-      <c r="K50" s="104" t="s">
+      <c r="K51" s="104" t="s">
         <v>284</v>
       </c>
-      <c r="L50" s="103">
+      <c r="L51" s="103">
         <v>2</v>
       </c>
-      <c r="M50" s="96">
+      <c r="M51" s="96">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N50" s="96">
+      <c r="N51" s="96">
         <v>100</v>
       </c>
-      <c r="O50" s="105" t="s">
+      <c r="O51" s="105" t="s">
         <v>343</v>
       </c>
-      <c r="P50" s="96">
+      <c r="P51" s="96">
         <v>1E-3</v>
       </c>
-      <c r="Q50" s="96">
-        <f t="shared" ref="Q50" si="40">N50*P50</f>
+      <c r="Q51" s="96">
+        <f t="shared" ref="Q51" si="43">N51*P51</f>
         <v>0.1</v>
       </c>
-      <c r="R50" s="96"/>
-    </row>
-    <row r="51" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="1"/>
-      <c r="B51" s="53">
-        <f>ROW(B51) - ROW($B$9)</f>
-        <v>42</v>
-      </c>
-      <c r="C51" s="106" t="s">
+      <c r="R51" s="96"/>
+    </row>
+    <row r="52" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="1"/>
+      <c r="B52" s="53">
+        <v>40</v>
+      </c>
+      <c r="C52" s="106" t="s">
         <v>324</v>
       </c>
-      <c r="D51" s="107" t="s">
+      <c r="D52" s="107" t="s">
         <v>37</v>
       </c>
-      <c r="E51" s="108" t="s">
+      <c r="E52" s="108" t="s">
         <v>106</v>
       </c>
-      <c r="F51" s="107" t="s">
+      <c r="F52" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="G51" s="108" t="s">
+      <c r="G52" s="108" t="s">
         <v>202</v>
       </c>
-      <c r="H51" s="107" t="s">
+      <c r="H52" s="107" t="s">
         <v>229</v>
       </c>
-      <c r="I51" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J51" s="107" t="s">
+      <c r="I52" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J52" s="107" t="s">
         <v>388</v>
       </c>
-      <c r="K51" s="108" t="s">
+      <c r="K52" s="108" t="s">
         <v>285</v>
       </c>
-      <c r="L51" s="107">
+      <c r="L52" s="107">
         <v>1</v>
       </c>
-      <c r="M51" s="109">
+      <c r="M52" s="109">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N51" s="109">
+      <c r="N52" s="109">
         <v>100</v>
       </c>
-      <c r="O51" s="110" t="s">
+      <c r="O52" s="110" t="s">
         <v>343</v>
       </c>
-      <c r="P51" s="109">
+      <c r="P52" s="109">
         <v>1.4E-3</v>
       </c>
-      <c r="Q51" s="109">
-        <f t="shared" ref="Q51" si="41">P51*N51</f>
+      <c r="Q52" s="109">
+        <f t="shared" ref="Q52" si="44">P52*N52</f>
         <v>0.13999999999999999</v>
       </c>
-      <c r="R51" s="109"/>
-    </row>
-    <row r="52" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="1"/>
-      <c r="B52" s="53">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-      <c r="C52" s="102" t="s">
+      <c r="R52" s="109"/>
+    </row>
+    <row r="53" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="1"/>
+      <c r="B53" s="53">
+        <f t="shared" ref="B53:B88" si="45">ROW(B53) - ROW($B$9)</f>
+        <v>44</v>
+      </c>
+      <c r="C53" s="102" t="s">
         <v>324</v>
       </c>
-      <c r="D52" s="103" t="s">
+      <c r="D53" s="103" t="s">
         <v>38</v>
       </c>
-      <c r="E52" s="104" t="s">
+      <c r="E53" s="104" t="s">
         <v>107</v>
       </c>
-      <c r="F52" s="103" t="s">
+      <c r="F53" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="G52" s="104" t="s">
+      <c r="G53" s="104" t="s">
         <v>203</v>
       </c>
-      <c r="H52" s="103" t="s">
+      <c r="H53" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="I52" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J52" s="103" t="s">
+      <c r="I53" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J53" s="103" t="s">
         <v>389</v>
       </c>
-      <c r="K52" s="104" t="s">
+      <c r="K53" s="104" t="s">
         <v>286</v>
       </c>
-      <c r="L52" s="103">
+      <c r="L53" s="103">
         <v>1</v>
       </c>
-      <c r="M52" s="96">
+      <c r="M53" s="96">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N52" s="96">
+      <c r="N53" s="96">
         <v>100</v>
       </c>
-      <c r="O52" s="105" t="s">
+      <c r="O53" s="105" t="s">
         <v>343</v>
       </c>
-      <c r="P52" s="96">
+      <c r="P53" s="96">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="Q52" s="96">
-        <f t="shared" ref="Q52" si="42">N52*P52</f>
+      <c r="Q53" s="96">
+        <f t="shared" ref="Q53" si="46">N53*P53</f>
         <v>0.16</v>
       </c>
-      <c r="R52" s="96"/>
-    </row>
-    <row r="53" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="1"/>
-      <c r="B53" s="53">
-        <f>ROW(B53) - ROW($B$9)</f>
-        <v>44</v>
-      </c>
-      <c r="C53" s="106" t="s">
-        <v>324</v>
-      </c>
-      <c r="D53" s="107" t="s">
-        <v>39</v>
-      </c>
-      <c r="E53" s="108" t="s">
-        <v>108</v>
-      </c>
-      <c r="F53" s="107" t="s">
-        <v>166</v>
-      </c>
-      <c r="G53" s="108" t="s">
-        <v>204</v>
-      </c>
-      <c r="H53" s="107" t="s">
-        <v>229</v>
-      </c>
-      <c r="I53" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J53" s="107" t="s">
-        <v>390</v>
-      </c>
-      <c r="K53" s="108" t="s">
-        <v>287</v>
-      </c>
-      <c r="L53" s="107">
-        <v>2</v>
-      </c>
-      <c r="M53" s="109">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="N53" s="109">
-        <v>100</v>
-      </c>
-      <c r="O53" s="110" t="s">
-        <v>343</v>
-      </c>
-      <c r="P53" s="109">
-        <v>1.4E-3</v>
-      </c>
-      <c r="Q53" s="109">
-        <f t="shared" ref="Q53" si="43">P53*N53</f>
-        <v>0.13999999999999999</v>
-      </c>
-      <c r="R53" s="109"/>
+      <c r="R53" s="96"/>
     </row>
     <row r="54" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1"/>
       <c r="B54" s="53">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-      <c r="C54" s="102" t="s">
+        <v>41</v>
+      </c>
+      <c r="C54" s="106" t="s">
         <v>324</v>
       </c>
-      <c r="D54" s="103" t="s">
+      <c r="D54" s="107" t="s">
+        <v>39</v>
+      </c>
+      <c r="E54" s="108" t="s">
+        <v>108</v>
+      </c>
+      <c r="F54" s="107" t="s">
+        <v>166</v>
+      </c>
+      <c r="G54" s="108" t="s">
+        <v>204</v>
+      </c>
+      <c r="H54" s="107" t="s">
+        <v>229</v>
+      </c>
+      <c r="I54" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J54" s="107" t="s">
+        <v>390</v>
+      </c>
+      <c r="K54" s="108" t="s">
+        <v>287</v>
+      </c>
+      <c r="L54" s="107">
+        <v>2</v>
+      </c>
+      <c r="M54" s="109">
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="E54" s="104" t="s">
+      <c r="N54" s="109">
+        <v>100</v>
+      </c>
+      <c r="O54" s="110" t="s">
+        <v>343</v>
+      </c>
+      <c r="P54" s="109">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q54" s="109">
+        <f t="shared" ref="Q54" si="47">P54*N54</f>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="R54" s="109"/>
+    </row>
+    <row r="55" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="1"/>
+      <c r="B55" s="53">
+        <f t="shared" ref="B55:B88" si="48">ROW(B55) - ROW($B$9)</f>
+        <v>46</v>
+      </c>
+      <c r="C55" s="102" t="s">
+        <v>324</v>
+      </c>
+      <c r="D55" s="103" t="s">
+        <v>40</v>
+      </c>
+      <c r="E55" s="104" t="s">
         <v>109</v>
       </c>
-      <c r="F54" s="103" t="s">
+      <c r="F55" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="G54" s="104" t="s">
+      <c r="G55" s="104" t="s">
         <v>205</v>
       </c>
-      <c r="H54" s="103" t="s">
+      <c r="H55" s="103" t="s">
         <v>229</v>
       </c>
-      <c r="I54" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J54" s="103" t="s">
+      <c r="I55" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J55" s="103" t="s">
         <v>391</v>
       </c>
-      <c r="K54" s="104" t="s">
+      <c r="K55" s="104" t="s">
         <v>288</v>
       </c>
-      <c r="L54" s="103">
+      <c r="L55" s="103">
         <v>4</v>
       </c>
-      <c r="M54" s="96">
+      <c r="M55" s="96">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="N54" s="96">
+      <c r="N55" s="96">
         <v>100</v>
       </c>
-      <c r="O54" s="105" t="s">
+      <c r="O55" s="105" t="s">
         <v>343</v>
       </c>
-      <c r="P54" s="96">
+      <c r="P55" s="96">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="Q54" s="96">
-        <f t="shared" ref="Q54" si="44">N54*P54</f>
+      <c r="Q55" s="96">
+        <f t="shared" ref="Q55" si="49">N55*P55</f>
         <v>0.13</v>
       </c>
-      <c r="R54" s="96"/>
-    </row>
-    <row r="55" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="1"/>
-      <c r="B55" s="53">
-        <f>ROW(B55) - ROW($B$9)</f>
-        <v>46</v>
-      </c>
-      <c r="C55" s="106" t="s">
+      <c r="R55" s="96"/>
+    </row>
+    <row r="56" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="1"/>
+      <c r="B56" s="53">
+        <v>42</v>
+      </c>
+      <c r="C56" s="106" t="s">
         <v>324</v>
       </c>
-      <c r="D55" s="107" t="s">
+      <c r="D56" s="107" t="s">
         <v>41</v>
       </c>
-      <c r="E55" s="108" t="s">
+      <c r="E56" s="108" t="s">
         <v>110</v>
       </c>
-      <c r="F55" s="107" t="s">
+      <c r="F56" s="107" t="s">
         <v>167</v>
       </c>
-      <c r="G55" s="108" t="s">
+      <c r="G56" s="108" t="s">
         <v>329</v>
       </c>
-      <c r="H55" s="107" t="s">
+      <c r="H56" s="107" t="s">
         <v>250</v>
       </c>
-      <c r="I55" s="107" t="s">
+      <c r="I56" s="107" t="s">
         <v>392</v>
       </c>
-      <c r="J55" s="107" t="s">
+      <c r="J56" s="107" t="s">
         <v>393</v>
       </c>
-      <c r="K55" s="108" t="s">
+      <c r="K56" s="108" t="s">
         <v>289</v>
       </c>
-      <c r="L55" s="107">
+      <c r="L56" s="107">
         <v>4</v>
       </c>
-      <c r="M55" s="109">
+      <c r="M56" s="109">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="N55" s="109">
+      <c r="N56" s="109">
         <v>90</v>
       </c>
-      <c r="O55" s="110" t="s">
+      <c r="O56" s="110" t="s">
         <v>343</v>
       </c>
-      <c r="P55" s="109">
+      <c r="P56" s="109">
         <v>6.4500000000000002E-2</v>
       </c>
-      <c r="Q55" s="109">
-        <f t="shared" ref="Q55" si="45">P55*N55</f>
+      <c r="Q56" s="109">
+        <f t="shared" ref="Q56" si="50">P56*N56</f>
         <v>5.8049999999999997</v>
       </c>
-      <c r="R55" s="109"/>
-    </row>
-    <row r="56" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="1"/>
-      <c r="B56" s="53">
-        <f>ROW(B56) - ROW($B$9)</f>
-        <v>47</v>
-      </c>
-      <c r="C56" s="60" t="s">
-        <v>324</v>
-      </c>
-      <c r="D56" s="37" t="s">
-        <v>423</v>
-      </c>
-      <c r="E56" s="37" t="s">
-        <v>440</v>
-      </c>
-      <c r="F56" s="37" t="s">
-        <v>166</v>
-      </c>
-      <c r="G56" s="37" t="s">
-        <v>425</v>
-      </c>
-      <c r="H56" s="37" t="s">
-        <v>252</v>
-      </c>
-      <c r="I56" s="37" t="s">
-        <v>314</v>
-      </c>
-      <c r="J56" s="37" t="s">
-        <v>426</v>
-      </c>
-      <c r="K56" s="37" t="s">
-        <v>427</v>
-      </c>
-      <c r="L56" s="37">
-        <v>8</v>
-      </c>
-      <c r="M56" s="37">
-        <f t="shared" si="1"/>
-        <v>160</v>
-      </c>
-      <c r="N56" s="96">
-        <v>100</v>
-      </c>
-      <c r="O56" s="80" t="s">
-        <v>343</v>
-      </c>
-      <c r="P56" s="37">
-        <v>1.1000000000000001E-3</v>
-      </c>
-      <c r="Q56" s="37">
-        <f t="shared" ref="Q56" si="46">N56*P56</f>
-        <v>0.11</v>
-      </c>
-      <c r="R56" s="76"/>
+      <c r="R56" s="109"/>
     </row>
     <row r="57" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1"/>
       <c r="B57" s="53">
-        <f>ROW(B57) - ROW($B$9)</f>
+        <f t="shared" ref="B57:B88" si="51">ROW(B57) - ROW($B$9)</f>
         <v>48</v>
       </c>
-      <c r="C57" s="106" t="s">
+      <c r="C57" s="60" t="s">
         <v>324</v>
       </c>
-      <c r="D57" s="107" t="s">
-        <v>42</v>
-      </c>
-      <c r="E57" s="108" t="s">
-        <v>112</v>
-      </c>
-      <c r="F57" s="107" t="s">
+      <c r="D57" s="37" t="s">
+        <v>423</v>
+      </c>
+      <c r="E57" s="37" t="s">
+        <v>440</v>
+      </c>
+      <c r="F57" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="G57" s="108" t="s">
-        <v>207</v>
-      </c>
-      <c r="H57" s="107" t="s">
-        <v>251</v>
-      </c>
-      <c r="I57" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J57" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="K57" s="108" t="s">
-        <v>291</v>
-      </c>
-      <c r="L57" s="107">
-        <v>1</v>
-      </c>
-      <c r="M57" s="109">
+      <c r="G57" s="37" t="s">
+        <v>425</v>
+      </c>
+      <c r="H57" s="37" t="s">
+        <v>252</v>
+      </c>
+      <c r="I57" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="J57" s="37" t="s">
+        <v>426</v>
+      </c>
+      <c r="K57" s="37" t="s">
+        <v>427</v>
+      </c>
+      <c r="L57" s="37">
+        <v>8</v>
+      </c>
+      <c r="M57" s="37">
         <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N57" s="109">
-        <v>30</v>
-      </c>
-      <c r="O57" s="110" t="s">
-        <v>382</v>
-      </c>
-      <c r="P57" s="109">
-        <v>1.8589999999999999E-2</v>
-      </c>
-      <c r="Q57" s="109">
-        <f t="shared" ref="Q57" si="47">P57*N57</f>
-        <v>0.55769999999999997</v>
-      </c>
-      <c r="R57" s="109"/>
+        <v>160</v>
+      </c>
+      <c r="N57" s="96">
+        <v>100</v>
+      </c>
+      <c r="O57" s="80" t="s">
+        <v>343</v>
+      </c>
+      <c r="P57" s="37">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q57" s="37">
+        <f t="shared" ref="Q57" si="52">N57*P57</f>
+        <v>0.11</v>
+      </c>
+      <c r="R57" s="76"/>
     </row>
     <row r="58" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1"/>
       <c r="B58" s="53">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-      <c r="C58" s="102" t="s">
+        <v>43</v>
+      </c>
+      <c r="C58" s="106" t="s">
         <v>324</v>
       </c>
-      <c r="D58" s="103" t="s">
-        <v>43</v>
-      </c>
-      <c r="E58" s="104" t="s">
-        <v>113</v>
-      </c>
-      <c r="F58" s="103" t="s">
+      <c r="D58" s="107" t="s">
+        <v>42</v>
+      </c>
+      <c r="E58" s="108" t="s">
+        <v>112</v>
+      </c>
+      <c r="F58" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="G58" s="104" t="s">
-        <v>208</v>
-      </c>
-      <c r="H58" s="103" t="s">
-        <v>229</v>
-      </c>
-      <c r="I58" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J58" s="103" t="s">
-        <v>395</v>
-      </c>
-      <c r="K58" s="104" t="s">
-        <v>292</v>
-      </c>
-      <c r="L58" s="103">
+      <c r="G58" s="108" t="s">
+        <v>207</v>
+      </c>
+      <c r="H58" s="107" t="s">
+        <v>251</v>
+      </c>
+      <c r="I58" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J58" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="K58" s="108" t="s">
+        <v>291</v>
+      </c>
+      <c r="L58" s="107">
         <v>1</v>
       </c>
-      <c r="M58" s="96">
+      <c r="M58" s="109">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N58" s="96">
-        <v>100</v>
-      </c>
-      <c r="O58" s="105" t="s">
-        <v>343</v>
-      </c>
-      <c r="P58" s="96">
-        <v>1.4E-3</v>
-      </c>
-      <c r="Q58" s="96">
-        <f t="shared" ref="Q58" si="48">N58*P58</f>
-        <v>0.13999999999999999</v>
-      </c>
-      <c r="R58" s="96"/>
+      <c r="N58" s="109">
+        <v>30</v>
+      </c>
+      <c r="O58" s="110" t="s">
+        <v>382</v>
+      </c>
+      <c r="P58" s="109">
+        <v>1.8589999999999999E-2</v>
+      </c>
+      <c r="Q58" s="109">
+        <f t="shared" ref="Q58" si="53">P58*N58</f>
+        <v>0.55769999999999997</v>
+      </c>
+      <c r="R58" s="109"/>
     </row>
     <row r="59" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1"/>
       <c r="B59" s="53">
-        <f>ROW(B59) - ROW($B$9)</f>
+        <f t="shared" ref="B59:B88" si="54">ROW(B59) - ROW($B$9)</f>
         <v>50</v>
       </c>
-      <c r="C59" s="106" t="s">
+      <c r="C59" s="102" t="s">
         <v>324</v>
       </c>
-      <c r="D59" s="107" t="s">
-        <v>44</v>
-      </c>
-      <c r="E59" s="108" t="s">
-        <v>114</v>
-      </c>
-      <c r="F59" s="107" t="s">
+      <c r="D59" s="103" t="s">
+        <v>43</v>
+      </c>
+      <c r="E59" s="104" t="s">
+        <v>113</v>
+      </c>
+      <c r="F59" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="G59" s="108" t="s">
-        <v>209</v>
-      </c>
-      <c r="H59" s="107" t="s">
-        <v>251</v>
-      </c>
-      <c r="I59" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J59" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="K59" s="108" t="s">
-        <v>293</v>
-      </c>
-      <c r="L59" s="107">
+      <c r="G59" s="104" t="s">
+        <v>208</v>
+      </c>
+      <c r="H59" s="103" t="s">
+        <v>229</v>
+      </c>
+      <c r="I59" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J59" s="103" t="s">
+        <v>395</v>
+      </c>
+      <c r="K59" s="104" t="s">
+        <v>292</v>
+      </c>
+      <c r="L59" s="103">
         <v>1</v>
       </c>
-      <c r="M59" s="109">
+      <c r="M59" s="96">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N59" s="109">
-        <v>50</v>
-      </c>
-      <c r="O59" s="110" t="s">
-        <v>382</v>
-      </c>
-      <c r="P59" s="109">
-        <v>4.6699999999999997E-3</v>
-      </c>
-      <c r="Q59" s="109">
-        <f t="shared" ref="Q59" si="49">P59*N59</f>
-        <v>0.23349999999999999</v>
-      </c>
-      <c r="R59" s="109"/>
+      <c r="N59" s="96">
+        <v>100</v>
+      </c>
+      <c r="O59" s="105" t="s">
+        <v>343</v>
+      </c>
+      <c r="P59" s="96">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q59" s="96">
+        <f t="shared" ref="Q59" si="55">N59*P59</f>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="R59" s="96"/>
     </row>
     <row r="60" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1"/>
       <c r="B60" s="53">
-        <f t="shared" si="0"/>
-        <v>51</v>
-      </c>
-      <c r="C60" s="102" t="s">
+        <v>44</v>
+      </c>
+      <c r="C60" s="106" t="s">
         <v>324</v>
       </c>
-      <c r="D60" s="103" t="s">
-        <v>45</v>
-      </c>
-      <c r="E60" s="104" t="s">
-        <v>115</v>
-      </c>
-      <c r="F60" s="103" t="s">
+      <c r="D60" s="107" t="s">
+        <v>44</v>
+      </c>
+      <c r="E60" s="108" t="s">
+        <v>114</v>
+      </c>
+      <c r="F60" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="G60" s="104" t="s">
-        <v>210</v>
-      </c>
-      <c r="H60" s="103" t="s">
-        <v>229</v>
-      </c>
-      <c r="I60" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J60" s="103" t="s">
-        <v>396</v>
-      </c>
-      <c r="K60" s="104" t="s">
-        <v>294</v>
-      </c>
-      <c r="L60" s="103">
+      <c r="G60" s="108" t="s">
+        <v>209</v>
+      </c>
+      <c r="H60" s="107" t="s">
+        <v>251</v>
+      </c>
+      <c r="I60" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J60" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="K60" s="108" t="s">
+        <v>293</v>
+      </c>
+      <c r="L60" s="107">
         <v>1</v>
       </c>
-      <c r="M60" s="96">
+      <c r="M60" s="109">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N60" s="96">
-        <v>100</v>
-      </c>
-      <c r="O60" s="105" t="s">
-        <v>343</v>
-      </c>
-      <c r="P60" s="96">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="Q60" s="96">
-        <f t="shared" ref="Q60" si="50">N60*P60</f>
-        <v>0.12</v>
-      </c>
-      <c r="R60" s="96"/>
+      <c r="N60" s="109">
+        <v>50</v>
+      </c>
+      <c r="O60" s="110" t="s">
+        <v>382</v>
+      </c>
+      <c r="P60" s="109">
+        <v>4.6699999999999997E-3</v>
+      </c>
+      <c r="Q60" s="109">
+        <f t="shared" ref="Q60" si="56">P60*N60</f>
+        <v>0.23349999999999999</v>
+      </c>
+      <c r="R60" s="109"/>
     </row>
     <row r="61" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1"/>
       <c r="B61" s="53">
-        <f>ROW(B61) - ROW($B$9)</f>
+        <f t="shared" ref="B61:B88" si="57">ROW(B61) - ROW($B$9)</f>
         <v>52</v>
       </c>
-      <c r="C61" s="106" t="s">
+      <c r="C61" s="102" t="s">
         <v>324</v>
       </c>
-      <c r="D61" s="107" t="s">
-        <v>46</v>
-      </c>
-      <c r="E61" s="108" t="s">
-        <v>116</v>
-      </c>
-      <c r="F61" s="107" t="s">
+      <c r="D61" s="103" t="s">
+        <v>45</v>
+      </c>
+      <c r="E61" s="104" t="s">
+        <v>115</v>
+      </c>
+      <c r="F61" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="G61" s="108" t="s">
-        <v>211</v>
-      </c>
-      <c r="H61" s="107" t="s">
-        <v>251</v>
-      </c>
-      <c r="I61" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J61" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="K61" s="108" t="s">
-        <v>295</v>
-      </c>
-      <c r="L61" s="107">
+      <c r="G61" s="104" t="s">
+        <v>210</v>
+      </c>
+      <c r="H61" s="103" t="s">
+        <v>229</v>
+      </c>
+      <c r="I61" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J61" s="103" t="s">
+        <v>396</v>
+      </c>
+      <c r="K61" s="104" t="s">
+        <v>294</v>
+      </c>
+      <c r="L61" s="103">
         <v>1</v>
       </c>
-      <c r="M61" s="109">
+      <c r="M61" s="96">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N61" s="109">
-        <v>50</v>
-      </c>
-      <c r="O61" s="110" t="s">
-        <v>382</v>
-      </c>
-      <c r="P61" s="109">
-        <v>1.11E-2</v>
-      </c>
-      <c r="Q61" s="109">
-        <f t="shared" ref="Q61" si="51">P61*N61</f>
-        <v>0.55500000000000005</v>
-      </c>
-      <c r="R61" s="109"/>
+      <c r="N61" s="96">
+        <v>100</v>
+      </c>
+      <c r="O61" s="105" t="s">
+        <v>343</v>
+      </c>
+      <c r="P61" s="96">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q61" s="96">
+        <f t="shared" ref="Q61" si="58">N61*P61</f>
+        <v>0.12</v>
+      </c>
+      <c r="R61" s="96"/>
     </row>
     <row r="62" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1"/>
       <c r="B62" s="53">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-      <c r="C62" s="102" t="s">
+        <v>45</v>
+      </c>
+      <c r="C62" s="106" t="s">
         <v>324</v>
       </c>
-      <c r="D62" s="103" t="s">
-        <v>47</v>
-      </c>
-      <c r="E62" s="104" t="s">
-        <v>117</v>
-      </c>
-      <c r="F62" s="103" t="s">
+      <c r="D62" s="107" t="s">
+        <v>46</v>
+      </c>
+      <c r="E62" s="108" t="s">
+        <v>116</v>
+      </c>
+      <c r="F62" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="G62" s="104" t="s">
-        <v>212</v>
-      </c>
-      <c r="H62" s="103" t="s">
-        <v>229</v>
-      </c>
-      <c r="I62" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J62" s="103" t="s">
-        <v>397</v>
-      </c>
-      <c r="K62" s="104" t="s">
-        <v>296</v>
-      </c>
-      <c r="L62" s="103">
+      <c r="G62" s="108" t="s">
+        <v>211</v>
+      </c>
+      <c r="H62" s="107" t="s">
+        <v>251</v>
+      </c>
+      <c r="I62" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J62" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="K62" s="108" t="s">
+        <v>295</v>
+      </c>
+      <c r="L62" s="107">
         <v>1</v>
       </c>
-      <c r="M62" s="96">
+      <c r="M62" s="109">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N62" s="96">
-        <v>100</v>
-      </c>
-      <c r="O62" s="105" t="s">
-        <v>343</v>
-      </c>
-      <c r="P62" s="96">
-        <v>2.0999999999999999E-3</v>
-      </c>
-      <c r="Q62" s="96">
-        <f t="shared" ref="Q62" si="52">N62*P62</f>
-        <v>0.21</v>
-      </c>
-      <c r="R62" s="96"/>
+      <c r="N62" s="109">
+        <v>50</v>
+      </c>
+      <c r="O62" s="110" t="s">
+        <v>382</v>
+      </c>
+      <c r="P62" s="109">
+        <v>1.11E-2</v>
+      </c>
+      <c r="Q62" s="109">
+        <f t="shared" ref="Q62" si="59">P62*N62</f>
+        <v>0.55500000000000005</v>
+      </c>
+      <c r="R62" s="109"/>
     </row>
     <row r="63" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1"/>
       <c r="B63" s="53">
-        <f>ROW(B63) - ROW($B$9)</f>
+        <f t="shared" ref="B63:B88" si="60">ROW(B63) - ROW($B$9)</f>
         <v>54</v>
       </c>
-      <c r="C63" s="106" t="s">
+      <c r="C63" s="102" t="s">
         <v>324</v>
       </c>
-      <c r="D63" s="107" t="s">
-        <v>48</v>
-      </c>
-      <c r="E63" s="108" t="s">
-        <v>118</v>
-      </c>
-      <c r="F63" s="107" t="s">
+      <c r="D63" s="103" t="s">
+        <v>47</v>
+      </c>
+      <c r="E63" s="104" t="s">
+        <v>117</v>
+      </c>
+      <c r="F63" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="G63" s="108" t="s">
-        <v>213</v>
-      </c>
-      <c r="H63" s="107" t="s">
+      <c r="G63" s="104" t="s">
+        <v>212</v>
+      </c>
+      <c r="H63" s="103" t="s">
         <v>229</v>
       </c>
-      <c r="I63" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J63" s="107" t="s">
-        <v>398</v>
-      </c>
-      <c r="K63" s="108" t="s">
-        <v>297</v>
-      </c>
-      <c r="L63" s="107">
+      <c r="I63" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J63" s="103" t="s">
+        <v>397</v>
+      </c>
+      <c r="K63" s="104" t="s">
+        <v>296</v>
+      </c>
+      <c r="L63" s="103">
         <v>1</v>
       </c>
-      <c r="M63" s="109">
+      <c r="M63" s="96">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N63" s="109">
+      <c r="N63" s="96">
         <v>100</v>
       </c>
-      <c r="O63" s="110" t="s">
+      <c r="O63" s="105" t="s">
         <v>343</v>
       </c>
-      <c r="P63" s="109">
-        <v>1.6000000000000001E-3</v>
-      </c>
-      <c r="Q63" s="109">
-        <f t="shared" ref="Q63" si="53">P63*N63</f>
-        <v>0.16</v>
-      </c>
-      <c r="R63" s="109"/>
+      <c r="P63" s="96">
+        <v>2.0999999999999999E-3</v>
+      </c>
+      <c r="Q63" s="96">
+        <f t="shared" ref="Q63" si="61">N63*P63</f>
+        <v>0.21</v>
+      </c>
+      <c r="R63" s="96"/>
     </row>
     <row r="64" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1"/>
       <c r="B64" s="53">
-        <f t="shared" si="0"/>
-        <v>55</v>
-      </c>
-      <c r="C64" s="102" t="s">
+        <v>46</v>
+      </c>
+      <c r="C64" s="106" t="s">
         <v>324</v>
       </c>
-      <c r="D64" s="103" t="s">
-        <v>49</v>
-      </c>
-      <c r="E64" s="104" t="s">
-        <v>119</v>
-      </c>
-      <c r="F64" s="103" t="s">
+      <c r="D64" s="107" t="s">
+        <v>48</v>
+      </c>
+      <c r="E64" s="108" t="s">
+        <v>118</v>
+      </c>
+      <c r="F64" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="G64" s="104" t="s">
-        <v>214</v>
-      </c>
-      <c r="H64" s="103" t="s">
+      <c r="G64" s="108" t="s">
+        <v>213</v>
+      </c>
+      <c r="H64" s="107" t="s">
         <v>229</v>
       </c>
-      <c r="I64" s="103" t="s">
-        <v>399</v>
-      </c>
-      <c r="J64" s="103" t="s">
-        <v>400</v>
-      </c>
-      <c r="K64" s="104" t="s">
-        <v>298</v>
-      </c>
-      <c r="L64" s="103">
+      <c r="I64" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J64" s="107" t="s">
+        <v>398</v>
+      </c>
+      <c r="K64" s="108" t="s">
+        <v>297</v>
+      </c>
+      <c r="L64" s="107">
         <v>1</v>
       </c>
-      <c r="M64" s="96">
+      <c r="M64" s="109">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N64" s="96">
-        <v>50</v>
-      </c>
-      <c r="O64" s="105" t="s">
+      <c r="N64" s="109">
+        <v>100</v>
+      </c>
+      <c r="O64" s="110" t="s">
         <v>343</v>
       </c>
-      <c r="P64" s="96">
-        <v>6.8999999999999999E-3</v>
-      </c>
-      <c r="Q64" s="96">
-        <f t="shared" ref="Q64" si="54">N64*P64</f>
-        <v>0.34499999999999997</v>
-      </c>
-      <c r="R64" s="96"/>
-    </row>
-    <row r="65" spans="1:28" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P64" s="109">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="Q64" s="109">
+        <f t="shared" ref="Q64" si="62">P64*N64</f>
+        <v>0.16</v>
+      </c>
+      <c r="R64" s="109"/>
+    </row>
+    <row r="65" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1"/>
       <c r="B65" s="53">
-        <f>ROW(B65) - ROW($B$9)</f>
+        <f t="shared" ref="B65:B88" si="63">ROW(B65) - ROW($B$9)</f>
         <v>56</v>
       </c>
-      <c r="C65" s="106" t="s">
+      <c r="C65" s="102" t="s">
         <v>324</v>
       </c>
-      <c r="D65" s="107" t="s">
+      <c r="D65" s="103" t="s">
+        <v>49</v>
+      </c>
+      <c r="E65" s="104" t="s">
+        <v>119</v>
+      </c>
+      <c r="F65" s="103" t="s">
+        <v>166</v>
+      </c>
+      <c r="G65" s="104" t="s">
+        <v>214</v>
+      </c>
+      <c r="H65" s="103" t="s">
+        <v>229</v>
+      </c>
+      <c r="I65" s="103" t="s">
+        <v>399</v>
+      </c>
+      <c r="J65" s="103" t="s">
+        <v>400</v>
+      </c>
+      <c r="K65" s="104" t="s">
+        <v>298</v>
+      </c>
+      <c r="L65" s="103">
+        <v>1</v>
+      </c>
+      <c r="M65" s="96">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N65" s="96">
+        <v>50</v>
+      </c>
+      <c r="O65" s="105" t="s">
+        <v>343</v>
+      </c>
+      <c r="P65" s="96">
+        <v>6.8999999999999999E-3</v>
+      </c>
+      <c r="Q65" s="96">
+        <f t="shared" ref="Q65" si="64">N65*P65</f>
+        <v>0.34499999999999997</v>
+      </c>
+      <c r="R65" s="96"/>
+    </row>
+    <row r="66" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="1"/>
+      <c r="B66" s="53">
+        <v>47</v>
+      </c>
+      <c r="C66" s="106" t="s">
+        <v>324</v>
+      </c>
+      <c r="D66" s="107" t="s">
         <v>462</v>
       </c>
-      <c r="E65" s="108" t="s">
+      <c r="E66" s="108" t="s">
         <v>120</v>
       </c>
-      <c r="F65" s="107" t="s">
+      <c r="F66" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="G65" s="108" t="s">
+      <c r="G66" s="108" t="s">
         <v>215</v>
       </c>
-      <c r="H65" s="107" t="s">
+      <c r="H66" s="107" t="s">
         <v>229</v>
       </c>
-      <c r="I65" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J65" s="107" t="s">
+      <c r="I66" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J66" s="107" t="s">
         <v>401</v>
       </c>
-      <c r="K65" s="108" t="s">
+      <c r="K66" s="108" t="s">
         <v>299</v>
       </c>
-      <c r="L65" s="107">
+      <c r="L66" s="107">
         <v>2</v>
       </c>
-      <c r="M65" s="109">
+      <c r="M66" s="109">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N65" s="109">
+      <c r="N66" s="109">
         <v>100</v>
       </c>
-      <c r="O65" s="110" t="s">
+      <c r="O66" s="110" t="s">
         <v>343</v>
       </c>
-      <c r="P65" s="109">
+      <c r="P66" s="109">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="Q65" s="109">
-        <f t="shared" ref="Q65" si="55">P65*N65</f>
+      <c r="Q66" s="109">
+        <f t="shared" ref="Q66" si="65">P66*N66</f>
         <v>0.11</v>
       </c>
-      <c r="R65" s="109"/>
-    </row>
-    <row r="66" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="1"/>
-      <c r="B66" s="53">
-        <f>ROW(B66) - ROW($B$9)</f>
-        <v>57</v>
-      </c>
-      <c r="C66" s="60" t="s">
+      <c r="R66" s="109"/>
+    </row>
+    <row r="67" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="1"/>
+      <c r="B67" s="53">
+        <f t="shared" ref="B67:B88" si="66">ROW(B67) - ROW($B$9)</f>
+        <v>58</v>
+      </c>
+      <c r="C67" s="60" t="s">
         <v>324</v>
       </c>
-      <c r="D66" s="37" t="s">
+      <c r="D67" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="E66" s="38" t="s">
+      <c r="E67" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="F66" s="37" t="s">
+      <c r="F67" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="G66" s="38" t="s">
+      <c r="G67" s="38" t="s">
         <v>216</v>
       </c>
-      <c r="H66" s="37" t="s">
+      <c r="H67" s="37" t="s">
         <v>229</v>
       </c>
-      <c r="I66" s="37" t="s">
-        <v>314</v>
-      </c>
-      <c r="J66" s="37" t="s">
+      <c r="I67" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="J67" s="37" t="s">
         <v>402</v>
       </c>
-      <c r="K66" s="38" t="s">
+      <c r="K67" s="38" t="s">
         <v>300</v>
       </c>
-      <c r="L66" s="37">
+      <c r="L67" s="37">
         <v>2</v>
       </c>
-      <c r="M66" s="41">
+      <c r="M67" s="41">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N66" s="41">
+      <c r="N67" s="41">
         <v>100</v>
       </c>
-      <c r="O66" s="63" t="s">
+      <c r="O67" s="63" t="s">
         <v>343</v>
       </c>
-      <c r="P66" s="41">
+      <c r="P67" s="41">
         <v>1.5E-3</v>
       </c>
-      <c r="Q66" s="41">
-        <f t="shared" ref="Q66" si="56">P66*N66</f>
+      <c r="Q67" s="41">
+        <f t="shared" ref="Q67" si="67">P67*N67</f>
         <v>0.15</v>
       </c>
-      <c r="R66" s="41"/>
-    </row>
-    <row r="67" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="1"/>
-      <c r="B67" s="53">
-        <f>ROW(B67) - ROW($B$9)</f>
-        <v>58</v>
-      </c>
-      <c r="C67" s="59" t="s">
-        <v>324</v>
-      </c>
-      <c r="D67" s="87" t="s">
-        <v>424</v>
-      </c>
-      <c r="E67" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="F67" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="G67" s="40" t="s">
-        <v>206</v>
-      </c>
-      <c r="H67" s="39" t="s">
-        <v>229</v>
-      </c>
-      <c r="I67" s="39"/>
-      <c r="J67" s="39" t="s">
-        <v>394</v>
-      </c>
-      <c r="K67" s="40" t="s">
-        <v>290</v>
-      </c>
-      <c r="L67" s="39">
-        <v>1</v>
-      </c>
-      <c r="M67" s="42">
-        <f>L67*20</f>
-        <v>20</v>
-      </c>
-      <c r="N67" s="42">
-        <v>100</v>
-      </c>
-      <c r="O67" s="64" t="s">
-        <v>343</v>
-      </c>
-      <c r="P67" s="42">
-        <v>1.5E-3</v>
-      </c>
-      <c r="Q67" s="42">
-        <f>N67*P67</f>
-        <v>0.15</v>
-      </c>
-      <c r="R67" s="77"/>
-    </row>
-    <row r="68" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R67" s="41"/>
+    </row>
+    <row r="68" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="1"/>
       <c r="B68" s="53">
-        <f>ROW(B68) - ROW($B$9)</f>
-        <v>59</v>
-      </c>
-      <c r="C68" s="60" t="s">
+        <v>48</v>
+      </c>
+      <c r="C68" s="59" t="s">
         <v>324</v>
       </c>
-      <c r="D68" s="37" t="s">
+      <c r="D68" s="87" t="s">
+        <v>424</v>
+      </c>
+      <c r="E68" s="40" t="s">
+        <v>111</v>
+      </c>
+      <c r="F68" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="G68" s="40" t="s">
+        <v>206</v>
+      </c>
+      <c r="H68" s="39" t="s">
+        <v>229</v>
+      </c>
+      <c r="I68" s="39"/>
+      <c r="J68" s="39" t="s">
+        <v>394</v>
+      </c>
+      <c r="K68" s="40" t="s">
+        <v>290</v>
+      </c>
+      <c r="L68" s="39">
+        <v>1</v>
+      </c>
+      <c r="M68" s="42">
+        <f>L68*20</f>
+        <v>20</v>
+      </c>
+      <c r="N68" s="42">
+        <v>100</v>
+      </c>
+      <c r="O68" s="64" t="s">
+        <v>343</v>
+      </c>
+      <c r="P68" s="42">
+        <v>1.5E-3</v>
+      </c>
+      <c r="Q68" s="42">
+        <f>N68*P68</f>
+        <v>0.15</v>
+      </c>
+      <c r="R68" s="77"/>
+    </row>
+    <row r="69" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="1"/>
+      <c r="B69" s="53">
+        <f t="shared" ref="B69:B88" si="68">ROW(B69) - ROW($B$9)</f>
+        <v>60</v>
+      </c>
+      <c r="C69" s="60" t="s">
+        <v>324</v>
+      </c>
+      <c r="D69" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="E68" s="38" t="s">
+      <c r="E69" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="F68" s="37" t="s">
+      <c r="F69" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="G68" s="38" t="s">
+      <c r="G69" s="38" t="s">
         <v>217</v>
       </c>
-      <c r="H68" s="37" t="s">
+      <c r="H69" s="37" t="s">
         <v>229</v>
       </c>
-      <c r="I68" s="37" t="s">
-        <v>314</v>
-      </c>
-      <c r="J68" s="37" t="s">
+      <c r="I69" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="J69" s="37" t="s">
         <v>403</v>
       </c>
-      <c r="K68" s="38" t="s">
+      <c r="K69" s="38" t="s">
         <v>301</v>
       </c>
-      <c r="L68" s="37">
+      <c r="L69" s="37">
         <v>2</v>
       </c>
-      <c r="M68" s="41">
+      <c r="M69" s="41">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N68" s="41">
+      <c r="N69" s="41">
         <v>100</v>
       </c>
-      <c r="O68" s="63" t="s">
+      <c r="O69" s="63" t="s">
         <v>343</v>
       </c>
-      <c r="P68" s="41">
+      <c r="P69" s="41">
         <v>1.5E-3</v>
       </c>
-      <c r="Q68" s="41">
-        <f t="shared" ref="Q68" si="57">P68*N68</f>
+      <c r="Q69" s="41">
+        <f t="shared" ref="Q69" si="69">P69*N69</f>
         <v>0.15</v>
       </c>
-      <c r="R68" s="41"/>
-    </row>
-    <row r="69" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="1"/>
-      <c r="B69" s="53">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="C69" s="59" t="s">
+      <c r="R69" s="41"/>
+    </row>
+    <row r="70" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A70" s="1"/>
+      <c r="B70" s="53">
+        <v>49</v>
+      </c>
+      <c r="C70" s="59" t="s">
         <v>324</v>
       </c>
-      <c r="D69" s="39" t="s">
+      <c r="D70" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="E69" s="40" t="s">
+      <c r="E70" s="40" t="s">
         <v>123</v>
       </c>
-      <c r="F69" s="39" t="s">
+      <c r="F70" s="39" t="s">
         <v>166</v>
       </c>
-      <c r="G69" s="40" t="s">
+      <c r="G70" s="40" t="s">
         <v>218</v>
       </c>
-      <c r="H69" s="39" t="s">
+      <c r="H70" s="39" t="s">
         <v>251</v>
       </c>
-      <c r="I69" s="39" t="s">
-        <v>314</v>
-      </c>
-      <c r="J69" s="39" t="s">
-        <v>314</v>
-      </c>
-      <c r="K69" s="40" t="s">
+      <c r="I70" s="39" t="s">
+        <v>314</v>
+      </c>
+      <c r="J70" s="39" t="s">
+        <v>314</v>
+      </c>
+      <c r="K70" s="40" t="s">
         <v>302</v>
       </c>
-      <c r="L69" s="39">
+      <c r="L70" s="39">
         <v>1</v>
       </c>
-      <c r="M69" s="42">
+      <c r="M70" s="42">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N69" s="42">
+      <c r="N70" s="42">
         <v>25</v>
       </c>
-      <c r="O69" s="64" t="s">
+      <c r="O70" s="64" t="s">
         <v>404</v>
       </c>
-      <c r="P69" s="42">
+      <c r="P70" s="42">
         <v>8.5400000000000004E-2</v>
       </c>
-      <c r="Q69" s="42">
-        <f t="shared" ref="Q69" si="58">N69*P69</f>
+      <c r="Q70" s="42">
+        <f t="shared" ref="Q70" si="70">N70*P70</f>
         <v>2.1350000000000002</v>
       </c>
-      <c r="R69" s="42"/>
-    </row>
-    <row r="70" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="1"/>
-      <c r="B70" s="53">
-        <f>ROW(B70) - ROW($B$9)</f>
-        <v>61</v>
-      </c>
-      <c r="C70" s="60" t="s">
-        <v>324</v>
-      </c>
-      <c r="D70" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="E70" s="38" t="s">
-        <v>434</v>
-      </c>
-      <c r="F70" s="86" t="s">
-        <v>166</v>
-      </c>
-      <c r="G70" s="38" t="s">
-        <v>450</v>
-      </c>
-      <c r="H70" s="37" t="s">
-        <v>252</v>
-      </c>
-      <c r="I70" s="37" t="s">
-        <v>314</v>
-      </c>
-      <c r="J70" s="37" t="s">
-        <v>435</v>
-      </c>
-      <c r="K70" s="38" t="s">
-        <v>449</v>
-      </c>
-      <c r="L70" s="37">
-        <v>1</v>
-      </c>
-      <c r="M70" s="41">
-        <f t="shared" ref="M70:M87" si="59">L70*20</f>
-        <v>20</v>
-      </c>
-      <c r="N70" s="41">
-        <v>50</v>
-      </c>
-      <c r="O70" s="63" t="s">
-        <v>343</v>
-      </c>
-      <c r="P70" s="41">
-        <v>3.8E-3</v>
-      </c>
-      <c r="Q70" s="41">
-        <f t="shared" ref="Q70" si="60">P70*N70</f>
-        <v>0.19</v>
-      </c>
-      <c r="R70" s="76"/>
-    </row>
-    <row r="71" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R70" s="42"/>
+    </row>
+    <row r="71" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1"/>
       <c r="B71" s="53">
-        <f>ROW(B71) - ROW($B$9)</f>
+        <f t="shared" ref="B71:B88" si="71">ROW(B71) - ROW($B$9)</f>
         <v>62</v>
       </c>
-      <c r="C71" s="59" t="s">
+      <c r="C71" s="60" t="s">
         <v>324</v>
       </c>
-      <c r="D71" s="39" t="s">
-        <v>451</v>
-      </c>
-      <c r="E71" s="40" t="s">
-        <v>127</v>
-      </c>
-      <c r="F71" s="39" t="s">
+      <c r="D71" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="E71" s="38" t="s">
+        <v>434</v>
+      </c>
+      <c r="F71" s="86" t="s">
         <v>166</v>
       </c>
-      <c r="G71" s="40" t="s">
-        <v>220</v>
-      </c>
-      <c r="H71" s="39" t="s">
-        <v>229</v>
-      </c>
-      <c r="I71" s="39" t="s">
-        <v>314</v>
-      </c>
-      <c r="J71" s="39" t="s">
-        <v>408</v>
-      </c>
-      <c r="K71" s="40" t="s">
-        <v>306</v>
-      </c>
-      <c r="L71" s="39">
-        <v>6</v>
-      </c>
-      <c r="M71" s="42">
-        <f>L71*20</f>
-        <v>120</v>
-      </c>
-      <c r="N71" s="42">
-        <v>200</v>
-      </c>
-      <c r="O71" s="64" t="s">
+      <c r="G71" s="38" t="s">
+        <v>450</v>
+      </c>
+      <c r="H71" s="37" t="s">
+        <v>252</v>
+      </c>
+      <c r="I71" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="J71" s="37" t="s">
+        <v>435</v>
+      </c>
+      <c r="K71" s="38" t="s">
+        <v>449</v>
+      </c>
+      <c r="L71" s="37">
+        <v>1</v>
+      </c>
+      <c r="M71" s="41">
+        <f t="shared" ref="M71:M88" si="72">L71*20</f>
+        <v>20</v>
+      </c>
+      <c r="N71" s="41">
+        <v>50</v>
+      </c>
+      <c r="O71" s="63" t="s">
         <v>343</v>
       </c>
-      <c r="P71" s="42">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="Q71" s="42">
-        <f t="shared" ref="Q71" si="61">N71*P71</f>
-        <v>0.24</v>
-      </c>
-      <c r="R71" s="77"/>
-    </row>
-    <row r="72" spans="1:28" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P71" s="41">
+        <v>3.8E-3</v>
+      </c>
+      <c r="Q71" s="41">
+        <f t="shared" ref="Q71" si="73">P71*N71</f>
+        <v>0.19</v>
+      </c>
+      <c r="R71" s="76"/>
+    </row>
+    <row r="72" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1"/>
       <c r="B72" s="53">
-        <f>ROW(B72) - ROW($B$9)</f>
-        <v>63</v>
-      </c>
-      <c r="C72" s="60" t="s">
+        <v>50</v>
+      </c>
+      <c r="C72" s="59" t="s">
         <v>324</v>
       </c>
-      <c r="D72" s="37" t="s">
-        <v>54</v>
-      </c>
-      <c r="E72" s="38" t="s">
-        <v>124</v>
-      </c>
-      <c r="F72" s="37" t="s">
+      <c r="D72" s="39" t="s">
+        <v>451</v>
+      </c>
+      <c r="E72" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="F72" s="39" t="s">
         <v>166</v>
       </c>
-      <c r="G72" s="38" t="s">
-        <v>330</v>
-      </c>
-      <c r="H72" s="37" t="s">
-        <v>252</v>
-      </c>
-      <c r="I72" s="37" t="s">
-        <v>314</v>
-      </c>
-      <c r="J72" s="37" t="s">
-        <v>405</v>
-      </c>
-      <c r="K72" s="38" t="s">
-        <v>303</v>
-      </c>
-      <c r="L72" s="37">
-        <v>1</v>
-      </c>
-      <c r="M72" s="41">
-        <f t="shared" si="59"/>
-        <v>20</v>
-      </c>
-      <c r="N72" s="41">
-        <v>100</v>
-      </c>
-      <c r="O72" s="63" t="s">
+      <c r="G72" s="40" t="s">
+        <v>220</v>
+      </c>
+      <c r="H72" s="39" t="s">
+        <v>229</v>
+      </c>
+      <c r="I72" s="39" t="s">
+        <v>314</v>
+      </c>
+      <c r="J72" s="39" t="s">
+        <v>408</v>
+      </c>
+      <c r="K72" s="40" t="s">
+        <v>306</v>
+      </c>
+      <c r="L72" s="39">
+        <v>6</v>
+      </c>
+      <c r="M72" s="42">
+        <f>L72*20</f>
+        <v>120</v>
+      </c>
+      <c r="N72" s="42">
+        <v>200</v>
+      </c>
+      <c r="O72" s="64" t="s">
         <v>343</v>
       </c>
-      <c r="P72" s="41">
-        <v>1E-3</v>
-      </c>
-      <c r="Q72" s="41">
-        <f t="shared" ref="Q72" si="62">P72*N72</f>
-        <v>0.1</v>
-      </c>
-      <c r="R72" s="41"/>
-    </row>
-    <row r="73" spans="1:28" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P72" s="42">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q72" s="42">
+        <f t="shared" ref="Q72" si="74">N72*P72</f>
+        <v>0.24</v>
+      </c>
+      <c r="R72" s="77"/>
+    </row>
+    <row r="73" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1"/>
       <c r="B73" s="53">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B73:B88" si="75">ROW(B73) - ROW($B$9)</f>
         <v>64</v>
       </c>
-      <c r="C73" s="59" t="s">
+      <c r="C73" s="60" t="s">
         <v>324</v>
       </c>
-      <c r="D73" s="39" t="s">
-        <v>55</v>
-      </c>
-      <c r="E73" s="40" t="s">
-        <v>125</v>
-      </c>
-      <c r="F73" s="39" t="s">
+      <c r="D73" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="E73" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="F73" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="G73" s="40" t="s">
-        <v>331</v>
-      </c>
-      <c r="H73" s="39" t="s">
-        <v>253</v>
-      </c>
-      <c r="I73" s="39" t="s">
-        <v>314</v>
-      </c>
-      <c r="J73" s="39" t="s">
-        <v>406</v>
-      </c>
-      <c r="K73" s="40" t="s">
-        <v>304</v>
-      </c>
-      <c r="L73" s="39">
+      <c r="G73" s="38" t="s">
+        <v>330</v>
+      </c>
+      <c r="H73" s="37" t="s">
+        <v>252</v>
+      </c>
+      <c r="I73" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="J73" s="37" t="s">
+        <v>405</v>
+      </c>
+      <c r="K73" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="L73" s="37">
         <v>1</v>
       </c>
-      <c r="M73" s="42">
-        <f t="shared" si="59"/>
+      <c r="M73" s="41">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N73" s="42">
-        <v>50</v>
-      </c>
-      <c r="O73" s="64" t="s">
+      <c r="N73" s="41">
+        <v>100</v>
+      </c>
+      <c r="O73" s="63" t="s">
         <v>343</v>
       </c>
-      <c r="P73" s="42">
-        <v>4.3E-3</v>
-      </c>
-      <c r="Q73" s="42">
-        <f t="shared" ref="Q73" si="63">N73*P73</f>
-        <v>0.215</v>
-      </c>
-      <c r="R73" s="42"/>
-    </row>
-    <row r="74" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P73" s="41">
+        <v>1E-3</v>
+      </c>
+      <c r="Q73" s="41">
+        <f t="shared" ref="Q73" si="76">P73*N73</f>
+        <v>0.1</v>
+      </c>
+      <c r="R73" s="41"/>
+    </row>
+    <row r="74" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1"/>
       <c r="B74" s="53">
-        <f>ROW(B74) - ROW($B$9)</f>
-        <v>65</v>
-      </c>
-      <c r="C74" s="97" t="s">
+        <v>51</v>
+      </c>
+      <c r="C74" s="59" t="s">
         <v>324</v>
       </c>
-      <c r="D74" s="98" t="s">
-        <v>56</v>
-      </c>
-      <c r="E74" s="99" t="s">
-        <v>126</v>
-      </c>
-      <c r="F74" s="98" t="s">
-        <v>168</v>
-      </c>
-      <c r="G74" s="99" t="s">
-        <v>219</v>
-      </c>
-      <c r="H74" s="98" t="s">
-        <v>229</v>
-      </c>
-      <c r="I74" s="98" t="s">
-        <v>314</v>
-      </c>
-      <c r="J74" s="98" t="s">
-        <v>407</v>
-      </c>
-      <c r="K74" s="99" t="s">
-        <v>305</v>
-      </c>
-      <c r="L74" s="98">
-        <v>4</v>
-      </c>
-      <c r="M74" s="66">
-        <f t="shared" si="59"/>
-        <v>80</v>
-      </c>
-      <c r="N74" s="66">
-        <v>100</v>
-      </c>
-      <c r="O74" s="100" t="s">
+      <c r="D74" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="E74" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="F74" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="G74" s="40" t="s">
+        <v>331</v>
+      </c>
+      <c r="H74" s="39" t="s">
+        <v>253</v>
+      </c>
+      <c r="I74" s="39" t="s">
+        <v>314</v>
+      </c>
+      <c r="J74" s="39" t="s">
+        <v>406</v>
+      </c>
+      <c r="K74" s="40" t="s">
+        <v>304</v>
+      </c>
+      <c r="L74" s="39">
+        <v>1</v>
+      </c>
+      <c r="M74" s="42">
+        <f t="shared" si="72"/>
+        <v>20</v>
+      </c>
+      <c r="N74" s="42">
+        <v>50</v>
+      </c>
+      <c r="O74" s="64" t="s">
         <v>343</v>
       </c>
-      <c r="P74" s="66">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="Q74" s="66">
-        <f t="shared" ref="Q74" si="64">P74*N74</f>
-        <v>0.12</v>
-      </c>
-      <c r="R74" s="66" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="75" spans="1:28" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P74" s="42">
+        <v>4.3E-3</v>
+      </c>
+      <c r="Q74" s="42">
+        <f t="shared" ref="Q74" si="77">N74*P74</f>
+        <v>0.215</v>
+      </c>
+      <c r="R74" s="42"/>
+    </row>
+    <row r="75" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1"/>
       <c r="B75" s="53">
-        <f>ROW(B75) - ROW($B$9)</f>
+        <f t="shared" ref="B75:B88" si="78">ROW(B75) - ROW($B$9)</f>
         <v>66</v>
       </c>
       <c r="C75" s="97" t="s">
-        <v>169</v>
+        <v>324</v>
       </c>
       <c r="D75" s="98" t="s">
-        <v>453</v>
+        <v>56</v>
       </c>
       <c r="E75" s="99" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F75" s="98" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G75" s="99" t="s">
-        <v>314</v>
+        <v>219</v>
       </c>
       <c r="H75" s="98" t="s">
-        <v>314</v>
+        <v>229</v>
       </c>
       <c r="I75" s="98" t="s">
         <v>314</v>
       </c>
       <c r="J75" s="98" t="s">
-        <v>314</v>
+        <v>407</v>
       </c>
       <c r="K75" s="99" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="L75" s="98">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="M75" s="66">
-        <f t="shared" si="59"/>
-        <v>300</v>
+        <f t="shared" si="72"/>
+        <v>80</v>
       </c>
       <c r="N75" s="66">
-        <f t="shared" ref="N75:N76" si="65">M75+(M75*0.1)</f>
-        <v>330</v>
-      </c>
-      <c r="O75" s="66"/>
-      <c r="P75" s="66"/>
+        <v>100</v>
+      </c>
+      <c r="O75" s="100" t="s">
+        <v>343</v>
+      </c>
+      <c r="P75" s="66">
+        <v>1.1999999999999999E-3</v>
+      </c>
       <c r="Q75" s="66">
-        <f t="shared" ref="Q75" si="66">P75*N75</f>
-        <v>0</v>
+        <f t="shared" ref="Q75" si="79">P75*N75</f>
+        <v>0.12</v>
       </c>
       <c r="R75" s="66" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="76" spans="1:28" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="76" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1"/>
       <c r="B76" s="53">
-        <f t="shared" si="0"/>
-        <v>67</v>
-      </c>
-      <c r="C76" s="102" t="s">
-        <v>326</v>
-      </c>
-      <c r="D76" s="103" t="s">
-        <v>57</v>
-      </c>
-      <c r="E76" s="104" t="s">
-        <v>129</v>
-      </c>
-      <c r="F76" s="103" t="s">
-        <v>170</v>
-      </c>
-      <c r="G76" s="104" t="s">
-        <v>314</v>
-      </c>
-      <c r="H76" s="103" t="s">
-        <v>254</v>
-      </c>
-      <c r="I76" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J76" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="K76" s="104" t="s">
-        <v>314</v>
-      </c>
-      <c r="L76" s="103">
-        <v>1</v>
-      </c>
-      <c r="M76" s="96">
-        <f t="shared" si="59"/>
-        <v>20</v>
-      </c>
-      <c r="N76" s="96">
-        <f t="shared" si="65"/>
-        <v>22</v>
-      </c>
-      <c r="O76" s="96"/>
-      <c r="P76" s="96"/>
-      <c r="Q76" s="96">
-        <f t="shared" ref="Q76" si="67">N76*P76</f>
+        <v>52</v>
+      </c>
+      <c r="C76" s="97" t="s">
+        <v>169</v>
+      </c>
+      <c r="D76" s="98" t="s">
+        <v>453</v>
+      </c>
+      <c r="E76" s="99" t="s">
+        <v>128</v>
+      </c>
+      <c r="F76" s="98" t="s">
+        <v>169</v>
+      </c>
+      <c r="G76" s="99" t="s">
+        <v>314</v>
+      </c>
+      <c r="H76" s="98" t="s">
+        <v>314</v>
+      </c>
+      <c r="I76" s="98" t="s">
+        <v>314</v>
+      </c>
+      <c r="J76" s="98" t="s">
+        <v>314</v>
+      </c>
+      <c r="K76" s="99" t="s">
+        <v>314</v>
+      </c>
+      <c r="L76" s="98">
+        <v>15</v>
+      </c>
+      <c r="M76" s="66">
+        <f t="shared" si="72"/>
+        <v>300</v>
+      </c>
+      <c r="N76" s="66">
+        <f t="shared" ref="N76:N77" si="80">M76+(M76*0.1)</f>
+        <v>330</v>
+      </c>
+      <c r="O76" s="66"/>
+      <c r="P76" s="66"/>
+      <c r="Q76" s="66">
+        <f t="shared" ref="Q76" si="81">P76*N76</f>
         <v>0</v>
       </c>
-      <c r="R76" s="96"/>
-      <c r="T76" t="s">
-        <v>57</v>
-      </c>
-      <c r="V76" t="s">
-        <v>314</v>
-      </c>
-      <c r="W76">
-        <v>1</v>
-      </c>
-      <c r="Y76" t="str">
-        <f>IF(T76=D76, "Match", "Mismatch")</f>
-        <v>Match</v>
-      </c>
-      <c r="Z76" t="str">
-        <f>IF(G76=U76, "Match", "Mismatch")</f>
-        <v>Mismatch</v>
-      </c>
-      <c r="AA76" t="str">
-        <f>IF(K76=V76, "Match", "Mismatch")</f>
-        <v>Match</v>
-      </c>
-      <c r="AB76" t="str">
-        <f>IF(W76=L76, "Match", "Mismatch")</f>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="77" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R76" s="66" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="77" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1"/>
       <c r="B77" s="53">
-        <f>ROW(B77) - ROW($B$9)</f>
+        <f t="shared" ref="B77:B88" si="82">ROW(B77) - ROW($B$9)</f>
         <v>68</v>
       </c>
-      <c r="C77" s="106" t="s">
-        <v>327</v>
-      </c>
-      <c r="D77" s="107" t="s">
-        <v>58</v>
-      </c>
-      <c r="E77" s="108" t="s">
-        <v>130</v>
-      </c>
-      <c r="F77" s="107" t="s">
-        <v>308</v>
-      </c>
-      <c r="G77" s="108">
-        <v>750314597</v>
-      </c>
-      <c r="H77" s="107" t="s">
-        <v>255</v>
-      </c>
-      <c r="I77" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J77" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="K77" s="108" t="s">
-        <v>314</v>
-      </c>
-      <c r="L77" s="107">
+      <c r="C77" s="102" t="s">
+        <v>326</v>
+      </c>
+      <c r="D77" s="103" t="s">
+        <v>57</v>
+      </c>
+      <c r="E77" s="104" t="s">
+        <v>129</v>
+      </c>
+      <c r="F77" s="103" t="s">
+        <v>170</v>
+      </c>
+      <c r="G77" s="104" t="s">
+        <v>314</v>
+      </c>
+      <c r="H77" s="103" t="s">
+        <v>254</v>
+      </c>
+      <c r="I77" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J77" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="K77" s="104" t="s">
+        <v>314</v>
+      </c>
+      <c r="L77" s="103">
         <v>1</v>
       </c>
-      <c r="M77" s="109">
-        <f t="shared" si="59"/>
+      <c r="M77" s="96">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N77" s="109">
-        <v>21</v>
-      </c>
-      <c r="O77" s="110" t="s">
-        <v>379</v>
-      </c>
-      <c r="P77" s="109">
-        <v>3.81</v>
-      </c>
-      <c r="Q77" s="109">
-        <f t="shared" ref="Q77" si="68">P77*N77</f>
-        <v>80.010000000000005</v>
-      </c>
-      <c r="R77" s="109"/>
-      <c r="T77" t="s">
-        <v>58</v>
-      </c>
-      <c r="U77">
-        <v>750314597</v>
-      </c>
-      <c r="V77" t="s">
-        <v>314</v>
-      </c>
-      <c r="W77">
-        <v>1</v>
-      </c>
-      <c r="Y77" t="str">
-        <f t="shared" ref="Y77:Y87" si="69">IF(T77=D77, "Match", "Mismatch")</f>
-        <v>Match</v>
-      </c>
-      <c r="Z77" t="str">
-        <f t="shared" ref="Z77:Z87" si="70">IF(G77=U77, "Match", "Mismatch")</f>
-        <v>Match</v>
-      </c>
-      <c r="AA77" t="str">
-        <f t="shared" ref="AA77:AA87" si="71">IF(K77=V77, "Match", "Mismatch")</f>
-        <v>Match</v>
-      </c>
-      <c r="AB77" t="str">
-        <f t="shared" ref="AB77:AB87" si="72">IF(W77=L77, "Match", "Mismatch")</f>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="78" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N77" s="96">
+        <f t="shared" si="80"/>
+        <v>22</v>
+      </c>
+      <c r="O77" s="96"/>
+      <c r="P77" s="96"/>
+      <c r="Q77" s="96">
+        <f t="shared" ref="Q77" si="83">N77*P77</f>
+        <v>0</v>
+      </c>
+      <c r="R77" s="96"/>
+    </row>
+    <row r="78" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1"/>
       <c r="B78" s="53">
-        <f t="shared" si="0"/>
-        <v>69</v>
-      </c>
-      <c r="C78" s="102" t="s">
-        <v>328</v>
-      </c>
-      <c r="D78" s="103" t="s">
-        <v>59</v>
-      </c>
-      <c r="E78" s="104" t="s">
-        <v>131</v>
-      </c>
-      <c r="F78" s="103" t="s">
+        <v>53</v>
+      </c>
+      <c r="C78" s="106" t="s">
+        <v>327</v>
+      </c>
+      <c r="D78" s="107" t="s">
+        <v>58</v>
+      </c>
+      <c r="E78" s="108" t="s">
+        <v>130</v>
+      </c>
+      <c r="F78" s="107" t="s">
         <v>308</v>
       </c>
-      <c r="G78" s="104" t="s">
-        <v>171</v>
-      </c>
-      <c r="H78" s="103" t="s">
-        <v>256</v>
-      </c>
-      <c r="I78" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J78" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="K78" s="104" t="s">
-        <v>314</v>
-      </c>
-      <c r="L78" s="103">
+      <c r="G78" s="108">
+        <v>750314597</v>
+      </c>
+      <c r="H78" s="107" t="s">
+        <v>255</v>
+      </c>
+      <c r="I78" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J78" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="K78" s="108" t="s">
+        <v>314</v>
+      </c>
+      <c r="L78" s="107">
         <v>1</v>
       </c>
-      <c r="M78" s="96">
-        <f t="shared" si="59"/>
+      <c r="M78" s="109">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N78" s="96">
+      <c r="N78" s="109">
         <v>21</v>
       </c>
-      <c r="O78" s="105" t="s">
-        <v>409</v>
-      </c>
-      <c r="P78" s="96">
-        <v>2.48</v>
-      </c>
-      <c r="Q78" s="96">
-        <f t="shared" ref="Q78" si="73">N78*P78</f>
-        <v>52.08</v>
-      </c>
-      <c r="R78" s="96"/>
-      <c r="T78" t="s">
-        <v>59</v>
-      </c>
-      <c r="U78" t="s">
-        <v>171</v>
-      </c>
-      <c r="V78" t="s">
-        <v>314</v>
-      </c>
-      <c r="W78">
-        <v>1</v>
-      </c>
-      <c r="Y78" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z78" t="str">
-        <f t="shared" si="70"/>
-        <v>Match</v>
-      </c>
-      <c r="AA78" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB78" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="79" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O78" s="110" t="s">
+        <v>379</v>
+      </c>
+      <c r="P78" s="109">
+        <v>3.81</v>
+      </c>
+      <c r="Q78" s="109">
+        <f t="shared" ref="Q78" si="84">P78*N78</f>
+        <v>80.010000000000005</v>
+      </c>
+      <c r="R78" s="109"/>
+    </row>
+    <row r="79" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1"/>
       <c r="B79" s="53">
-        <f>ROW(B79) - ROW($B$9)</f>
+        <f t="shared" ref="B79:B88" si="85">ROW(B79) - ROW($B$9)</f>
         <v>70</v>
       </c>
-      <c r="C79" s="106" t="s">
+      <c r="C79" s="102" t="s">
         <v>328</v>
       </c>
-      <c r="D79" s="107" t="s">
-        <v>60</v>
-      </c>
-      <c r="E79" s="108" t="s">
-        <v>132</v>
-      </c>
-      <c r="F79" s="107" t="s">
-        <v>172</v>
-      </c>
-      <c r="G79" s="108" t="s">
-        <v>221</v>
-      </c>
-      <c r="H79" s="107" t="s">
-        <v>257</v>
-      </c>
-      <c r="I79" s="107" t="s">
-        <v>410</v>
-      </c>
-      <c r="J79" s="107" t="s">
-        <v>411</v>
-      </c>
-      <c r="K79" s="108" t="s">
-        <v>314</v>
-      </c>
-      <c r="L79" s="107">
+      <c r="D79" s="103" t="s">
+        <v>59</v>
+      </c>
+      <c r="E79" s="104" t="s">
+        <v>131</v>
+      </c>
+      <c r="F79" s="103" t="s">
+        <v>308</v>
+      </c>
+      <c r="G79" s="104" t="s">
+        <v>171</v>
+      </c>
+      <c r="H79" s="103" t="s">
+        <v>256</v>
+      </c>
+      <c r="I79" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J79" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="K79" s="104" t="s">
+        <v>314</v>
+      </c>
+      <c r="L79" s="103">
         <v>1</v>
       </c>
-      <c r="M79" s="109">
-        <f t="shared" si="59"/>
+      <c r="M79" s="96">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N79" s="109">
+      <c r="N79" s="96">
         <v>21</v>
       </c>
-      <c r="O79" s="110" t="s">
-        <v>343</v>
-      </c>
-      <c r="P79" s="109">
-        <v>1.3939999999999999</v>
-      </c>
-      <c r="Q79" s="109">
-        <f t="shared" ref="Q79" si="74">P79*N79</f>
-        <v>29.273999999999997</v>
-      </c>
-      <c r="R79" s="79"/>
-      <c r="T79" t="s">
-        <v>60</v>
-      </c>
-      <c r="U79" t="s">
-        <v>410</v>
-      </c>
-      <c r="V79" t="s">
-        <v>314</v>
-      </c>
-      <c r="W79">
-        <v>1</v>
-      </c>
-      <c r="Y79" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z79" t="str">
-        <f t="shared" si="70"/>
-        <v>Mismatch</v>
-      </c>
-      <c r="AA79" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB79" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="80" spans="1:28" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O79" s="105" t="s">
+        <v>409</v>
+      </c>
+      <c r="P79" s="96">
+        <v>2.48</v>
+      </c>
+      <c r="Q79" s="96">
+        <f t="shared" ref="Q79" si="86">N79*P79</f>
+        <v>52.08</v>
+      </c>
+      <c r="R79" s="96"/>
+    </row>
+    <row r="80" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A80" s="1"/>
       <c r="B80" s="53">
-        <f t="shared" si="0"/>
-        <v>71</v>
-      </c>
-      <c r="C80" s="102" t="s">
+        <v>54</v>
+      </c>
+      <c r="C80" s="106" t="s">
         <v>328</v>
       </c>
-      <c r="D80" s="103" t="s">
-        <v>61</v>
-      </c>
-      <c r="E80" s="104" t="s">
-        <v>133</v>
-      </c>
-      <c r="F80" s="103" t="s">
-        <v>173</v>
-      </c>
-      <c r="G80" s="104" t="s">
-        <v>222</v>
-      </c>
-      <c r="H80" s="103" t="s">
-        <v>256</v>
-      </c>
-      <c r="I80" s="103" t="s">
-        <v>412</v>
-      </c>
-      <c r="J80" s="103" t="s">
-        <v>413</v>
-      </c>
-      <c r="K80" s="104" t="s">
-        <v>314</v>
-      </c>
-      <c r="L80" s="103">
+      <c r="D80" s="107" t="s">
+        <v>60</v>
+      </c>
+      <c r="E80" s="108" t="s">
+        <v>132</v>
+      </c>
+      <c r="F80" s="107" t="s">
+        <v>172</v>
+      </c>
+      <c r="G80" s="108" t="s">
+        <v>221</v>
+      </c>
+      <c r="H80" s="107" t="s">
+        <v>257</v>
+      </c>
+      <c r="I80" s="107" t="s">
+        <v>410</v>
+      </c>
+      <c r="J80" s="107" t="s">
+        <v>411</v>
+      </c>
+      <c r="K80" s="108" t="s">
+        <v>314</v>
+      </c>
+      <c r="L80" s="107">
         <v>1</v>
       </c>
-      <c r="M80" s="96">
-        <f t="shared" si="59"/>
+      <c r="M80" s="109">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N80" s="96">
+      <c r="N80" s="109">
         <v>21</v>
       </c>
-      <c r="O80" s="105" t="s">
+      <c r="O80" s="110" t="s">
         <v>343</v>
       </c>
-      <c r="P80" s="96">
-        <v>0.69430000000000003</v>
-      </c>
-      <c r="Q80" s="96">
-        <f t="shared" ref="Q80" si="75">N80*P80</f>
-        <v>14.580300000000001</v>
-      </c>
-      <c r="R80" s="78"/>
-      <c r="T80" t="s">
-        <v>61</v>
-      </c>
-      <c r="U80" t="s">
-        <v>412</v>
-      </c>
-      <c r="V80" t="s">
-        <v>314</v>
-      </c>
-      <c r="W80">
-        <v>1</v>
-      </c>
-      <c r="Y80" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z80" t="str">
-        <f t="shared" si="70"/>
-        <v>Mismatch</v>
-      </c>
-      <c r="AA80" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB80" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="81" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P80" s="109">
+        <v>1.3939999999999999</v>
+      </c>
+      <c r="Q80" s="109">
+        <f t="shared" ref="Q80" si="87">P80*N80</f>
+        <v>29.273999999999997</v>
+      </c>
+      <c r="R80" s="79"/>
+    </row>
+    <row r="81" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1"/>
       <c r="B81" s="53">
-        <f>ROW(B81) - ROW($B$9)</f>
+        <f t="shared" ref="B81:B88" si="88">ROW(B81) - ROW($B$9)</f>
         <v>72</v>
       </c>
-      <c r="C81" s="106" t="s">
+      <c r="C81" s="102" t="s">
         <v>328</v>
       </c>
-      <c r="D81" s="107" t="s">
-        <v>62</v>
-      </c>
-      <c r="E81" s="108" t="s">
-        <v>134</v>
-      </c>
-      <c r="F81" s="107" t="s">
-        <v>310</v>
-      </c>
-      <c r="G81" s="108" t="s">
-        <v>174</v>
-      </c>
-      <c r="H81" s="107" t="s">
+      <c r="D81" s="103" t="s">
+        <v>61</v>
+      </c>
+      <c r="E81" s="104" t="s">
+        <v>133</v>
+      </c>
+      <c r="F81" s="103" t="s">
+        <v>173</v>
+      </c>
+      <c r="G81" s="104" t="s">
+        <v>222</v>
+      </c>
+      <c r="H81" s="103" t="s">
         <v>256</v>
       </c>
-      <c r="I81" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="J81" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="K81" s="108" t="s">
-        <v>314</v>
-      </c>
-      <c r="L81" s="107">
+      <c r="I81" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="J81" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="K81" s="104" t="s">
+        <v>314</v>
+      </c>
+      <c r="L81" s="103">
         <v>1</v>
       </c>
-      <c r="M81" s="109">
-        <f t="shared" si="59"/>
+      <c r="M81" s="96">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N81" s="109">
+      <c r="N81" s="96">
         <v>21</v>
       </c>
-      <c r="O81" s="110" t="s">
-        <v>409</v>
-      </c>
-      <c r="P81" s="109">
-        <v>3.637</v>
-      </c>
-      <c r="Q81" s="109">
-        <f t="shared" ref="Q81" si="76">P81*N81</f>
-        <v>76.376999999999995</v>
-      </c>
-      <c r="R81" s="109"/>
-      <c r="T81" t="s">
-        <v>62</v>
-      </c>
-      <c r="U81" t="s">
-        <v>174</v>
-      </c>
-      <c r="V81" t="s">
-        <v>314</v>
-      </c>
-      <c r="W81">
-        <v>1</v>
-      </c>
-      <c r="Y81" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z81" t="str">
-        <f t="shared" si="70"/>
-        <v>Match</v>
-      </c>
-      <c r="AA81" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB81" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="82" spans="1:28" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O81" s="105" t="s">
+        <v>343</v>
+      </c>
+      <c r="P81" s="96">
+        <v>0.69430000000000003</v>
+      </c>
+      <c r="Q81" s="96">
+        <f t="shared" ref="Q81" si="89">N81*P81</f>
+        <v>14.580300000000001</v>
+      </c>
+      <c r="R81" s="78"/>
+    </row>
+    <row r="82" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1"/>
       <c r="B82" s="53">
-        <f t="shared" si="0"/>
-        <v>73</v>
-      </c>
-      <c r="C82" s="102" t="s">
+        <v>55</v>
+      </c>
+      <c r="C82" s="106" t="s">
         <v>328</v>
       </c>
-      <c r="D82" s="103" t="s">
-        <v>63</v>
-      </c>
-      <c r="E82" s="104" t="s">
-        <v>135</v>
-      </c>
-      <c r="F82" s="103" t="s">
-        <v>175</v>
-      </c>
-      <c r="G82" s="104" t="s">
-        <v>223</v>
-      </c>
-      <c r="H82" s="103" t="s">
+      <c r="D82" s="107" t="s">
+        <v>62</v>
+      </c>
+      <c r="E82" s="108" t="s">
+        <v>134</v>
+      </c>
+      <c r="F82" s="107" t="s">
+        <v>310</v>
+      </c>
+      <c r="G82" s="108" t="s">
+        <v>174</v>
+      </c>
+      <c r="H82" s="107" t="s">
         <v>256</v>
       </c>
-      <c r="I82" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J82" s="103" t="s">
-        <v>414</v>
-      </c>
-      <c r="K82" s="104" t="s">
-        <v>314</v>
-      </c>
-      <c r="L82" s="103">
+      <c r="I82" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="J82" s="107" t="s">
+        <v>314</v>
+      </c>
+      <c r="K82" s="108" t="s">
+        <v>314</v>
+      </c>
+      <c r="L82" s="107">
         <v>1</v>
       </c>
-      <c r="M82" s="96">
-        <f t="shared" si="59"/>
+      <c r="M82" s="109">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N82" s="96">
+      <c r="N82" s="109">
         <v>21</v>
       </c>
-      <c r="O82" s="105" t="s">
-        <v>343</v>
-      </c>
-      <c r="P82" s="96">
-        <v>0.43280000000000002</v>
-      </c>
-      <c r="Q82" s="96">
-        <f t="shared" ref="Q82" si="77">N82*P82</f>
-        <v>9.0888000000000009</v>
-      </c>
-      <c r="R82" s="96"/>
-      <c r="T82" t="s">
-        <v>63</v>
-      </c>
-      <c r="U82" t="s">
-        <v>223</v>
-      </c>
-      <c r="V82" t="s">
-        <v>314</v>
-      </c>
-      <c r="W82">
-        <v>1</v>
-      </c>
-      <c r="Y82" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z82" t="str">
-        <f t="shared" si="70"/>
-        <v>Match</v>
-      </c>
-      <c r="AA82" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB82" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="83" spans="1:28" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O82" s="110" t="s">
+        <v>409</v>
+      </c>
+      <c r="P82" s="109">
+        <v>3.637</v>
+      </c>
+      <c r="Q82" s="109">
+        <f t="shared" ref="Q82" si="90">P82*N82</f>
+        <v>76.376999999999995</v>
+      </c>
+      <c r="R82" s="109"/>
+    </row>
+    <row r="83" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1"/>
       <c r="B83" s="53">
-        <f>ROW(B83) - ROW($B$9)</f>
+        <f t="shared" ref="B83:B88" si="91">ROW(B83) - ROW($B$9)</f>
         <v>74</v>
       </c>
-      <c r="C83" s="71" t="s">
+      <c r="C83" s="102" t="s">
         <v>328</v>
       </c>
-      <c r="D83" s="72" t="s">
-        <v>64</v>
-      </c>
-      <c r="E83" s="73" t="s">
-        <v>136</v>
-      </c>
-      <c r="F83" s="72" t="s">
-        <v>176</v>
-      </c>
-      <c r="G83" s="73" t="s">
-        <v>224</v>
-      </c>
-      <c r="H83" s="72" t="s">
-        <v>258</v>
-      </c>
-      <c r="I83" s="72" t="s">
-        <v>314</v>
-      </c>
-      <c r="J83" s="72" t="s">
-        <v>415</v>
-      </c>
-      <c r="K83" s="73" t="s">
-        <v>314</v>
-      </c>
-      <c r="L83" s="72">
+      <c r="D83" s="103" t="s">
+        <v>63</v>
+      </c>
+      <c r="E83" s="104" t="s">
+        <v>135</v>
+      </c>
+      <c r="F83" s="103" t="s">
+        <v>175</v>
+      </c>
+      <c r="G83" s="104" t="s">
+        <v>223</v>
+      </c>
+      <c r="H83" s="103" t="s">
+        <v>256</v>
+      </c>
+      <c r="I83" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J83" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="K83" s="104" t="s">
+        <v>314</v>
+      </c>
+      <c r="L83" s="103">
         <v>1</v>
       </c>
-      <c r="M83" s="74">
-        <f t="shared" si="59"/>
+      <c r="M83" s="96">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N83" s="74">
+      <c r="N83" s="96">
         <v>21</v>
       </c>
-      <c r="O83" s="75" t="s">
+      <c r="O83" s="105" t="s">
         <v>343</v>
       </c>
-      <c r="P83" s="74">
-        <v>7.4638</v>
-      </c>
-      <c r="Q83" s="74">
-        <f t="shared" ref="Q83" si="78">P83*N83</f>
-        <v>156.7398</v>
-      </c>
-      <c r="R83" s="74" t="s">
-        <v>438</v>
-      </c>
-      <c r="T83" t="s">
-        <v>64</v>
-      </c>
-      <c r="U83" t="s">
-        <v>224</v>
-      </c>
-      <c r="V83" t="s">
-        <v>314</v>
-      </c>
-      <c r="W83">
-        <v>1</v>
-      </c>
-      <c r="Y83" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z83" t="str">
-        <f t="shared" si="70"/>
-        <v>Match</v>
-      </c>
-      <c r="AA83" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB83" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="84" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P83" s="96">
+        <v>0.43280000000000002</v>
+      </c>
+      <c r="Q83" s="96">
+        <f t="shared" ref="Q83" si="92">N83*P83</f>
+        <v>9.0888000000000009</v>
+      </c>
+      <c r="R83" s="96"/>
+    </row>
+    <row r="84" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1"/>
       <c r="B84" s="53">
-        <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="C84" s="102" t="s">
+        <v>56</v>
+      </c>
+      <c r="C84" s="71" t="s">
         <v>328</v>
       </c>
-      <c r="D84" s="103" t="s">
-        <v>65</v>
-      </c>
-      <c r="E84" s="104" t="s">
-        <v>137</v>
-      </c>
-      <c r="F84" s="103" t="s">
-        <v>177</v>
-      </c>
-      <c r="G84" s="104" t="s">
-        <v>225</v>
-      </c>
-      <c r="H84" s="103" t="s">
-        <v>259</v>
-      </c>
-      <c r="I84" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="J84" s="103" t="s">
-        <v>314</v>
-      </c>
-      <c r="K84" s="114" t="s">
-        <v>314</v>
-      </c>
-      <c r="L84" s="103">
+      <c r="D84" s="72" t="s">
+        <v>64</v>
+      </c>
+      <c r="E84" s="73" t="s">
+        <v>136</v>
+      </c>
+      <c r="F84" s="72" t="s">
+        <v>176</v>
+      </c>
+      <c r="G84" s="73" t="s">
+        <v>224</v>
+      </c>
+      <c r="H84" s="72" t="s">
+        <v>258</v>
+      </c>
+      <c r="I84" s="72" t="s">
+        <v>314</v>
+      </c>
+      <c r="J84" s="72" t="s">
+        <v>415</v>
+      </c>
+      <c r="K84" s="73" t="s">
+        <v>314</v>
+      </c>
+      <c r="L84" s="72">
         <v>1</v>
       </c>
-      <c r="M84" s="96">
-        <f t="shared" si="59"/>
+      <c r="M84" s="74">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N84" s="96">
+      <c r="N84" s="74">
         <v>21</v>
       </c>
-      <c r="O84" s="105" t="s">
-        <v>409</v>
-      </c>
-      <c r="P84" s="96">
-        <v>2.6459999999999999</v>
-      </c>
-      <c r="Q84" s="96">
-        <f t="shared" ref="Q84" si="79">N84*P84</f>
-        <v>55.565999999999995</v>
-      </c>
-      <c r="R84" s="96"/>
-      <c r="T84" t="s">
-        <v>65</v>
-      </c>
-      <c r="U84" t="s">
-        <v>225</v>
-      </c>
-      <c r="V84" t="s">
-        <v>314</v>
-      </c>
-      <c r="W84">
-        <v>1</v>
-      </c>
-      <c r="Y84" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z84" t="str">
-        <f t="shared" si="70"/>
-        <v>Match</v>
-      </c>
-      <c r="AA84" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB84" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="85" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O84" s="75" t="s">
+        <v>343</v>
+      </c>
+      <c r="P84" s="74">
+        <v>7.4638</v>
+      </c>
+      <c r="Q84" s="74">
+        <f t="shared" ref="Q84" si="93">P84*N84</f>
+        <v>156.7398</v>
+      </c>
+      <c r="R84" s="74" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="85" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A85" s="1"/>
       <c r="B85" s="53">
-        <f>ROW(B85) - ROW($B$9)</f>
+        <f t="shared" ref="B85:B88" si="94">ROW(B85) - ROW($B$9)</f>
         <v>76</v>
       </c>
-      <c r="C85" s="106" t="s">
+      <c r="C85" s="102" t="s">
         <v>328</v>
       </c>
-      <c r="D85" s="107" t="s">
-        <v>454</v>
-      </c>
-      <c r="E85" s="108" t="s">
-        <v>138</v>
-      </c>
-      <c r="F85" s="107" t="s">
-        <v>311</v>
-      </c>
-      <c r="G85" s="108" t="s">
-        <v>178</v>
-      </c>
-      <c r="H85" s="107" t="s">
-        <v>256</v>
-      </c>
-      <c r="I85" s="107" t="s">
-        <v>416</v>
-      </c>
-      <c r="J85" s="107" t="s">
-        <v>417</v>
-      </c>
-      <c r="K85" s="108" t="s">
-        <v>314</v>
-      </c>
-      <c r="L85" s="115">
-        <v>2</v>
-      </c>
-      <c r="M85" s="109">
-        <f t="shared" si="59"/>
-        <v>40</v>
-      </c>
-      <c r="N85" s="109">
-        <v>42</v>
-      </c>
-      <c r="O85" s="110" t="s">
-        <v>343</v>
-      </c>
-      <c r="P85" s="109">
-        <v>2.2974000000000001</v>
-      </c>
-      <c r="Q85" s="109">
-        <f t="shared" ref="Q85" si="80">P85*N85</f>
-        <v>96.490800000000007</v>
-      </c>
-      <c r="R85" s="79"/>
-      <c r="T85" t="s">
-        <v>454</v>
-      </c>
-      <c r="U85" t="s">
-        <v>416</v>
-      </c>
-      <c r="V85" t="s">
-        <v>314</v>
-      </c>
-      <c r="W85">
-        <v>2</v>
-      </c>
-      <c r="Y85" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z85" t="str">
-        <f t="shared" si="70"/>
-        <v>Mismatch</v>
-      </c>
-      <c r="AA85" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB85" t="str">
+      <c r="D85" s="103" t="s">
+        <v>65</v>
+      </c>
+      <c r="E85" s="104" t="s">
+        <v>137</v>
+      </c>
+      <c r="F85" s="103" t="s">
+        <v>177</v>
+      </c>
+      <c r="G85" s="104" t="s">
+        <v>225</v>
+      </c>
+      <c r="H85" s="103" t="s">
+        <v>259</v>
+      </c>
+      <c r="I85" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="J85" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="K85" s="113" t="s">
+        <v>314</v>
+      </c>
+      <c r="L85" s="103">
+        <v>1</v>
+      </c>
+      <c r="M85" s="96">
         <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="86" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+      <c r="N85" s="96">
+        <v>21</v>
+      </c>
+      <c r="O85" s="105" t="s">
+        <v>409</v>
+      </c>
+      <c r="P85" s="96">
+        <v>2.6459999999999999</v>
+      </c>
+      <c r="Q85" s="96">
+        <f t="shared" ref="Q85" si="95">N85*P85</f>
+        <v>55.565999999999995</v>
+      </c>
+      <c r="R85" s="96"/>
+    </row>
+    <row r="86" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1"/>
       <c r="B86" s="53">
-        <f>ROW(B86) - ROW($B$9)</f>
-        <v>77</v>
-      </c>
-      <c r="C86" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="C86" s="106" t="s">
         <v>328</v>
       </c>
-      <c r="D86" s="37" t="s">
-        <v>66</v>
-      </c>
-      <c r="E86" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="F86" s="37" t="s">
-        <v>313</v>
-      </c>
-      <c r="G86" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="H86" s="37" t="s">
+      <c r="D86" s="107" t="s">
+        <v>454</v>
+      </c>
+      <c r="E86" s="108" t="s">
+        <v>138</v>
+      </c>
+      <c r="F86" s="107" t="s">
+        <v>311</v>
+      </c>
+      <c r="G86" s="108" t="s">
+        <v>178</v>
+      </c>
+      <c r="H86" s="107" t="s">
         <v>256</v>
       </c>
-      <c r="I86" s="62" t="s">
-        <v>314</v>
-      </c>
-      <c r="J86" s="62" t="s">
-        <v>420</v>
-      </c>
-      <c r="K86" s="38" t="s">
-        <v>314</v>
-      </c>
-      <c r="L86" s="37">
-        <v>1</v>
-      </c>
-      <c r="M86" s="41">
-        <f>L86*20</f>
-        <v>20</v>
-      </c>
-      <c r="N86" s="41">
-        <v>21</v>
-      </c>
-      <c r="O86" s="63" t="s">
+      <c r="I86" s="107" t="s">
+        <v>416</v>
+      </c>
+      <c r="J86" s="107" t="s">
+        <v>417</v>
+      </c>
+      <c r="K86" s="108" t="s">
+        <v>314</v>
+      </c>
+      <c r="L86" s="114">
+        <v>2</v>
+      </c>
+      <c r="M86" s="109">
+        <f t="shared" si="72"/>
+        <v>40</v>
+      </c>
+      <c r="N86" s="109">
+        <v>42</v>
+      </c>
+      <c r="O86" s="110" t="s">
         <v>343</v>
       </c>
-      <c r="P86" s="41">
-        <v>0.39140000000000003</v>
-      </c>
-      <c r="Q86" s="41">
-        <f t="shared" ref="Q86" si="81">P86*N86</f>
-        <v>8.2194000000000003</v>
-      </c>
-      <c r="R86" s="41"/>
-      <c r="T86" t="s">
-        <v>66</v>
-      </c>
-      <c r="U86" t="s">
-        <v>180</v>
-      </c>
-      <c r="V86" t="s">
-        <v>314</v>
-      </c>
-      <c r="W86">
-        <v>1</v>
-      </c>
-      <c r="Y86" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z86" t="str">
-        <f t="shared" si="70"/>
-        <v>Match</v>
-      </c>
-      <c r="AA86" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB86" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="87" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P86" s="109">
+        <v>2.2974000000000001</v>
+      </c>
+      <c r="Q86" s="109">
+        <f t="shared" ref="Q86" si="96">P86*N86</f>
+        <v>96.490800000000007</v>
+      </c>
+      <c r="R86" s="79"/>
+    </row>
+    <row r="87" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1"/>
       <c r="B87" s="53">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B87:B88" si="97">ROW(B87) - ROW($B$9)</f>
         <v>78</v>
       </c>
-      <c r="C87" s="59" t="s">
+      <c r="C87" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="D87" s="39" t="s">
+      <c r="D87" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="E87" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="F87" s="37" t="s">
+        <v>313</v>
+      </c>
+      <c r="G87" s="38" t="s">
+        <v>180</v>
+      </c>
+      <c r="H87" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="I87" s="62" t="s">
+        <v>314</v>
+      </c>
+      <c r="J87" s="62" t="s">
+        <v>420</v>
+      </c>
+      <c r="K87" s="38" t="s">
+        <v>314</v>
+      </c>
+      <c r="L87" s="37">
+        <v>1</v>
+      </c>
+      <c r="M87" s="41">
+        <f>L87*20</f>
+        <v>20</v>
+      </c>
+      <c r="N87" s="41">
+        <v>21</v>
+      </c>
+      <c r="O87" s="63" t="s">
+        <v>343</v>
+      </c>
+      <c r="P87" s="41">
+        <v>0.39140000000000003</v>
+      </c>
+      <c r="Q87" s="41">
+        <f t="shared" ref="Q87" si="98">P87*N87</f>
+        <v>8.2194000000000003</v>
+      </c>
+      <c r="R87" s="41"/>
+    </row>
+    <row r="88" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A88" s="1"/>
+      <c r="B88" s="53">
+        <v>58</v>
+      </c>
+      <c r="C88" s="59" t="s">
+        <v>328</v>
+      </c>
+      <c r="D88" s="39" t="s">
         <v>455</v>
       </c>
-      <c r="E87" s="40" t="s">
+      <c r="E88" s="40" t="s">
         <v>139</v>
       </c>
-      <c r="F87" s="39" t="s">
+      <c r="F88" s="39" t="s">
         <v>312</v>
       </c>
-      <c r="G87" s="40" t="s">
+      <c r="G88" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="H87" s="39" t="s">
+      <c r="H88" s="39" t="s">
         <v>259</v>
       </c>
-      <c r="I87" s="39" t="s">
+      <c r="I88" s="39" t="s">
         <v>418</v>
       </c>
-      <c r="J87" s="39" t="s">
-        <v>314</v>
-      </c>
-      <c r="K87" s="40" t="s">
-        <v>314</v>
-      </c>
-      <c r="L87" s="39">
+      <c r="J88" s="39" t="s">
+        <v>314</v>
+      </c>
+      <c r="K88" s="40" t="s">
+        <v>314</v>
+      </c>
+      <c r="L88" s="39">
         <v>1</v>
       </c>
-      <c r="M87" s="42">
-        <f t="shared" si="59"/>
+      <c r="M88" s="42">
+        <f t="shared" si="72"/>
         <v>20</v>
       </c>
-      <c r="N87" s="42">
+      <c r="N88" s="42">
         <v>21</v>
       </c>
-      <c r="O87" s="64" t="s">
+      <c r="O88" s="64" t="s">
         <v>419</v>
       </c>
-      <c r="P87" s="42">
+      <c r="P88" s="42">
         <v>3.532</v>
       </c>
-      <c r="Q87" s="42">
-        <f t="shared" ref="Q87" si="82">N87*P87</f>
+      <c r="Q88" s="42">
+        <f t="shared" ref="Q88" si="99">N88*P88</f>
         <v>74.171999999999997</v>
       </c>
-      <c r="R87" s="79"/>
-      <c r="T87" t="s">
-        <v>455</v>
-      </c>
-      <c r="U87" t="s">
-        <v>418</v>
-      </c>
-      <c r="V87" t="s">
-        <v>314</v>
-      </c>
-      <c r="W87">
-        <v>1</v>
-      </c>
-      <c r="Y87" t="str">
-        <f t="shared" si="69"/>
-        <v>Match</v>
-      </c>
-      <c r="Z87" t="str">
-        <f t="shared" si="70"/>
-        <v>Mismatch</v>
-      </c>
-      <c r="AA87" t="str">
-        <f t="shared" si="71"/>
-        <v>Match</v>
-      </c>
-      <c r="AB87" t="str">
-        <f t="shared" si="72"/>
-        <v>Match</v>
-      </c>
-    </row>
-    <row r="88" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A88" s="1"/>
-      <c r="B88" s="32"/>
-      <c r="C88" s="51"/>
-      <c r="D88" s="33" t="s">
+      <c r="R88" s="79"/>
+    </row>
+    <row r="89" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A89" s="1"/>
+      <c r="B89" s="32"/>
+      <c r="C89" s="51"/>
+      <c r="D89" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="E88" s="34"/>
-      <c r="F88" s="35"/>
-      <c r="G88" s="36"/>
-      <c r="H88" s="35"/>
-      <c r="I88" s="35"/>
-      <c r="J88" s="35"/>
-      <c r="K88" s="36"/>
-      <c r="L88" s="36"/>
-      <c r="M88" s="36"/>
-      <c r="N88" s="36"/>
-      <c r="O88" s="69" t="s">
+      <c r="E89" s="34"/>
+      <c r="F89" s="35"/>
+      <c r="G89" s="36"/>
+      <c r="H89" s="35"/>
+      <c r="I89" s="35"/>
+      <c r="J89" s="35"/>
+      <c r="K89" s="36"/>
+      <c r="L89" s="36"/>
+      <c r="M89" s="36"/>
+      <c r="N89" s="36"/>
+      <c r="O89" s="69" t="s">
         <v>421</v>
       </c>
-      <c r="P88" s="67"/>
-      <c r="Q88" s="67">
-        <f>SUM(Q10:Q87)</f>
-        <v>960.72630000000004</v>
-      </c>
-      <c r="R88" s="44"/>
-    </row>
-    <row r="89" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A89" s="1"/>
-      <c r="B89" s="24"/>
-      <c r="C89" s="52"/>
-      <c r="D89" s="8" t="s">
+      <c r="P89" s="67"/>
+      <c r="Q89" s="67">
+        <f>SUM(Q10:Q88)</f>
+        <v>969.96630000000005</v>
+      </c>
+      <c r="R89" s="44"/>
+    </row>
+    <row r="90" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A90" s="1"/>
+      <c r="B90" s="24"/>
+      <c r="C90" s="52"/>
+      <c r="D90" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E89" s="9"/>
-      <c r="F89" s="9"/>
-      <c r="G89" s="9"/>
-      <c r="H89" s="9"/>
-      <c r="I89" s="9"/>
-      <c r="J89" s="9"/>
-      <c r="K89" s="9"/>
-      <c r="L89" s="9"/>
-      <c r="M89" s="9"/>
-      <c r="N89" s="9"/>
-      <c r="O89" s="70" t="s">
+      <c r="E90" s="9"/>
+      <c r="F90" s="9"/>
+      <c r="G90" s="9"/>
+      <c r="H90" s="9"/>
+      <c r="I90" s="9"/>
+      <c r="J90" s="9"/>
+      <c r="K90" s="9"/>
+      <c r="L90" s="9"/>
+      <c r="M90" s="9"/>
+      <c r="N90" s="9"/>
+      <c r="O90" s="70" t="s">
         <v>422</v>
       </c>
-      <c r="P89" s="68"/>
-      <c r="Q89" s="68">
-        <f>Q88/20</f>
-        <v>48.036315000000002</v>
-      </c>
-      <c r="R89" s="45"/>
+      <c r="P90" s="68"/>
+      <c r="Q90" s="68">
+        <f>Q89/20</f>
+        <v>48.498315000000005</v>
+      </c>
+      <c r="R90" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7702,47 +7419,48 @@
     <hyperlink ref="O43" r:id="rId34"/>
     <hyperlink ref="O44" r:id="rId35"/>
     <hyperlink ref="O45" r:id="rId36"/>
-    <hyperlink ref="O46" r:id="rId37"/>
-    <hyperlink ref="O48" r:id="rId38"/>
-    <hyperlink ref="O49" r:id="rId39"/>
-    <hyperlink ref="O50" r:id="rId40"/>
-    <hyperlink ref="O51" r:id="rId41"/>
-    <hyperlink ref="O52" r:id="rId42"/>
-    <hyperlink ref="O53" r:id="rId43"/>
-    <hyperlink ref="O54" r:id="rId44"/>
-    <hyperlink ref="O55" r:id="rId45"/>
-    <hyperlink ref="O67" r:id="rId46"/>
-    <hyperlink ref="O57" r:id="rId47"/>
-    <hyperlink ref="O58" r:id="rId48"/>
-    <hyperlink ref="O59" r:id="rId49"/>
-    <hyperlink ref="O60" r:id="rId50"/>
-    <hyperlink ref="O61" r:id="rId51"/>
-    <hyperlink ref="O62" r:id="rId52"/>
-    <hyperlink ref="O63" r:id="rId53"/>
-    <hyperlink ref="O64" r:id="rId54"/>
-    <hyperlink ref="O65" r:id="rId55"/>
-    <hyperlink ref="O66" r:id="rId56"/>
-    <hyperlink ref="O68" r:id="rId57"/>
-    <hyperlink ref="O69" r:id="rId58"/>
-    <hyperlink ref="O70" r:id="rId59"/>
-    <hyperlink ref="O73" r:id="rId60"/>
-    <hyperlink ref="O74" r:id="rId61"/>
-    <hyperlink ref="O71" r:id="rId62"/>
-    <hyperlink ref="O77" r:id="rId63"/>
-    <hyperlink ref="O78" r:id="rId64"/>
-    <hyperlink ref="O79" r:id="rId65"/>
-    <hyperlink ref="O80" r:id="rId66"/>
-    <hyperlink ref="O81" r:id="rId67"/>
-    <hyperlink ref="O82" r:id="rId68"/>
-    <hyperlink ref="O83" r:id="rId69"/>
-    <hyperlink ref="O84" r:id="rId70"/>
-    <hyperlink ref="O85" r:id="rId71"/>
-    <hyperlink ref="O87" r:id="rId72"/>
-    <hyperlink ref="O86" r:id="rId73"/>
-    <hyperlink ref="O56" r:id="rId74"/>
+    <hyperlink ref="O47" r:id="rId37"/>
+    <hyperlink ref="O49" r:id="rId38"/>
+    <hyperlink ref="O50" r:id="rId39"/>
+    <hyperlink ref="O51" r:id="rId40"/>
+    <hyperlink ref="O52" r:id="rId41"/>
+    <hyperlink ref="O53" r:id="rId42"/>
+    <hyperlink ref="O54" r:id="rId43"/>
+    <hyperlink ref="O55" r:id="rId44"/>
+    <hyperlink ref="O56" r:id="rId45"/>
+    <hyperlink ref="O68" r:id="rId46"/>
+    <hyperlink ref="O58" r:id="rId47"/>
+    <hyperlink ref="O59" r:id="rId48"/>
+    <hyperlink ref="O60" r:id="rId49"/>
+    <hyperlink ref="O61" r:id="rId50"/>
+    <hyperlink ref="O62" r:id="rId51"/>
+    <hyperlink ref="O63" r:id="rId52"/>
+    <hyperlink ref="O64" r:id="rId53"/>
+    <hyperlink ref="O65" r:id="rId54"/>
+    <hyperlink ref="O66" r:id="rId55"/>
+    <hyperlink ref="O67" r:id="rId56"/>
+    <hyperlink ref="O69" r:id="rId57"/>
+    <hyperlink ref="O70" r:id="rId58"/>
+    <hyperlink ref="O71" r:id="rId59"/>
+    <hyperlink ref="O74" r:id="rId60"/>
+    <hyperlink ref="O75" r:id="rId61"/>
+    <hyperlink ref="O72" r:id="rId62"/>
+    <hyperlink ref="O78" r:id="rId63"/>
+    <hyperlink ref="O79" r:id="rId64"/>
+    <hyperlink ref="O80" r:id="rId65"/>
+    <hyperlink ref="O81" r:id="rId66"/>
+    <hyperlink ref="O82" r:id="rId67"/>
+    <hyperlink ref="O83" r:id="rId68"/>
+    <hyperlink ref="O84" r:id="rId69"/>
+    <hyperlink ref="O85" r:id="rId70"/>
+    <hyperlink ref="O86" r:id="rId71"/>
+    <hyperlink ref="O88" r:id="rId72"/>
+    <hyperlink ref="O87" r:id="rId73"/>
+    <hyperlink ref="O57" r:id="rId74"/>
+    <hyperlink ref="O46" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId75"/>
-  <drawing r:id="rId76"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId76"/>
+  <drawing r:id="rId77"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
LED Glass pipe link corrected #143
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/eSpark BOM_Top (20 Boards).xlsx
+++ b/Deliverables/SM_Top Board/_BOM/eSpark BOM_Top (20 Boards).xlsx
@@ -5,16 +5,16 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11496" windowHeight="7596"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11490" windowHeight="7590"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="470">
   <si>
     <t>Component list</t>
   </si>
@@ -1563,25 +1563,22 @@
     <t>LED Glass Pipe</t>
   </si>
   <si>
-    <t>LED Light Pipes PCB Mount</t>
-  </si>
-  <si>
-    <t>3mm .5 inch</t>
-  </si>
-  <si>
-    <t>VBL3D0500C</t>
-  </si>
-  <si>
-    <t>VCC</t>
-  </si>
-  <si>
     <t>Mounting Holes required in design</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> LIGHT PIPE VERT 0.500" RND FACE</t>
+  </si>
+  <si>
+    <t>VLP-500-R</t>
+  </si>
+  <si>
+    <t>Bivar Inc.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -2455,7 +2452,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2754,26 +2751,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R90"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.109375" style="25" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="30.109375" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="22.109375" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="16.6640625" customWidth="1"/>
-    <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="30.140625" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="22.140625" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="16.7109375" customWidth="1"/>
+    <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -2793,7 +2790,7 @@
       <c r="Q1" s="115"/>
       <c r="R1" s="115"/>
     </row>
-    <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="46"/>
@@ -2817,7 +2814,7 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="43"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="47"/>
@@ -2841,7 +2838,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="116"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="47"/>
@@ -2865,7 +2862,7 @@
       <c r="Q4" s="61"/>
       <c r="R4" s="117"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="47"/>
@@ -2887,7 +2884,7 @@
       <c r="Q5" s="61"/>
       <c r="R5" s="117"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="48"/>
@@ -2907,7 +2904,7 @@
       <c r="Q6" s="61"/>
       <c r="R6" s="117"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="49"/>
@@ -2927,7 +2924,7 @@
       <c r="Q7" s="7"/>
       <c r="R7" s="117"/>
     </row>
-    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="50"/>
@@ -2947,7 +2944,7 @@
       <c r="Q8" s="7"/>
       <c r="R8" s="117"/>
     </row>
-    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -3001,7 +2998,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="53">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -3056,10 +3053,10 @@
       </c>
       <c r="R10" s="41"/>
     </row>
-    <row r="11" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="53">
-        <f t="shared" ref="B11:B88" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B44" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="81" t="s">
@@ -3113,7 +3110,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -3168,7 +3165,7 @@
       </c>
       <c r="R12" s="76"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="53">
         <f t="shared" si="0"/>
@@ -3223,7 +3220,7 @@
       </c>
       <c r="R13" s="77"/>
     </row>
-    <row r="14" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="53">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -3278,7 +3275,7 @@
       </c>
       <c r="R14" s="76"/>
     </row>
-    <row r="15" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="53">
         <f t="shared" si="0"/>
@@ -3333,7 +3330,7 @@
       </c>
       <c r="R15" s="77"/>
     </row>
-    <row r="16" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="53">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -3388,7 +3385,7 @@
       </c>
       <c r="R16" s="76"/>
     </row>
-    <row r="17" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
         <f t="shared" si="0"/>
@@ -3443,7 +3440,7 @@
       </c>
       <c r="R17" s="42"/>
     </row>
-    <row r="18" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
         <f t="shared" si="0"/>
@@ -3498,7 +3495,7 @@
       </c>
       <c r="R18" s="96"/>
     </row>
-    <row r="19" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
         <f>ROW(B19) - ROW($B$9)</f>
@@ -3553,7 +3550,7 @@
       </c>
       <c r="R19" s="109"/>
     </row>
-    <row r="20" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="53">
         <f t="shared" si="0"/>
@@ -3608,7 +3605,7 @@
       </c>
       <c r="R20" s="96"/>
     </row>
-    <row r="21" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
         <f>ROW(B21) - ROW($B$9)</f>
@@ -3663,7 +3660,7 @@
       </c>
       <c r="R21" s="109"/>
     </row>
-    <row r="22" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="53">
         <f>ROW(B22) - ROW($B$9)</f>
@@ -3718,7 +3715,7 @@
       </c>
       <c r="R22" s="41"/>
     </row>
-    <row r="23" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="53">
         <f t="shared" si="0"/>
@@ -3773,7 +3770,7 @@
       </c>
       <c r="R23" s="77"/>
     </row>
-    <row r="24" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="53">
         <f>ROW(B24) - ROW($B$9)</f>
@@ -3828,7 +3825,7 @@
       </c>
       <c r="R24" s="41"/>
     </row>
-    <row r="25" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="53">
         <f t="shared" si="0"/>
@@ -3883,7 +3880,7 @@
       </c>
       <c r="R25" s="42"/>
     </row>
-    <row r="26" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="53">
         <f t="shared" si="0"/>
@@ -3938,7 +3935,7 @@
       </c>
       <c r="R26" s="76"/>
     </row>
-    <row r="27" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="53">
         <f>ROW(B27) - ROW($B$9)</f>
@@ -3993,7 +3990,7 @@
       </c>
       <c r="R27" s="79"/>
     </row>
-    <row r="28" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="53">
         <f>ROW(B28) - ROW($B$9)</f>
@@ -4048,7 +4045,7 @@
       </c>
       <c r="R28" s="41"/>
     </row>
-    <row r="29" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="53">
         <f t="shared" si="0"/>
@@ -4103,7 +4100,7 @@
       </c>
       <c r="R29" s="42"/>
     </row>
-    <row r="30" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="53">
         <f>ROW(B30) - ROW($B$9)</f>
@@ -4158,7 +4155,7 @@
       </c>
       <c r="R30" s="41"/>
     </row>
-    <row r="31" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="53">
         <f>ROW(B31) - ROW($B$9)</f>
@@ -4213,7 +4210,7 @@
       </c>
       <c r="R31" s="109"/>
     </row>
-    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="53">
         <f t="shared" si="0"/>
@@ -4268,7 +4265,7 @@
       </c>
       <c r="R32" s="96"/>
     </row>
-    <row r="33" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="53">
         <f>ROW(B33) - ROW($B$9)</f>
@@ -4323,7 +4320,7 @@
       </c>
       <c r="R33" s="109"/>
     </row>
-    <row r="34" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f t="shared" si="0"/>
@@ -4378,7 +4375,7 @@
       </c>
       <c r="R34" s="78"/>
     </row>
-    <row r="35" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f>ROW(B35) - ROW($B$9)</f>
@@ -4435,7 +4432,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f t="shared" si="0"/>
@@ -4490,7 +4487,7 @@
       </c>
       <c r="R36" s="96"/>
     </row>
-    <row r="37" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="53">
         <f>ROW(B37) - ROW($B$9)</f>
@@ -4545,7 +4542,7 @@
       </c>
       <c r="R37" s="109"/>
     </row>
-    <row r="38" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="53">
         <f t="shared" si="0"/>
@@ -4600,7 +4597,7 @@
       </c>
       <c r="R38" s="78"/>
     </row>
-    <row r="39" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="53">
         <f>ROW(B39) - ROW($B$9)</f>
@@ -4655,7 +4652,7 @@
       </c>
       <c r="R39" s="79"/>
     </row>
-    <row r="40" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="53">
         <f t="shared" si="0"/>
@@ -4710,7 +4707,7 @@
       </c>
       <c r="R40" s="96"/>
     </row>
-    <row r="41" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="53">
         <f>ROW(B41) - ROW($B$9)</f>
@@ -4765,7 +4762,7 @@
       </c>
       <c r="R41" s="109"/>
     </row>
-    <row r="42" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="53">
         <f t="shared" si="0"/>
@@ -4820,7 +4817,7 @@
       </c>
       <c r="R42" s="96"/>
     </row>
-    <row r="43" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="53">
         <f>ROW(B43) - ROW($B$9)</f>
@@ -4875,7 +4872,7 @@
       </c>
       <c r="R43" s="77"/>
     </row>
-    <row r="44" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="53">
         <f t="shared" si="0"/>
@@ -4930,7 +4927,7 @@
       </c>
       <c r="R44" s="96"/>
     </row>
-    <row r="45" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="53">
         <f>ROW(B45) - ROW($B$9)</f>
@@ -4985,7 +4982,7 @@
       </c>
       <c r="R45" s="109"/>
     </row>
-    <row r="46" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="53">
         <v>37</v>
@@ -4997,10 +4994,10 @@
         <v>314</v>
       </c>
       <c r="E46" s="108" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F46" s="107" t="s">
-        <v>467</v>
+        <v>308</v>
       </c>
       <c r="G46" s="108" t="s">
         <v>468</v>
@@ -5028,23 +5025,23 @@
         <v>20</v>
       </c>
       <c r="O46" s="110" t="s">
-        <v>379</v>
+        <v>419</v>
       </c>
       <c r="P46" s="109">
-        <v>0.46200000000000002</v>
+        <v>0.435</v>
       </c>
       <c r="Q46" s="109">
         <f t="shared" si="34"/>
-        <v>9.24</v>
-      </c>
-      <c r="R46" s="109" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="47" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="R46" s="79" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="53">
-        <f t="shared" ref="B47:B88" si="35">ROW(B47) - ROW($B$9)</f>
+        <f t="shared" ref="B47" si="35">ROW(B47) - ROW($B$9)</f>
         <v>38</v>
       </c>
       <c r="C47" s="102" t="s">
@@ -5096,7 +5093,7 @@
       </c>
       <c r="R47" s="96"/>
     </row>
-    <row r="48" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="53">
         <v>38</v>
@@ -5145,10 +5142,10 @@
         <v>384</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="53">
-        <f t="shared" ref="B49:B88" si="39">ROW(B49) - ROW($B$9)</f>
+        <f t="shared" ref="B49" si="39">ROW(B49) - ROW($B$9)</f>
         <v>40</v>
       </c>
       <c r="C49" s="102" t="s">
@@ -5200,7 +5197,7 @@
       </c>
       <c r="R49" s="96"/>
     </row>
-    <row r="50" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="53">
         <v>39</v>
@@ -5254,10 +5251,10 @@
       </c>
       <c r="R50" s="109"/>
     </row>
-    <row r="51" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="53">
-        <f t="shared" ref="B51:B88" si="42">ROW(B51) - ROW($B$9)</f>
+        <f t="shared" ref="B51" si="42">ROW(B51) - ROW($B$9)</f>
         <v>42</v>
       </c>
       <c r="C51" s="102" t="s">
@@ -5309,7 +5306,7 @@
       </c>
       <c r="R51" s="96"/>
     </row>
-    <row r="52" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="53">
         <v>40</v>
@@ -5363,10 +5360,10 @@
       </c>
       <c r="R52" s="109"/>
     </row>
-    <row r="53" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="53">
-        <f t="shared" ref="B53:B88" si="45">ROW(B53) - ROW($B$9)</f>
+        <f t="shared" ref="B53" si="45">ROW(B53) - ROW($B$9)</f>
         <v>44</v>
       </c>
       <c r="C53" s="102" t="s">
@@ -5418,7 +5415,7 @@
       </c>
       <c r="R53" s="96"/>
     </row>
-    <row r="54" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="53">
         <v>41</v>
@@ -5472,10 +5469,10 @@
       </c>
       <c r="R54" s="109"/>
     </row>
-    <row r="55" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="53">
-        <f t="shared" ref="B55:B88" si="48">ROW(B55) - ROW($B$9)</f>
+        <f t="shared" ref="B55" si="48">ROW(B55) - ROW($B$9)</f>
         <v>46</v>
       </c>
       <c r="C55" s="102" t="s">
@@ -5527,7 +5524,7 @@
       </c>
       <c r="R55" s="96"/>
     </row>
-    <row r="56" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="53">
         <v>42</v>
@@ -5581,10 +5578,10 @@
       </c>
       <c r="R56" s="109"/>
     </row>
-    <row r="57" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="53">
-        <f t="shared" ref="B57:B88" si="51">ROW(B57) - ROW($B$9)</f>
+        <f t="shared" ref="B57" si="51">ROW(B57) - ROW($B$9)</f>
         <v>48</v>
       </c>
       <c r="C57" s="60" t="s">
@@ -5636,7 +5633,7 @@
       </c>
       <c r="R57" s="76"/>
     </row>
-    <row r="58" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="53">
         <v>43</v>
@@ -5690,10 +5687,10 @@
       </c>
       <c r="R58" s="109"/>
     </row>
-    <row r="59" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="53">
-        <f t="shared" ref="B59:B88" si="54">ROW(B59) - ROW($B$9)</f>
+        <f t="shared" ref="B59" si="54">ROW(B59) - ROW($B$9)</f>
         <v>50</v>
       </c>
       <c r="C59" s="102" t="s">
@@ -5745,7 +5742,7 @@
       </c>
       <c r="R59" s="96"/>
     </row>
-    <row r="60" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="53">
         <v>44</v>
@@ -5799,10 +5796,10 @@
       </c>
       <c r="R60" s="109"/>
     </row>
-    <row r="61" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="53">
-        <f t="shared" ref="B61:B88" si="57">ROW(B61) - ROW($B$9)</f>
+        <f t="shared" ref="B61" si="57">ROW(B61) - ROW($B$9)</f>
         <v>52</v>
       </c>
       <c r="C61" s="102" t="s">
@@ -5854,7 +5851,7 @@
       </c>
       <c r="R61" s="96"/>
     </row>
-    <row r="62" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="53">
         <v>45</v>
@@ -5908,10 +5905,10 @@
       </c>
       <c r="R62" s="109"/>
     </row>
-    <row r="63" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="53">
-        <f t="shared" ref="B63:B88" si="60">ROW(B63) - ROW($B$9)</f>
+        <f t="shared" ref="B63" si="60">ROW(B63) - ROW($B$9)</f>
         <v>54</v>
       </c>
       <c r="C63" s="102" t="s">
@@ -5963,7 +5960,7 @@
       </c>
       <c r="R63" s="96"/>
     </row>
-    <row r="64" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="53">
         <v>46</v>
@@ -6017,10 +6014,10 @@
       </c>
       <c r="R64" s="109"/>
     </row>
-    <row r="65" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="53">
-        <f t="shared" ref="B65:B88" si="63">ROW(B65) - ROW($B$9)</f>
+        <f t="shared" ref="B65" si="63">ROW(B65) - ROW($B$9)</f>
         <v>56</v>
       </c>
       <c r="C65" s="102" t="s">
@@ -6072,7 +6069,7 @@
       </c>
       <c r="R65" s="96"/>
     </row>
-    <row r="66" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="53">
         <v>47</v>
@@ -6126,10 +6123,10 @@
       </c>
       <c r="R66" s="109"/>
     </row>
-    <row r="67" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="53">
-        <f t="shared" ref="B67:B88" si="66">ROW(B67) - ROW($B$9)</f>
+        <f t="shared" ref="B67" si="66">ROW(B67) - ROW($B$9)</f>
         <v>58</v>
       </c>
       <c r="C67" s="60" t="s">
@@ -6181,7 +6178,7 @@
       </c>
       <c r="R67" s="41"/>
     </row>
-    <row r="68" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="53">
         <v>48</v>
@@ -6233,10 +6230,10 @@
       </c>
       <c r="R68" s="77"/>
     </row>
-    <row r="69" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="53">
-        <f t="shared" ref="B69:B88" si="68">ROW(B69) - ROW($B$9)</f>
+        <f t="shared" ref="B69" si="68">ROW(B69) - ROW($B$9)</f>
         <v>60</v>
       </c>
       <c r="C69" s="60" t="s">
@@ -6288,7 +6285,7 @@
       </c>
       <c r="R69" s="41"/>
     </row>
-    <row r="70" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="53">
         <v>49</v>
@@ -6342,10 +6339,10 @@
       </c>
       <c r="R70" s="42"/>
     </row>
-    <row r="71" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="53">
-        <f t="shared" ref="B71:B88" si="71">ROW(B71) - ROW($B$9)</f>
+        <f t="shared" ref="B71" si="71">ROW(B71) - ROW($B$9)</f>
         <v>62</v>
       </c>
       <c r="C71" s="60" t="s">
@@ -6397,7 +6394,7 @@
       </c>
       <c r="R71" s="76"/>
     </row>
-    <row r="72" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="53">
         <v>50</v>
@@ -6451,10 +6448,10 @@
       </c>
       <c r="R72" s="77"/>
     </row>
-    <row r="73" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="53">
-        <f t="shared" ref="B73:B88" si="75">ROW(B73) - ROW($B$9)</f>
+        <f t="shared" ref="B73" si="75">ROW(B73) - ROW($B$9)</f>
         <v>64</v>
       </c>
       <c r="C73" s="60" t="s">
@@ -6506,7 +6503,7 @@
       </c>
       <c r="R73" s="41"/>
     </row>
-    <row r="74" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="53">
         <v>51</v>
@@ -6560,10 +6557,10 @@
       </c>
       <c r="R74" s="42"/>
     </row>
-    <row r="75" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="53">
-        <f t="shared" ref="B75:B88" si="78">ROW(B75) - ROW($B$9)</f>
+        <f t="shared" ref="B75" si="78">ROW(B75) - ROW($B$9)</f>
         <v>66</v>
       </c>
       <c r="C75" s="97" t="s">
@@ -6617,7 +6614,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="53">
         <v>52</v>
@@ -6670,10 +6667,10 @@
         <v>384</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="53">
-        <f t="shared" ref="B77:B88" si="82">ROW(B77) - ROW($B$9)</f>
+        <f t="shared" ref="B77" si="82">ROW(B77) - ROW($B$9)</f>
         <v>68</v>
       </c>
       <c r="C77" s="102" t="s">
@@ -6722,7 +6719,7 @@
       </c>
       <c r="R77" s="96"/>
     </row>
-    <row r="78" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="53">
         <v>53</v>
@@ -6776,10 +6773,10 @@
       </c>
       <c r="R78" s="109"/>
     </row>
-    <row r="79" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="53">
-        <f t="shared" ref="B79:B88" si="85">ROW(B79) - ROW($B$9)</f>
+        <f t="shared" ref="B79" si="85">ROW(B79) - ROW($B$9)</f>
         <v>70</v>
       </c>
       <c r="C79" s="102" t="s">
@@ -6831,7 +6828,7 @@
       </c>
       <c r="R79" s="96"/>
     </row>
-    <row r="80" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="53">
         <v>54</v>
@@ -6885,10 +6882,10 @@
       </c>
       <c r="R80" s="79"/>
     </row>
-    <row r="81" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="53">
-        <f t="shared" ref="B81:B88" si="88">ROW(B81) - ROW($B$9)</f>
+        <f t="shared" ref="B81" si="88">ROW(B81) - ROW($B$9)</f>
         <v>72</v>
       </c>
       <c r="C81" s="102" t="s">
@@ -6940,7 +6937,7 @@
       </c>
       <c r="R81" s="78"/>
     </row>
-    <row r="82" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="53">
         <v>55</v>
@@ -6994,10 +6991,10 @@
       </c>
       <c r="R82" s="109"/>
     </row>
-    <row r="83" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
       <c r="B83" s="53">
-        <f t="shared" ref="B83:B88" si="91">ROW(B83) - ROW($B$9)</f>
+        <f t="shared" ref="B83" si="91">ROW(B83) - ROW($B$9)</f>
         <v>74</v>
       </c>
       <c r="C83" s="102" t="s">
@@ -7049,7 +7046,7 @@
       </c>
       <c r="R83" s="96"/>
     </row>
-    <row r="84" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
       <c r="B84" s="53">
         <v>56</v>
@@ -7105,10 +7102,10 @@
         <v>438</v>
       </c>
     </row>
-    <row r="85" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
       <c r="B85" s="53">
-        <f t="shared" ref="B85:B88" si="94">ROW(B85) - ROW($B$9)</f>
+        <f t="shared" ref="B85" si="94">ROW(B85) - ROW($B$9)</f>
         <v>76</v>
       </c>
       <c r="C85" s="102" t="s">
@@ -7160,7 +7157,7 @@
       </c>
       <c r="R85" s="96"/>
     </row>
-    <row r="86" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
       <c r="B86" s="53">
         <v>57</v>
@@ -7214,10 +7211,10 @@
       </c>
       <c r="R86" s="79"/>
     </row>
-    <row r="87" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
       <c r="B87" s="53">
-        <f t="shared" ref="B87:B88" si="97">ROW(B87) - ROW($B$9)</f>
+        <f t="shared" ref="B87" si="97">ROW(B87) - ROW($B$9)</f>
         <v>78</v>
       </c>
       <c r="C87" s="60" t="s">
@@ -7269,7 +7266,7 @@
       </c>
       <c r="R87" s="41"/>
     </row>
-    <row r="88" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
       <c r="B88" s="53">
         <v>58</v>
@@ -7323,7 +7320,7 @@
       </c>
       <c r="R88" s="79"/>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="B89" s="32"/>
       <c r="C89" s="51"/>
@@ -7346,11 +7343,11 @@
       <c r="P89" s="67"/>
       <c r="Q89" s="67">
         <f>SUM(Q10:Q88)</f>
-        <v>969.96630000000005</v>
+        <v>969.42630000000008</v>
       </c>
       <c r="R89" s="44"/>
     </row>
-    <row r="90" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1"/>
       <c r="B90" s="24"/>
       <c r="C90" s="52"/>
@@ -7373,7 +7370,7 @@
       <c r="P90" s="68"/>
       <c r="Q90" s="68">
         <f>Q89/20</f>
-        <v>48.498315000000005</v>
+        <v>48.471315000000004</v>
       </c>
       <c r="R90" s="45"/>
     </row>

</xml_diff>

<commit_message>
Design Files and Deliverables copied from Evaluation Branch.
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/eSpark BOM_Top (20 Boards).xlsx
+++ b/Deliverables/SM_Top Board/_BOM/eSpark BOM_Top (20 Boards).xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B3974B-7077-4EFB-AACA-BB30D08EB492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11490" windowHeight="7590"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="474">
   <si>
     <t>Component list</t>
   </si>
@@ -1574,11 +1575,23 @@
   <si>
     <t>Bivar Inc.</t>
   </si>
+  <si>
+    <t>Heat Sink</t>
+  </si>
+  <si>
+    <t>C4651</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XSD </t>
+  </si>
+  <si>
+    <t>18*6*14 Heat Sinks ROHS</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -2452,7 +2465,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2748,9 +2761,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:R90"/>
+  <dimension ref="A1:R91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -4985,6 +4998,7 @@
     <row r="46" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="53">
+        <f t="shared" ref="B46:B89" si="35">ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
       <c r="C46" s="106" t="s">
@@ -5041,7 +5055,7 @@
     <row r="47" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="53">
-        <f t="shared" ref="B47" si="35">ROW(B47) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>38</v>
       </c>
       <c r="C47" s="102" t="s">
@@ -5096,7 +5110,8 @@
     <row r="48" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="53">
-        <v>38</v>
+        <f t="shared" si="35"/>
+        <v>39</v>
       </c>
       <c r="C48" s="97" t="s">
         <v>283</v>
@@ -5145,7 +5160,7 @@
     <row r="49" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="53">
-        <f t="shared" ref="B49" si="39">ROW(B49) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>40</v>
       </c>
       <c r="C49" s="102" t="s">
@@ -5192,7 +5207,7 @@
         <v>0.13</v>
       </c>
       <c r="Q49" s="96">
-        <f t="shared" ref="Q49" si="40">N49*P49</f>
+        <f t="shared" ref="Q49" si="39">N49*P49</f>
         <v>11.700000000000001</v>
       </c>
       <c r="R49" s="96"/>
@@ -5200,7 +5215,8 @@
     <row r="50" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="53">
-        <v>39</v>
+        <f t="shared" si="35"/>
+        <v>41</v>
       </c>
       <c r="C50" s="106" t="s">
         <v>323</v>
@@ -5246,7 +5262,7 @@
         <v>0.21740000000000001</v>
       </c>
       <c r="Q50" s="109">
-        <f t="shared" ref="Q50" si="41">P50*N50</f>
+        <f t="shared" ref="Q50" si="40">P50*N50</f>
         <v>18.478999999999999</v>
       </c>
       <c r="R50" s="109"/>
@@ -5254,7 +5270,7 @@
     <row r="51" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="53">
-        <f t="shared" ref="B51" si="42">ROW(B51) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>42</v>
       </c>
       <c r="C51" s="102" t="s">
@@ -5301,7 +5317,7 @@
         <v>1E-3</v>
       </c>
       <c r="Q51" s="96">
-        <f t="shared" ref="Q51" si="43">N51*P51</f>
+        <f t="shared" ref="Q51" si="41">N51*P51</f>
         <v>0.1</v>
       </c>
       <c r="R51" s="96"/>
@@ -5309,7 +5325,8 @@
     <row r="52" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="53">
-        <v>40</v>
+        <f t="shared" si="35"/>
+        <v>43</v>
       </c>
       <c r="C52" s="106" t="s">
         <v>324</v>
@@ -5355,7 +5372,7 @@
         <v>1.4E-3</v>
       </c>
       <c r="Q52" s="109">
-        <f t="shared" ref="Q52" si="44">P52*N52</f>
+        <f t="shared" ref="Q52" si="42">P52*N52</f>
         <v>0.13999999999999999</v>
       </c>
       <c r="R52" s="109"/>
@@ -5363,7 +5380,7 @@
     <row r="53" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="53">
-        <f t="shared" ref="B53" si="45">ROW(B53) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>44</v>
       </c>
       <c r="C53" s="102" t="s">
@@ -5410,7 +5427,7 @@
         <v>1.6000000000000001E-3</v>
       </c>
       <c r="Q53" s="96">
-        <f t="shared" ref="Q53" si="46">N53*P53</f>
+        <f t="shared" ref="Q53" si="43">N53*P53</f>
         <v>0.16</v>
       </c>
       <c r="R53" s="96"/>
@@ -5418,7 +5435,8 @@
     <row r="54" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="53">
-        <v>41</v>
+        <f t="shared" si="35"/>
+        <v>45</v>
       </c>
       <c r="C54" s="106" t="s">
         <v>324</v>
@@ -5464,7 +5482,7 @@
         <v>1.4E-3</v>
       </c>
       <c r="Q54" s="109">
-        <f t="shared" ref="Q54" si="47">P54*N54</f>
+        <f t="shared" ref="Q54" si="44">P54*N54</f>
         <v>0.13999999999999999</v>
       </c>
       <c r="R54" s="109"/>
@@ -5472,7 +5490,7 @@
     <row r="55" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="53">
-        <f t="shared" ref="B55" si="48">ROW(B55) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>46</v>
       </c>
       <c r="C55" s="102" t="s">
@@ -5519,7 +5537,7 @@
         <v>1.2999999999999999E-3</v>
       </c>
       <c r="Q55" s="96">
-        <f t="shared" ref="Q55" si="49">N55*P55</f>
+        <f t="shared" ref="Q55" si="45">N55*P55</f>
         <v>0.13</v>
       </c>
       <c r="R55" s="96"/>
@@ -5527,7 +5545,8 @@
     <row r="56" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="53">
-        <v>42</v>
+        <f t="shared" si="35"/>
+        <v>47</v>
       </c>
       <c r="C56" s="106" t="s">
         <v>324</v>
@@ -5573,7 +5592,7 @@
         <v>6.4500000000000002E-2</v>
       </c>
       <c r="Q56" s="109">
-        <f t="shared" ref="Q56" si="50">P56*N56</f>
+        <f t="shared" ref="Q56" si="46">P56*N56</f>
         <v>5.8049999999999997</v>
       </c>
       <c r="R56" s="109"/>
@@ -5581,7 +5600,7 @@
     <row r="57" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="53">
-        <f t="shared" ref="B57" si="51">ROW(B57) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>48</v>
       </c>
       <c r="C57" s="60" t="s">
@@ -5628,7 +5647,7 @@
         <v>1.1000000000000001E-3</v>
       </c>
       <c r="Q57" s="37">
-        <f t="shared" ref="Q57" si="52">N57*P57</f>
+        <f t="shared" ref="Q57" si="47">N57*P57</f>
         <v>0.11</v>
       </c>
       <c r="R57" s="76"/>
@@ -5636,7 +5655,8 @@
     <row r="58" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="53">
-        <v>43</v>
+        <f t="shared" si="35"/>
+        <v>49</v>
       </c>
       <c r="C58" s="106" t="s">
         <v>324</v>
@@ -5682,7 +5702,7 @@
         <v>1.8589999999999999E-2</v>
       </c>
       <c r="Q58" s="109">
-        <f t="shared" ref="Q58" si="53">P58*N58</f>
+        <f t="shared" ref="Q58" si="48">P58*N58</f>
         <v>0.55769999999999997</v>
       </c>
       <c r="R58" s="109"/>
@@ -5690,7 +5710,7 @@
     <row r="59" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="53">
-        <f t="shared" ref="B59" si="54">ROW(B59) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>50</v>
       </c>
       <c r="C59" s="102" t="s">
@@ -5737,7 +5757,7 @@
         <v>1.4E-3</v>
       </c>
       <c r="Q59" s="96">
-        <f t="shared" ref="Q59" si="55">N59*P59</f>
+        <f t="shared" ref="Q59" si="49">N59*P59</f>
         <v>0.13999999999999999</v>
       </c>
       <c r="R59" s="96"/>
@@ -5745,7 +5765,8 @@
     <row r="60" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="53">
-        <v>44</v>
+        <f t="shared" si="35"/>
+        <v>51</v>
       </c>
       <c r="C60" s="106" t="s">
         <v>324</v>
@@ -5791,7 +5812,7 @@
         <v>4.6699999999999997E-3</v>
       </c>
       <c r="Q60" s="109">
-        <f t="shared" ref="Q60" si="56">P60*N60</f>
+        <f t="shared" ref="Q60" si="50">P60*N60</f>
         <v>0.23349999999999999</v>
       </c>
       <c r="R60" s="109"/>
@@ -5799,7 +5820,7 @@
     <row r="61" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="53">
-        <f t="shared" ref="B61" si="57">ROW(B61) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>52</v>
       </c>
       <c r="C61" s="102" t="s">
@@ -5846,7 +5867,7 @@
         <v>1.1999999999999999E-3</v>
       </c>
       <c r="Q61" s="96">
-        <f t="shared" ref="Q61" si="58">N61*P61</f>
+        <f t="shared" ref="Q61" si="51">N61*P61</f>
         <v>0.12</v>
       </c>
       <c r="R61" s="96"/>
@@ -5854,7 +5875,8 @@
     <row r="62" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="53">
-        <v>45</v>
+        <f t="shared" si="35"/>
+        <v>53</v>
       </c>
       <c r="C62" s="106" t="s">
         <v>324</v>
@@ -5900,7 +5922,7 @@
         <v>1.11E-2</v>
       </c>
       <c r="Q62" s="109">
-        <f t="shared" ref="Q62" si="59">P62*N62</f>
+        <f t="shared" ref="Q62" si="52">P62*N62</f>
         <v>0.55500000000000005</v>
       </c>
       <c r="R62" s="109"/>
@@ -5908,7 +5930,7 @@
     <row r="63" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="53">
-        <f t="shared" ref="B63" si="60">ROW(B63) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>54</v>
       </c>
       <c r="C63" s="102" t="s">
@@ -5955,7 +5977,7 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="Q63" s="96">
-        <f t="shared" ref="Q63" si="61">N63*P63</f>
+        <f t="shared" ref="Q63" si="53">N63*P63</f>
         <v>0.21</v>
       </c>
       <c r="R63" s="96"/>
@@ -5963,7 +5985,8 @@
     <row r="64" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="53">
-        <v>46</v>
+        <f t="shared" si="35"/>
+        <v>55</v>
       </c>
       <c r="C64" s="106" t="s">
         <v>324</v>
@@ -6009,7 +6032,7 @@
         <v>1.6000000000000001E-3</v>
       </c>
       <c r="Q64" s="109">
-        <f t="shared" ref="Q64" si="62">P64*N64</f>
+        <f t="shared" ref="Q64" si="54">P64*N64</f>
         <v>0.16</v>
       </c>
       <c r="R64" s="109"/>
@@ -6017,7 +6040,7 @@
     <row r="65" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="53">
-        <f t="shared" ref="B65" si="63">ROW(B65) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>56</v>
       </c>
       <c r="C65" s="102" t="s">
@@ -6064,7 +6087,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
       <c r="Q65" s="96">
-        <f t="shared" ref="Q65" si="64">N65*P65</f>
+        <f t="shared" ref="Q65" si="55">N65*P65</f>
         <v>0.34499999999999997</v>
       </c>
       <c r="R65" s="96"/>
@@ -6072,7 +6095,8 @@
     <row r="66" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="53">
-        <v>47</v>
+        <f t="shared" si="35"/>
+        <v>57</v>
       </c>
       <c r="C66" s="106" t="s">
         <v>324</v>
@@ -6118,7 +6142,7 @@
         <v>1.1000000000000001E-3</v>
       </c>
       <c r="Q66" s="109">
-        <f t="shared" ref="Q66" si="65">P66*N66</f>
+        <f t="shared" ref="Q66" si="56">P66*N66</f>
         <v>0.11</v>
       </c>
       <c r="R66" s="109"/>
@@ -6126,7 +6150,7 @@
     <row r="67" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="53">
-        <f t="shared" ref="B67" si="66">ROW(B67) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>58</v>
       </c>
       <c r="C67" s="60" t="s">
@@ -6173,7 +6197,7 @@
         <v>1.5E-3</v>
       </c>
       <c r="Q67" s="41">
-        <f t="shared" ref="Q67" si="67">P67*N67</f>
+        <f t="shared" ref="Q67" si="57">P67*N67</f>
         <v>0.15</v>
       </c>
       <c r="R67" s="41"/>
@@ -6181,7 +6205,8 @@
     <row r="68" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="53">
-        <v>48</v>
+        <f t="shared" si="35"/>
+        <v>59</v>
       </c>
       <c r="C68" s="59" t="s">
         <v>324</v>
@@ -6233,7 +6258,7 @@
     <row r="69" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="53">
-        <f t="shared" ref="B69" si="68">ROW(B69) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>60</v>
       </c>
       <c r="C69" s="60" t="s">
@@ -6280,7 +6305,7 @@
         <v>1.5E-3</v>
       </c>
       <c r="Q69" s="41">
-        <f t="shared" ref="Q69" si="69">P69*N69</f>
+        <f t="shared" ref="Q69" si="58">P69*N69</f>
         <v>0.15</v>
       </c>
       <c r="R69" s="41"/>
@@ -6288,7 +6313,8 @@
     <row r="70" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="53">
-        <v>49</v>
+        <f t="shared" si="35"/>
+        <v>61</v>
       </c>
       <c r="C70" s="59" t="s">
         <v>324</v>
@@ -6334,7 +6360,7 @@
         <v>8.5400000000000004E-2</v>
       </c>
       <c r="Q70" s="42">
-        <f t="shared" ref="Q70" si="70">N70*P70</f>
+        <f t="shared" ref="Q70" si="59">N70*P70</f>
         <v>2.1350000000000002</v>
       </c>
       <c r="R70" s="42"/>
@@ -6342,7 +6368,7 @@
     <row r="71" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="53">
-        <f t="shared" ref="B71" si="71">ROW(B71) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>62</v>
       </c>
       <c r="C71" s="60" t="s">
@@ -6376,7 +6402,7 @@
         <v>1</v>
       </c>
       <c r="M71" s="41">
-        <f t="shared" ref="M71:M88" si="72">L71*20</f>
+        <f t="shared" ref="M71:M89" si="60">L71*20</f>
         <v>20</v>
       </c>
       <c r="N71" s="41">
@@ -6389,7 +6415,7 @@
         <v>3.8E-3</v>
       </c>
       <c r="Q71" s="41">
-        <f t="shared" ref="Q71" si="73">P71*N71</f>
+        <f t="shared" ref="Q71" si="61">P71*N71</f>
         <v>0.19</v>
       </c>
       <c r="R71" s="76"/>
@@ -6397,7 +6423,8 @@
     <row r="72" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="53">
-        <v>50</v>
+        <f t="shared" si="35"/>
+        <v>63</v>
       </c>
       <c r="C72" s="59" t="s">
         <v>324</v>
@@ -6443,7 +6470,7 @@
         <v>1.1999999999999999E-3</v>
       </c>
       <c r="Q72" s="42">
-        <f t="shared" ref="Q72" si="74">N72*P72</f>
+        <f t="shared" ref="Q72" si="62">N72*P72</f>
         <v>0.24</v>
       </c>
       <c r="R72" s="77"/>
@@ -6451,7 +6478,7 @@
     <row r="73" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="53">
-        <f t="shared" ref="B73" si="75">ROW(B73) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>64</v>
       </c>
       <c r="C73" s="60" t="s">
@@ -6485,7 +6512,7 @@
         <v>1</v>
       </c>
       <c r="M73" s="41">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N73" s="41">
@@ -6498,7 +6525,7 @@
         <v>1E-3</v>
       </c>
       <c r="Q73" s="41">
-        <f t="shared" ref="Q73" si="76">P73*N73</f>
+        <f t="shared" ref="Q73" si="63">P73*N73</f>
         <v>0.1</v>
       </c>
       <c r="R73" s="41"/>
@@ -6506,7 +6533,8 @@
     <row r="74" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="53">
-        <v>51</v>
+        <f t="shared" si="35"/>
+        <v>65</v>
       </c>
       <c r="C74" s="59" t="s">
         <v>324</v>
@@ -6539,7 +6567,7 @@
         <v>1</v>
       </c>
       <c r="M74" s="42">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N74" s="42">
@@ -6552,7 +6580,7 @@
         <v>4.3E-3</v>
       </c>
       <c r="Q74" s="42">
-        <f t="shared" ref="Q74" si="77">N74*P74</f>
+        <f t="shared" ref="Q74" si="64">N74*P74</f>
         <v>0.215</v>
       </c>
       <c r="R74" s="42"/>
@@ -6560,7 +6588,7 @@
     <row r="75" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="53">
-        <f t="shared" ref="B75" si="78">ROW(B75) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>66</v>
       </c>
       <c r="C75" s="97" t="s">
@@ -6594,7 +6622,7 @@
         <v>4</v>
       </c>
       <c r="M75" s="66">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>80</v>
       </c>
       <c r="N75" s="66">
@@ -6607,7 +6635,7 @@
         <v>1.1999999999999999E-3</v>
       </c>
       <c r="Q75" s="66">
-        <f t="shared" ref="Q75" si="79">P75*N75</f>
+        <f t="shared" ref="Q75" si="65">P75*N75</f>
         <v>0.12</v>
       </c>
       <c r="R75" s="66" t="s">
@@ -6617,7 +6645,8 @@
     <row r="76" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="53">
-        <v>52</v>
+        <f t="shared" si="35"/>
+        <v>67</v>
       </c>
       <c r="C76" s="97" t="s">
         <v>169</v>
@@ -6650,17 +6679,17 @@
         <v>15</v>
       </c>
       <c r="M76" s="66">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>300</v>
       </c>
       <c r="N76" s="66">
-        <f t="shared" ref="N76:N77" si="80">M76+(M76*0.1)</f>
+        <f t="shared" ref="N76:N77" si="66">M76+(M76*0.1)</f>
         <v>330</v>
       </c>
       <c r="O76" s="66"/>
       <c r="P76" s="66"/>
       <c r="Q76" s="66">
-        <f t="shared" ref="Q76" si="81">P76*N76</f>
+        <f t="shared" ref="Q76" si="67">P76*N76</f>
         <v>0</v>
       </c>
       <c r="R76" s="66" t="s">
@@ -6670,7 +6699,7 @@
     <row r="77" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="53">
-        <f t="shared" ref="B77" si="82">ROW(B77) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>68</v>
       </c>
       <c r="C77" s="102" t="s">
@@ -6704,17 +6733,17 @@
         <v>1</v>
       </c>
       <c r="M77" s="96">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N77" s="96">
-        <f t="shared" si="80"/>
+        <f t="shared" si="66"/>
         <v>22</v>
       </c>
       <c r="O77" s="96"/>
       <c r="P77" s="96"/>
       <c r="Q77" s="96">
-        <f t="shared" ref="Q77" si="83">N77*P77</f>
+        <f t="shared" ref="Q77" si="68">N77*P77</f>
         <v>0</v>
       </c>
       <c r="R77" s="96"/>
@@ -6722,7 +6751,8 @@
     <row r="78" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="53">
-        <v>53</v>
+        <f t="shared" si="35"/>
+        <v>69</v>
       </c>
       <c r="C78" s="106" t="s">
         <v>327</v>
@@ -6755,7 +6785,7 @@
         <v>1</v>
       </c>
       <c r="M78" s="109">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N78" s="109">
@@ -6768,7 +6798,7 @@
         <v>3.81</v>
       </c>
       <c r="Q78" s="109">
-        <f t="shared" ref="Q78" si="84">P78*N78</f>
+        <f t="shared" ref="Q78" si="69">P78*N78</f>
         <v>80.010000000000005</v>
       </c>
       <c r="R78" s="109"/>
@@ -6776,7 +6806,7 @@
     <row r="79" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="53">
-        <f t="shared" ref="B79" si="85">ROW(B79) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>70</v>
       </c>
       <c r="C79" s="102" t="s">
@@ -6810,7 +6840,7 @@
         <v>1</v>
       </c>
       <c r="M79" s="96">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N79" s="96">
@@ -6823,7 +6853,7 @@
         <v>2.48</v>
       </c>
       <c r="Q79" s="96">
-        <f t="shared" ref="Q79" si="86">N79*P79</f>
+        <f t="shared" ref="Q79" si="70">N79*P79</f>
         <v>52.08</v>
       </c>
       <c r="R79" s="96"/>
@@ -6831,7 +6861,8 @@
     <row r="80" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="53">
-        <v>54</v>
+        <f t="shared" si="35"/>
+        <v>71</v>
       </c>
       <c r="C80" s="106" t="s">
         <v>328</v>
@@ -6864,7 +6895,7 @@
         <v>1</v>
       </c>
       <c r="M80" s="109">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N80" s="109">
@@ -6877,7 +6908,7 @@
         <v>1.3939999999999999</v>
       </c>
       <c r="Q80" s="109">
-        <f t="shared" ref="Q80" si="87">P80*N80</f>
+        <f t="shared" ref="Q80" si="71">P80*N80</f>
         <v>29.273999999999997</v>
       </c>
       <c r="R80" s="79"/>
@@ -6885,7 +6916,7 @@
     <row r="81" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="53">
-        <f t="shared" ref="B81" si="88">ROW(B81) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>72</v>
       </c>
       <c r="C81" s="102" t="s">
@@ -6919,7 +6950,7 @@
         <v>1</v>
       </c>
       <c r="M81" s="96">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N81" s="96">
@@ -6932,7 +6963,7 @@
         <v>0.69430000000000003</v>
       </c>
       <c r="Q81" s="96">
-        <f t="shared" ref="Q81" si="89">N81*P81</f>
+        <f t="shared" ref="Q81" si="72">N81*P81</f>
         <v>14.580300000000001</v>
       </c>
       <c r="R81" s="78"/>
@@ -6940,7 +6971,8 @@
     <row r="82" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="53">
-        <v>55</v>
+        <f t="shared" si="35"/>
+        <v>73</v>
       </c>
       <c r="C82" s="106" t="s">
         <v>328</v>
@@ -6973,7 +7005,7 @@
         <v>1</v>
       </c>
       <c r="M82" s="109">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N82" s="109">
@@ -6986,7 +7018,7 @@
         <v>3.637</v>
       </c>
       <c r="Q82" s="109">
-        <f t="shared" ref="Q82" si="90">P82*N82</f>
+        <f t="shared" ref="Q82" si="73">P82*N82</f>
         <v>76.376999999999995</v>
       </c>
       <c r="R82" s="109"/>
@@ -6994,7 +7026,7 @@
     <row r="83" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
       <c r="B83" s="53">
-        <f t="shared" ref="B83" si="91">ROW(B83) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>74</v>
       </c>
       <c r="C83" s="102" t="s">
@@ -7028,7 +7060,7 @@
         <v>1</v>
       </c>
       <c r="M83" s="96">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N83" s="96">
@@ -7041,7 +7073,7 @@
         <v>0.43280000000000002</v>
       </c>
       <c r="Q83" s="96">
-        <f t="shared" ref="Q83" si="92">N83*P83</f>
+        <f t="shared" ref="Q83" si="74">N83*P83</f>
         <v>9.0888000000000009</v>
       </c>
       <c r="R83" s="96"/>
@@ -7049,7 +7081,8 @@
     <row r="84" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
       <c r="B84" s="53">
-        <v>56</v>
+        <f t="shared" si="35"/>
+        <v>75</v>
       </c>
       <c r="C84" s="71" t="s">
         <v>328</v>
@@ -7082,7 +7115,7 @@
         <v>1</v>
       </c>
       <c r="M84" s="74">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N84" s="74">
@@ -7095,7 +7128,7 @@
         <v>7.4638</v>
       </c>
       <c r="Q84" s="74">
-        <f t="shared" ref="Q84" si="93">P84*N84</f>
+        <f t="shared" ref="Q84" si="75">P84*N84</f>
         <v>156.7398</v>
       </c>
       <c r="R84" s="74" t="s">
@@ -7105,7 +7138,7 @@
     <row r="85" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
       <c r="B85" s="53">
-        <f t="shared" ref="B85" si="94">ROW(B85) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>76</v>
       </c>
       <c r="C85" s="102" t="s">
@@ -7139,7 +7172,7 @@
         <v>1</v>
       </c>
       <c r="M85" s="96">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N85" s="96">
@@ -7152,7 +7185,7 @@
         <v>2.6459999999999999</v>
       </c>
       <c r="Q85" s="96">
-        <f t="shared" ref="Q85" si="95">N85*P85</f>
+        <f t="shared" ref="Q85" si="76">N85*P85</f>
         <v>55.565999999999995</v>
       </c>
       <c r="R85" s="96"/>
@@ -7160,7 +7193,8 @@
     <row r="86" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
       <c r="B86" s="53">
-        <v>57</v>
+        <f t="shared" si="35"/>
+        <v>77</v>
       </c>
       <c r="C86" s="106" t="s">
         <v>328</v>
@@ -7193,7 +7227,7 @@
         <v>2</v>
       </c>
       <c r="M86" s="109">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>40</v>
       </c>
       <c r="N86" s="109">
@@ -7206,7 +7240,7 @@
         <v>2.2974000000000001</v>
       </c>
       <c r="Q86" s="109">
-        <f t="shared" ref="Q86" si="96">P86*N86</f>
+        <f t="shared" ref="Q86" si="77">P86*N86</f>
         <v>96.490800000000007</v>
       </c>
       <c r="R86" s="79"/>
@@ -7214,7 +7248,7 @@
     <row r="87" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
       <c r="B87" s="53">
-        <f t="shared" ref="B87" si="97">ROW(B87) - ROW($B$9)</f>
+        <f t="shared" si="35"/>
         <v>78</v>
       </c>
       <c r="C87" s="60" t="s">
@@ -7261,7 +7295,7 @@
         <v>0.39140000000000003</v>
       </c>
       <c r="Q87" s="41">
-        <f t="shared" ref="Q87" si="98">P87*N87</f>
+        <f t="shared" ref="Q87" si="78">P87*N87</f>
         <v>8.2194000000000003</v>
       </c>
       <c r="R87" s="41"/>
@@ -7269,7 +7303,8 @@
     <row r="88" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
       <c r="B88" s="53">
-        <v>58</v>
+        <f t="shared" si="35"/>
+        <v>79</v>
       </c>
       <c r="C88" s="59" t="s">
         <v>328</v>
@@ -7302,7 +7337,7 @@
         <v>1</v>
       </c>
       <c r="M88" s="42">
-        <f t="shared" si="72"/>
+        <f t="shared" si="60"/>
         <v>20</v>
       </c>
       <c r="N88" s="42">
@@ -7315,64 +7350,117 @@
         <v>3.532</v>
       </c>
       <c r="Q88" s="42">
-        <f t="shared" ref="Q88" si="99">N88*P88</f>
+        <f t="shared" ref="Q88:Q89" si="79">N88*P88</f>
         <v>74.171999999999997</v>
       </c>
       <c r="R88" s="79"/>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
-      <c r="B89" s="32"/>
-      <c r="C89" s="51"/>
-      <c r="D89" s="33" t="s">
+      <c r="B89" s="53">
+        <f t="shared" si="35"/>
+        <v>80</v>
+      </c>
+      <c r="C89" s="59" t="s">
+        <v>470</v>
+      </c>
+      <c r="D89" s="39" t="s">
+        <v>314</v>
+      </c>
+      <c r="E89" s="40" t="s">
+        <v>473</v>
+      </c>
+      <c r="F89" s="39" t="s">
+        <v>308</v>
+      </c>
+      <c r="G89" s="40" t="s">
+        <v>471</v>
+      </c>
+      <c r="H89" s="39" t="s">
+        <v>472</v>
+      </c>
+      <c r="I89" s="39" t="s">
+        <v>314</v>
+      </c>
+      <c r="J89" s="39" t="s">
+        <v>471</v>
+      </c>
+      <c r="K89" s="40"/>
+      <c r="L89" s="39">
+        <v>1</v>
+      </c>
+      <c r="M89" s="42">
+        <f t="shared" si="60"/>
+        <v>20</v>
+      </c>
+      <c r="N89" s="42">
+        <v>25</v>
+      </c>
+      <c r="O89" s="64" t="s">
+        <v>343</v>
+      </c>
+      <c r="P89" s="42">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="Q89" s="42">
+        <f t="shared" si="79"/>
+        <v>2.2250000000000001</v>
+      </c>
+      <c r="R89" s="79"/>
+    </row>
+    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A90" s="1"/>
+      <c r="B90" s="32"/>
+      <c r="C90" s="51"/>
+      <c r="D90" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="E89" s="34"/>
-      <c r="F89" s="35"/>
-      <c r="G89" s="36"/>
-      <c r="H89" s="35"/>
-      <c r="I89" s="35"/>
-      <c r="J89" s="35"/>
-      <c r="K89" s="36"/>
-      <c r="L89" s="36"/>
-      <c r="M89" s="36"/>
-      <c r="N89" s="36"/>
-      <c r="O89" s="69" t="s">
+      <c r="E90" s="34"/>
+      <c r="F90" s="35"/>
+      <c r="G90" s="36"/>
+      <c r="H90" s="35"/>
+      <c r="I90" s="35"/>
+      <c r="J90" s="35"/>
+      <c r="K90" s="36"/>
+      <c r="L90" s="36"/>
+      <c r="M90" s="36"/>
+      <c r="N90" s="36"/>
+      <c r="O90" s="69" t="s">
         <v>421</v>
       </c>
-      <c r="P89" s="67"/>
-      <c r="Q89" s="67">
+      <c r="P90" s="67"/>
+      <c r="Q90" s="67">
         <f>SUM(Q10:Q88)</f>
         <v>969.42630000000008</v>
       </c>
-      <c r="R89" s="44"/>
-    </row>
-    <row r="90" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="1"/>
-      <c r="B90" s="24"/>
-      <c r="C90" s="52"/>
-      <c r="D90" s="8" t="s">
+      <c r="R90" s="44"/>
+    </row>
+    <row r="91" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="1"/>
+      <c r="B91" s="24"/>
+      <c r="C91" s="52"/>
+      <c r="D91" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E90" s="9"/>
-      <c r="F90" s="9"/>
-      <c r="G90" s="9"/>
-      <c r="H90" s="9"/>
-      <c r="I90" s="9"/>
-      <c r="J90" s="9"/>
-      <c r="K90" s="9"/>
-      <c r="L90" s="9"/>
-      <c r="M90" s="9"/>
-      <c r="N90" s="9"/>
-      <c r="O90" s="70" t="s">
+      <c r="E91" s="9"/>
+      <c r="F91" s="9"/>
+      <c r="G91" s="9"/>
+      <c r="H91" s="9"/>
+      <c r="I91" s="9"/>
+      <c r="J91" s="9"/>
+      <c r="K91" s="9"/>
+      <c r="L91" s="9"/>
+      <c r="M91" s="9"/>
+      <c r="N91" s="9"/>
+      <c r="O91" s="70" t="s">
         <v>422</v>
       </c>
-      <c r="P90" s="68"/>
-      <c r="Q90" s="68">
-        <f>Q89/20</f>
+      <c r="P91" s="68"/>
+      <c r="Q91" s="68">
+        <f>Q90/20</f>
         <v>48.471315000000004</v>
       </c>
-      <c r="R90" s="45"/>
+      <c r="R91" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7380,84 +7468,85 @@
     <mergeCell ref="R3:R8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O10" r:id="rId1"/>
-    <hyperlink ref="O11" r:id="rId2"/>
-    <hyperlink ref="O12" r:id="rId3"/>
-    <hyperlink ref="O13" r:id="rId4"/>
-    <hyperlink ref="O14" r:id="rId5"/>
-    <hyperlink ref="O15" r:id="rId6"/>
-    <hyperlink ref="O16" r:id="rId7"/>
-    <hyperlink ref="O17" r:id="rId8"/>
-    <hyperlink ref="O18" r:id="rId9"/>
-    <hyperlink ref="O19" r:id="rId10"/>
-    <hyperlink ref="O20" r:id="rId11"/>
-    <hyperlink ref="O21" r:id="rId12"/>
-    <hyperlink ref="O22" r:id="rId13"/>
-    <hyperlink ref="O23" r:id="rId14"/>
-    <hyperlink ref="O24" r:id="rId15"/>
-    <hyperlink ref="O25" r:id="rId16"/>
-    <hyperlink ref="O26" r:id="rId17"/>
-    <hyperlink ref="O27" r:id="rId18"/>
-    <hyperlink ref="O28" r:id="rId19"/>
-    <hyperlink ref="O29" r:id="rId20"/>
-    <hyperlink ref="O30" r:id="rId21"/>
-    <hyperlink ref="O31" r:id="rId22"/>
-    <hyperlink ref="O32" r:id="rId23"/>
-    <hyperlink ref="O33" r:id="rId24"/>
-    <hyperlink ref="O34" r:id="rId25"/>
-    <hyperlink ref="O35" r:id="rId26"/>
-    <hyperlink ref="O36" r:id="rId27"/>
-    <hyperlink ref="O37" r:id="rId28"/>
-    <hyperlink ref="O38" r:id="rId29"/>
-    <hyperlink ref="O39" r:id="rId30"/>
-    <hyperlink ref="O40" r:id="rId31"/>
-    <hyperlink ref="O41" r:id="rId32"/>
-    <hyperlink ref="O42" r:id="rId33"/>
-    <hyperlink ref="O43" r:id="rId34"/>
-    <hyperlink ref="O44" r:id="rId35"/>
-    <hyperlink ref="O45" r:id="rId36"/>
-    <hyperlink ref="O47" r:id="rId37"/>
-    <hyperlink ref="O49" r:id="rId38"/>
-    <hyperlink ref="O50" r:id="rId39"/>
-    <hyperlink ref="O51" r:id="rId40"/>
-    <hyperlink ref="O52" r:id="rId41"/>
-    <hyperlink ref="O53" r:id="rId42"/>
-    <hyperlink ref="O54" r:id="rId43"/>
-    <hyperlink ref="O55" r:id="rId44"/>
-    <hyperlink ref="O56" r:id="rId45"/>
-    <hyperlink ref="O68" r:id="rId46"/>
-    <hyperlink ref="O58" r:id="rId47"/>
-    <hyperlink ref="O59" r:id="rId48"/>
-    <hyperlink ref="O60" r:id="rId49"/>
-    <hyperlink ref="O61" r:id="rId50"/>
-    <hyperlink ref="O62" r:id="rId51"/>
-    <hyperlink ref="O63" r:id="rId52"/>
-    <hyperlink ref="O64" r:id="rId53"/>
-    <hyperlink ref="O65" r:id="rId54"/>
-    <hyperlink ref="O66" r:id="rId55"/>
-    <hyperlink ref="O67" r:id="rId56"/>
-    <hyperlink ref="O69" r:id="rId57"/>
-    <hyperlink ref="O70" r:id="rId58"/>
-    <hyperlink ref="O71" r:id="rId59"/>
-    <hyperlink ref="O74" r:id="rId60"/>
-    <hyperlink ref="O75" r:id="rId61"/>
-    <hyperlink ref="O72" r:id="rId62"/>
-    <hyperlink ref="O78" r:id="rId63"/>
-    <hyperlink ref="O79" r:id="rId64"/>
-    <hyperlink ref="O80" r:id="rId65"/>
-    <hyperlink ref="O81" r:id="rId66"/>
-    <hyperlink ref="O82" r:id="rId67"/>
-    <hyperlink ref="O83" r:id="rId68"/>
-    <hyperlink ref="O84" r:id="rId69"/>
-    <hyperlink ref="O85" r:id="rId70"/>
-    <hyperlink ref="O86" r:id="rId71"/>
-    <hyperlink ref="O88" r:id="rId72"/>
-    <hyperlink ref="O87" r:id="rId73"/>
-    <hyperlink ref="O57" r:id="rId74"/>
-    <hyperlink ref="O46" r:id="rId75"/>
+    <hyperlink ref="O10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="O11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="O12" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="O13" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="O14" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="O15" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="O16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="O17" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="O18" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="O19" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="O20" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="O21" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="O22" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="O23" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="O24" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="O25" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="O26" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="O27" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="O28" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="O29" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="O30" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="O31" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="O32" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="O33" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="O34" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="O35" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="O36" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="O37" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="O38" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="O39" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="O40" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="O41" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="O42" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="O43" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="O44" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="O45" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="O47" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="O49" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="O50" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="O51" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="O52" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="O53" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="O54" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="O55" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="O56" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="O68" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="O58" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="O59" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="O60" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="O61" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="O62" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="O63" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="O64" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="O65" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="O66" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="O67" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="O69" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="O70" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="O71" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="O74" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="O75" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="O72" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="O78" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="O79" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="O80" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="O81" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="O82" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="O83" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="O84" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="O85" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="O86" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="O88" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="O87" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="O57" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="O46" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="O89" r:id="rId76" xr:uid="{94AF4969-113D-4C22-911F-093FC1147D5D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId76"/>
-  <drawing r:id="rId77"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId77"/>
+  <drawing r:id="rId78"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#160 2.2nf Cap and 50mR resistor added in BOM
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/eSpark BOM_Top (20 Boards).xlsx
+++ b/Deliverables/SM_Top Board/_BOM/eSpark BOM_Top (20 Boards).xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD49FCC0-8CB8-4350-BC87-798A3C4365C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -33,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="482">
   <si>
     <t>Component list</t>
   </si>
@@ -80,9 +79,6 @@
     <t>C36</t>
   </si>
   <si>
-    <t>C37</t>
-  </si>
-  <si>
     <t>C42</t>
   </si>
   <si>
@@ -158,9 +154,6 @@
     <t>R6, R7, R8, R9</t>
   </si>
   <si>
-    <t>R10, R11, R12, R13</t>
-  </si>
-  <si>
     <t>R21</t>
   </si>
   <si>
@@ -365,9 +358,6 @@
     <t>RES SMD 47OHM 0.1W 0603</t>
   </si>
   <si>
-    <t>0.033Ω ±1% 2W ±1800ppm/°C 2512 Low Resistors &amp; Current Sense Resistors - Surface Mount RoHS</t>
-  </si>
-  <si>
     <t>RES SMD 150OHM 1/10W 0603</t>
   </si>
   <si>
@@ -902,9 +892,6 @@
     <t>47R</t>
   </si>
   <si>
-    <t>33m</t>
-  </si>
-  <si>
     <t>150R</t>
   </si>
   <si>
@@ -1022,9 +1009,6 @@
     <t>IC</t>
   </si>
   <si>
-    <t>CRH2512FR033E04Z</t>
-  </si>
-  <si>
     <t>0603WAF1201T5E</t>
   </si>
   <si>
@@ -1208,12 +1192,6 @@
     <t>C114623</t>
   </si>
   <si>
-    <t>LR2512-22R033F4</t>
-  </si>
-  <si>
-    <t>C2681032</t>
-  </si>
-  <si>
     <t>C114608</t>
   </si>
   <si>
@@ -1353,9 +1331,6 @@
   </si>
   <si>
     <t>RES SMD 22HM 1/10W 0603</t>
-  </si>
-  <si>
-    <t>C5, C6, C14, C23, C24, C29, C34, C35</t>
   </si>
   <si>
     <t>C43</t>
@@ -1617,11 +1592,32 @@
   <si>
     <t>Ali-E</t>
   </si>
+  <si>
+    <t>C23, C24, C37</t>
+  </si>
+  <si>
+    <t>C5, C6, C14, C29, C34, C35</t>
+  </si>
+  <si>
+    <t>R12, R13</t>
+  </si>
+  <si>
+    <t>2W 50mΩ ±1% 2512 Current Sense Resistors/Shunt Resistors ROHS</t>
+  </si>
+  <si>
+    <t>CRH2512FR050E04Z</t>
+  </si>
+  <si>
+    <t>C176035</t>
+  </si>
+  <si>
+    <t>50mR</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -2824,7 +2820,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:U92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2875,7 +2871,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="54" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -2899,7 +2895,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="55" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
@@ -2923,7 +2919,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="56" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
@@ -3026,52 +3022,52 @@
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="I9" s="29" t="s">
+        <v>330</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>331</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>257</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>303</v>
+      </c>
+      <c r="M9" s="31" t="s">
+        <v>332</v>
+      </c>
+      <c r="N9" s="31" t="s">
+        <v>333</v>
+      </c>
+      <c r="O9" s="31" t="s">
+        <v>334</v>
+      </c>
+      <c r="P9" s="31" t="s">
         <v>335</v>
       </c>
-      <c r="J9" s="29" t="s">
+      <c r="Q9" s="31" t="s">
         <v>336</v>
       </c>
-      <c r="K9" s="30" t="s">
-        <v>260</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>307</v>
-      </c>
-      <c r="M9" s="31" t="s">
-        <v>337</v>
-      </c>
-      <c r="N9" s="31" t="s">
-        <v>338</v>
-      </c>
-      <c r="O9" s="31" t="s">
-        <v>339</v>
-      </c>
-      <c r="P9" s="31" t="s">
-        <v>340</v>
-      </c>
-      <c r="Q9" s="31" t="s">
-        <v>341</v>
-      </c>
       <c r="R9" s="31" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3081,31 +3077,31 @@
         <v>1</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D10" s="37" t="s">
         <v>8</v>
       </c>
       <c r="E10" s="38" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G10" s="116" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>477</v>
+        <v>469</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>478</v>
+        <v>470</v>
       </c>
       <c r="K10" s="38" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="L10" s="37">
         <v>1</v>
@@ -3118,7 +3114,7 @@
         <v>22</v>
       </c>
       <c r="O10" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P10" s="41">
         <v>0.38819999999999999</v>
@@ -3136,31 +3132,31 @@
         <v>2</v>
       </c>
       <c r="C11" s="80" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D11" s="81" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="E11" s="82" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F11" s="81" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G11" s="82" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="H11" s="81" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="I11" s="81" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J11" s="81" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="K11" s="82" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="L11" s="81">
         <v>15</v>
@@ -3173,7 +3169,7 @@
         <v>300</v>
       </c>
       <c r="O11" s="84" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P11" s="83">
         <v>1.4E-3</v>
@@ -3183,7 +3179,7 @@
         <v>0.42</v>
       </c>
       <c r="R11" s="83" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3193,31 +3189,31 @@
         <v>3</v>
       </c>
       <c r="C12" s="60" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="K12" s="38" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="L12" s="85">
         <v>2</v>
@@ -3230,7 +3226,7 @@
         <v>100</v>
       </c>
       <c r="O12" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P12" s="41">
         <v>1.2999999999999999E-3</v>
@@ -3248,31 +3244,31 @@
         <v>4</v>
       </c>
       <c r="C13" s="59" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D13" s="39" t="s">
-        <v>428</v>
+        <v>421</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="H13" s="39" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="I13" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J13" s="39" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="K13" s="40" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="L13" s="86">
         <v>1</v>
@@ -3285,7 +3281,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P13" s="42">
         <v>3.5900000000000001E-2</v>
@@ -3303,44 +3299,44 @@
         <v>5</v>
       </c>
       <c r="C14" s="60" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>440</v>
+        <v>476</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="K14" s="38" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L14" s="37">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M14" s="41">
         <f t="shared" si="1"/>
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="N14" s="41">
         <v>200</v>
       </c>
       <c r="O14" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P14" s="41">
         <v>4.0899999999999999E-2</v>
@@ -3358,31 +3354,31 @@
         <v>6</v>
       </c>
       <c r="C15" s="59" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D15" s="39" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="E15" s="40" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F15" s="39" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I15" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J15" s="39" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="K15" s="40" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="L15" s="86">
         <v>3</v>
@@ -3395,7 +3391,7 @@
         <v>100</v>
       </c>
       <c r="O15" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P15" s="42">
         <v>5.8999999999999999E-3</v>
@@ -3413,31 +3409,31 @@
         <v>7</v>
       </c>
       <c r="C16" s="60" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G16" s="100" t="s">
-        <v>431</v>
+        <v>424</v>
       </c>
       <c r="H16" s="85" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>432</v>
+        <v>425</v>
       </c>
       <c r="K16" s="38" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="L16" s="37">
         <v>6</v>
@@ -3450,7 +3446,7 @@
         <v>130</v>
       </c>
       <c r="O16" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P16" s="41">
         <v>3.32E-2</v>
@@ -3468,31 +3464,31 @@
         <v>8</v>
       </c>
       <c r="C17" s="59" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D17" s="39" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="40" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F17" s="39" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G17" s="40" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I17" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J17" s="39" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="K17" s="40" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="L17" s="39">
         <v>1</v>
@@ -3505,7 +3501,7 @@
         <v>50</v>
       </c>
       <c r="O17" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P17" s="42">
         <v>9.9000000000000008E-3</v>
@@ -3523,31 +3519,31 @@
         <v>9</v>
       </c>
       <c r="C18" s="101" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D18" s="102" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="E18" s="103" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F18" s="102" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="G18" s="118" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="H18" s="102" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="I18" s="102" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="J18" s="102" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="K18" s="103" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="L18" s="102">
         <v>8</v>
@@ -3560,7 +3556,7 @@
         <v>180</v>
       </c>
       <c r="O18" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P18" s="95">
         <v>3.09E-2</v>
@@ -3578,31 +3574,31 @@
         <v>10</v>
       </c>
       <c r="C19" s="105" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D19" s="106" t="s">
         <v>10</v>
       </c>
       <c r="E19" s="107" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F19" s="106" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G19" s="119" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H19" s="106" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I19" s="106" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="J19" s="106" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="K19" s="107" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="L19" s="106">
         <v>1</v>
@@ -3615,7 +3611,7 @@
         <v>50</v>
       </c>
       <c r="O19" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P19" s="108">
         <v>5.3E-3</v>
@@ -3633,31 +3629,31 @@
         <v>11</v>
       </c>
       <c r="C20" s="101" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D20" s="102" t="s">
         <v>11</v>
       </c>
       <c r="E20" s="103" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F20" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G20" s="102" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H20" s="102" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="I20" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J20" s="102" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="K20" s="103" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="L20" s="102">
         <v>1</v>
@@ -3670,7 +3666,7 @@
         <v>22</v>
       </c>
       <c r="O20" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P20" s="95">
         <v>0.22189999999999999</v>
@@ -3688,31 +3684,31 @@
         <v>12</v>
       </c>
       <c r="C21" s="105" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D21" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E21" s="107" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F21" s="106" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G21" s="107" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="H21" s="106" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="I21" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J21" s="106" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="K21" s="107" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="L21" s="106">
         <v>2</v>
@@ -3725,7 +3721,7 @@
         <v>50</v>
       </c>
       <c r="O21" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P21" s="108">
         <v>7.7000000000000002E-3</v>
@@ -3743,31 +3739,31 @@
         <v>13</v>
       </c>
       <c r="C22" s="60" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D22" s="37" t="s">
         <v>13</v>
       </c>
       <c r="E22" s="38" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G22" s="38" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="H22" s="37" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="I22" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J22" s="37" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="K22" s="38" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="L22" s="37">
         <v>1</v>
@@ -3780,7 +3776,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P22" s="41">
         <v>3.49E-2</v>
@@ -3798,31 +3794,31 @@
         <v>14</v>
       </c>
       <c r="C23" s="59" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D23" s="39" t="s">
-        <v>427</v>
+        <v>420</v>
       </c>
       <c r="E23" s="40" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F23" s="39" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G23" s="40" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="H23" s="39" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="I23" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J23" s="39" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="K23" s="40" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="L23" s="39">
         <v>1</v>
@@ -3835,7 +3831,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P23" s="42">
         <v>1.9199999999999998E-2</v>
@@ -3853,31 +3849,31 @@
         <v>15</v>
       </c>
       <c r="C24" s="60" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D24" s="37" t="s">
         <v>14</v>
       </c>
       <c r="E24" s="38" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G24" s="120">
         <v>885012205080</v>
       </c>
       <c r="H24" s="37" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="I24" s="37" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="J24" s="37" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="L24" s="37">
         <v>1</v>
@@ -3890,7 +3886,7 @@
         <v>50</v>
       </c>
       <c r="O24" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P24" s="41">
         <v>5.1999999999999998E-3</v>
@@ -3908,44 +3904,44 @@
         <v>16</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D25" s="39" t="s">
-        <v>15</v>
+        <v>475</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F25" s="39" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G25" s="40" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="H25" s="39" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I25" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J25" s="39" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="K25" s="40" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="L25" s="39">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M25" s="42">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="N25" s="42">
         <v>100</v>
       </c>
       <c r="O25" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P25" s="42">
         <v>3.2000000000000002E-3</v>
@@ -3963,31 +3959,31 @@
         <v>17</v>
       </c>
       <c r="C26" s="101" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D26" s="102" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E26" s="110" t="s">
-        <v>429</v>
+        <v>422</v>
       </c>
       <c r="F26" s="102" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G26" s="110" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="H26" s="111" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="I26" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J26" s="102" t="s">
-        <v>430</v>
+        <v>423</v>
       </c>
       <c r="K26" s="110" t="s">
-        <v>442</v>
+        <v>434</v>
       </c>
       <c r="L26" s="102">
         <v>1</v>
@@ -4000,7 +3996,7 @@
         <v>100</v>
       </c>
       <c r="O26" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P26" s="95">
         <v>3.3999999999999998E-3</v>
@@ -4018,31 +4014,31 @@
         <v>18</v>
       </c>
       <c r="C27" s="105" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D27" s="106" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="E27" s="107" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F27" s="106" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G27" s="107" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H27" s="106" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I27" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J27" s="106" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="K27" s="107" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="L27" s="106">
         <v>1</v>
@@ -4055,7 +4051,7 @@
         <v>30</v>
       </c>
       <c r="O27" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P27" s="108">
         <v>0.2525</v>
@@ -4073,31 +4069,31 @@
         <v>19</v>
       </c>
       <c r="C28" s="60" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D28" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E28" s="38" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G28" s="38" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="H28" s="37" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="I28" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J28" s="37" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="K28" s="38" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="L28" s="37">
         <v>1</v>
@@ -4110,7 +4106,7 @@
         <v>22</v>
       </c>
       <c r="O28" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P28" s="41">
         <v>0.89629999999999999</v>
@@ -4128,31 +4124,31 @@
         <v>20</v>
       </c>
       <c r="C29" s="59" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D29" s="39" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G29" s="39" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H29" s="39" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I29" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J29" s="39" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="K29" s="40" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="L29" s="39">
         <v>1</v>
@@ -4165,7 +4161,7 @@
         <v>21</v>
       </c>
       <c r="O29" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P29" s="42">
         <v>0.47249999999999998</v>
@@ -4183,31 +4179,31 @@
         <v>21</v>
       </c>
       <c r="C30" s="60" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F30" s="37" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="H30" s="37" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I30" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J30" s="37" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="K30" s="38" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="L30" s="37">
         <v>1</v>
@@ -4220,7 +4216,7 @@
         <v>100</v>
       </c>
       <c r="O30" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P30" s="41">
         <v>3.0999999999999999E-3</v>
@@ -4238,31 +4234,31 @@
         <v>22</v>
       </c>
       <c r="C31" s="105" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D31" s="106" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E31" s="107" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F31" s="106" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G31" s="107" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="H31" s="106" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="I31" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J31" s="106" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="K31" s="107" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="L31" s="106">
         <v>4</v>
@@ -4275,7 +4271,7 @@
         <v>100</v>
       </c>
       <c r="O31" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P31" s="108">
         <v>5.4999999999999997E-3</v>
@@ -4293,31 +4289,31 @@
         <v>23</v>
       </c>
       <c r="C32" s="101" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E32" s="103" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F32" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G32" s="103" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H32" s="102" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I32" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J32" s="102" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="K32" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L32" s="102">
         <v>1</v>
@@ -4330,7 +4326,7 @@
         <v>30</v>
       </c>
       <c r="O32" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P32" s="95">
         <v>4.87E-2</v>
@@ -4348,31 +4344,31 @@
         <v>24</v>
       </c>
       <c r="C33" s="105" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D33" s="106" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E33" s="107" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F33" s="106" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="G33" s="107" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="H33" s="106" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="I33" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J33" s="106" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="K33" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L33" s="106">
         <v>1</v>
@@ -4385,7 +4381,7 @@
         <v>30</v>
       </c>
       <c r="O33" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P33" s="108">
         <v>7.4300000000000005E-2</v>
@@ -4403,31 +4399,31 @@
         <v>25</v>
       </c>
       <c r="C34" s="101" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D34" s="102" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="E34" s="103" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F34" s="102" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="G34" s="103" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="H34" s="102" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="I34" s="102" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="J34" s="102" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="K34" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L34" s="102">
         <v>2</v>
@@ -4440,7 +4436,7 @@
         <v>60</v>
       </c>
       <c r="O34" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P34" s="95">
         <v>2.8899999999999999E-2</v>
@@ -4458,31 +4454,31 @@
         <v>26</v>
       </c>
       <c r="C35" s="88" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D35" s="89" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="E35" s="90" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F35" s="89" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="G35" s="117" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="H35" s="89" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="I35" s="89" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="J35" s="89" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="K35" s="90" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L35" s="91">
         <v>8</v>
@@ -4495,7 +4491,7 @@
         <v>170</v>
       </c>
       <c r="O35" s="94" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P35" s="92">
         <v>0.12590000000000001</v>
@@ -4505,7 +4501,7 @@
         <v>21.403000000000002</v>
       </c>
       <c r="R35" s="83" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="U35" s="115"/>
     </row>
@@ -4516,31 +4512,31 @@
         <v>27</v>
       </c>
       <c r="C36" s="101" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="D36" s="102" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E36" s="103" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F36" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G36" s="118" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H36" s="102" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="I36" s="102" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="J36" s="102" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="K36" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L36" s="102">
         <v>1</v>
@@ -4553,7 +4549,7 @@
         <v>30</v>
       </c>
       <c r="O36" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P36" s="95">
         <v>5.6000000000000001E-2</v>
@@ -4571,31 +4567,31 @@
         <v>28</v>
       </c>
       <c r="C37" s="105" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="D37" s="106" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E37" s="107" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F37" s="106" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="G37" s="107" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H37" s="106" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I37" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J37" s="106" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="K37" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L37" s="106">
         <v>4</v>
@@ -4608,7 +4604,7 @@
         <v>100</v>
       </c>
       <c r="O37" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P37" s="108">
         <v>2.9499999999999998E-2</v>
@@ -4626,31 +4622,31 @@
         <v>29</v>
       </c>
       <c r="C38" s="101" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="D38" s="102" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38" s="103" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F38" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G38" s="118" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="H38" s="102" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I38" s="102" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="J38" s="102" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="K38" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L38" s="102">
         <v>1</v>
@@ -4663,7 +4659,7 @@
         <v>21</v>
       </c>
       <c r="O38" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P38" s="95">
         <v>0.53559999999999997</v>
@@ -4681,31 +4677,31 @@
         <v>30</v>
       </c>
       <c r="C39" s="105" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="D39" s="106" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E39" s="107" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F39" s="106" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G39" s="119" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H39" s="106" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="I39" s="106" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="J39" s="106" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="K39" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L39" s="106">
         <v>2</v>
@@ -4718,7 +4714,7 @@
         <v>42</v>
       </c>
       <c r="O39" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P39" s="108">
         <v>0.65639999999999998</v>
@@ -4736,31 +4732,31 @@
         <v>31</v>
       </c>
       <c r="C40" s="101" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D40" s="102" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E40" s="103" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F40" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G40" s="103" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H40" s="102" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="I40" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J40" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K40" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L40" s="102">
         <v>1</v>
@@ -4773,7 +4769,7 @@
         <v>21</v>
       </c>
       <c r="O40" s="104" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="P40" s="95">
         <v>1.2</v>
@@ -4791,31 +4787,31 @@
         <v>32</v>
       </c>
       <c r="C41" s="105" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D41" s="106" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E41" s="107" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F41" s="106" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G41" s="107" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H41" s="106" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="I41" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J41" s="106" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="K41" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L41" s="106">
         <v>1</v>
@@ -4828,7 +4824,7 @@
         <v>25</v>
       </c>
       <c r="O41" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P41" s="108">
         <v>9.2200000000000004E-2</v>
@@ -4846,31 +4842,31 @@
         <v>33</v>
       </c>
       <c r="C42" s="105" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D42" s="106" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="E42" s="107" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="F42" s="106" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G42" s="107" t="s">
-        <v>473</v>
+        <v>465</v>
       </c>
       <c r="H42" s="106" t="s">
-        <v>475</v>
+        <v>467</v>
       </c>
       <c r="I42" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J42" s="106" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
       <c r="K42" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L42" s="106">
         <v>1</v>
@@ -4883,7 +4879,7 @@
         <v>25</v>
       </c>
       <c r="O42" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P42" s="108">
         <v>0.21210000000000001</v>
@@ -4901,31 +4897,31 @@
         <v>34</v>
       </c>
       <c r="C43" s="101" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="D43" s="102" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E43" s="103" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F43" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G43" s="103" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="H43" s="102" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I43" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J43" s="102" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="K43" s="103" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="L43" s="102">
         <v>1</v>
@@ -4938,7 +4934,7 @@
         <v>21</v>
       </c>
       <c r="O43" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P43" s="95">
         <v>0.45629999999999998</v>
@@ -4956,31 +4952,31 @@
         <v>35</v>
       </c>
       <c r="C44" s="105" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="D44" s="106" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E44" s="107" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="F44" s="106" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G44" s="107" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
       <c r="H44" s="106" t="s">
-        <v>435</v>
+        <v>428</v>
       </c>
       <c r="I44" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J44" s="106" t="s">
-        <v>436</v>
+        <v>429</v>
       </c>
       <c r="K44" s="107" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="L44" s="106">
         <v>1</v>
@@ -4993,7 +4989,7 @@
         <v>25</v>
       </c>
       <c r="O44" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P44" s="108">
         <v>0.1012</v>
@@ -5011,31 +5007,31 @@
         <v>36</v>
       </c>
       <c r="C45" s="101" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D45" s="102" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E45" s="103" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F45" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G45" s="103" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="H45" s="102" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="I45" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J45" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K45" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L45" s="102">
         <v>1</v>
@@ -5048,7 +5044,7 @@
         <v>30</v>
       </c>
       <c r="O45" s="104" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="P45" s="95">
         <v>0.156</v>
@@ -5066,31 +5062,31 @@
         <v>37</v>
       </c>
       <c r="C46" s="105" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D46" s="106" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E46" s="107" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F46" s="106" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="G46" s="107" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H46" s="106" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="I46" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J46" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K46" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L46" s="106">
         <v>1</v>
@@ -5103,7 +5099,7 @@
         <v>30</v>
       </c>
       <c r="O46" s="109" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="P46" s="108">
         <v>0.08</v>
@@ -5121,31 +5117,31 @@
         <v>38</v>
       </c>
       <c r="C47" s="105" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="D47" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="E47" s="107" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="F47" s="106" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G47" s="107" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="H47" s="106" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="I47" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J47" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K47" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L47" s="106">
         <v>1</v>
@@ -5158,7 +5154,7 @@
         <v>20</v>
       </c>
       <c r="O47" s="109" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="P47" s="108">
         <v>0.435</v>
@@ -5168,7 +5164,7 @@
         <v>8.6999999999999993</v>
       </c>
       <c r="R47" s="78" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
     </row>
     <row r="48" spans="1:21" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5178,31 +5174,31 @@
         <v>39</v>
       </c>
       <c r="C48" s="101" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="D48" s="102" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E48" s="103" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F48" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G48" s="103" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="H48" s="102" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="I48" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J48" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K48" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L48" s="102">
         <v>2</v>
@@ -5215,7 +5211,7 @@
         <v>50</v>
       </c>
       <c r="O48" s="104" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="P48" s="95">
         <v>1.5</v>
@@ -5233,27 +5229,27 @@
         <v>40</v>
       </c>
       <c r="C49" s="96" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D49" s="97" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E49" s="98" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F49" s="97" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G49" s="98" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="H49" s="97" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I49" s="97"/>
       <c r="J49" s="97"/>
       <c r="K49" s="98" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L49" s="97">
         <v>4</v>
@@ -5273,7 +5269,7 @@
         <v>0</v>
       </c>
       <c r="R49" s="65" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="50" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5283,31 +5279,31 @@
         <v>41</v>
       </c>
       <c r="C50" s="101" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D50" s="102" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E50" s="103" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F50" s="102" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G50" s="118">
         <v>61300211121</v>
       </c>
       <c r="H50" s="102" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="I50" s="102" t="s">
-        <v>481</v>
+        <v>473</v>
       </c>
       <c r="J50" s="102" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
       <c r="K50" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L50" s="102">
         <v>4</v>
@@ -5320,7 +5316,7 @@
         <v>100</v>
       </c>
       <c r="O50" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P50" s="95">
         <v>1.47E-2</v>
@@ -5338,31 +5334,31 @@
         <v>42</v>
       </c>
       <c r="C51" s="105" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D51" s="106" t="s">
-        <v>438</v>
+        <v>431</v>
       </c>
       <c r="E51" s="107" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F51" s="106" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G51" s="119" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="H51" s="106" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="I51" s="106" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="J51" s="106" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="K51" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L51" s="106">
         <v>4</v>
@@ -5375,7 +5371,7 @@
         <v>85</v>
       </c>
       <c r="O51" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P51" s="108">
         <v>0.21740000000000001</v>
@@ -5393,31 +5389,31 @@
         <v>43</v>
       </c>
       <c r="C52" s="101" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D52" s="102" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E52" s="103" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F52" s="102" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G52" s="103" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H52" s="102" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I52" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J52" s="102" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="K52" s="103" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="L52" s="102">
         <v>2</v>
@@ -5430,7 +5426,7 @@
         <v>100</v>
       </c>
       <c r="O52" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P52" s="95">
         <v>1E-3</v>
@@ -5448,31 +5444,31 @@
         <v>44</v>
       </c>
       <c r="C53" s="105" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D53" s="106" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E53" s="107" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F53" s="106" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G53" s="107" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H53" s="106" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I53" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J53" s="106" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="K53" s="107" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="L53" s="106">
         <v>1</v>
@@ -5485,7 +5481,7 @@
         <v>100</v>
       </c>
       <c r="O53" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P53" s="108">
         <v>1.4E-3</v>
@@ -5503,31 +5499,31 @@
         <v>45</v>
       </c>
       <c r="C54" s="101" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D54" s="102" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E54" s="103" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F54" s="102" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G54" s="103" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H54" s="102" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="I54" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J54" s="102" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="K54" s="103" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="L54" s="102">
         <v>1</v>
@@ -5540,7 +5536,7 @@
         <v>100</v>
       </c>
       <c r="O54" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P54" s="95">
         <v>1.6000000000000001E-3</v>
@@ -5558,31 +5554,31 @@
         <v>46</v>
       </c>
       <c r="C55" s="105" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D55" s="106" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E55" s="107" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F55" s="106" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G55" s="107" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H55" s="106" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I55" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J55" s="106" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="K55" s="107" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="L55" s="106">
         <v>2</v>
@@ -5595,7 +5591,7 @@
         <v>100</v>
       </c>
       <c r="O55" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P55" s="108">
         <v>1.4E-3</v>
@@ -5613,31 +5609,31 @@
         <v>47</v>
       </c>
       <c r="C56" s="101" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D56" s="102" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E56" s="103" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F56" s="102" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G56" s="103" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H56" s="102" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I56" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J56" s="102" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="K56" s="103" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="L56" s="102">
         <v>4</v>
@@ -5650,7 +5646,7 @@
         <v>100</v>
       </c>
       <c r="O56" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P56" s="95">
         <v>1.2999999999999999E-3</v>
@@ -5661,58 +5657,58 @@
       </c>
       <c r="R56" s="95"/>
     </row>
-    <row r="57" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="53">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="C57" s="105" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D57" s="106" t="s">
-        <v>41</v>
-      </c>
-      <c r="E57" s="107" t="s">
-        <v>110</v>
+        <v>477</v>
+      </c>
+      <c r="E57" s="39" t="s">
+        <v>478</v>
       </c>
       <c r="F57" s="106" t="s">
-        <v>167</v>
-      </c>
-      <c r="G57" s="119" t="s">
-        <v>329</v>
+        <v>164</v>
+      </c>
+      <c r="G57" s="106" t="s">
+        <v>479</v>
       </c>
       <c r="H57" s="106" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="I57" s="106" t="s">
-        <v>391</v>
+        <v>310</v>
       </c>
       <c r="J57" s="106" t="s">
-        <v>392</v>
+        <v>480</v>
       </c>
       <c r="K57" s="107" t="s">
-        <v>289</v>
+        <v>481</v>
       </c>
       <c r="L57" s="106">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M57" s="108">
         <f t="shared" si="1"/>
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="N57" s="108">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="O57" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P57" s="108">
-        <v>6.4500000000000002E-2</v>
+        <v>2.9100000000000001E-2</v>
       </c>
       <c r="Q57" s="108">
         <f t="shared" ref="Q57" si="45">P57*N57</f>
-        <v>5.8049999999999997</v>
+        <v>1.3095000000000001</v>
       </c>
       <c r="R57" s="108"/>
     </row>
@@ -5723,31 +5719,31 @@
         <v>49</v>
       </c>
       <c r="C58" s="60" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D58" s="37" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
       <c r="E58" s="37" t="s">
-        <v>439</v>
+        <v>432</v>
       </c>
       <c r="F58" s="37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G58" s="37" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="H58" s="37" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="I58" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J58" s="37" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="K58" s="37" t="s">
-        <v>426</v>
+        <v>419</v>
       </c>
       <c r="L58" s="37">
         <v>8</v>
@@ -5760,7 +5756,7 @@
         <v>100</v>
       </c>
       <c r="O58" s="79" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P58" s="37">
         <v>1.1000000000000001E-3</v>
@@ -5778,31 +5774,31 @@
         <v>50</v>
       </c>
       <c r="C59" s="105" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D59" s="106" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E59" s="107" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F59" s="106" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G59" s="107" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="H59" s="106" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="I59" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J59" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K59" s="107" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="L59" s="106">
         <v>1</v>
@@ -5815,7 +5811,7 @@
         <v>30</v>
       </c>
       <c r="O59" s="109" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="P59" s="108">
         <v>1.8589999999999999E-2</v>
@@ -5833,31 +5829,31 @@
         <v>51</v>
       </c>
       <c r="C60" s="101" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D60" s="102" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E60" s="103" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F60" s="102" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G60" s="103" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H60" s="102" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I60" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J60" s="102" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="K60" s="103" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="L60" s="102">
         <v>1</v>
@@ -5870,7 +5866,7 @@
         <v>100</v>
       </c>
       <c r="O60" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P60" s="95">
         <v>1.4E-3</v>
@@ -5888,31 +5884,31 @@
         <v>52</v>
       </c>
       <c r="C61" s="105" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D61" s="106" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E61" s="107" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F61" s="106" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G61" s="107" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H61" s="106" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="I61" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J61" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K61" s="107" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="L61" s="106">
         <v>1</v>
@@ -5925,7 +5921,7 @@
         <v>50</v>
       </c>
       <c r="O61" s="109" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="P61" s="108">
         <v>4.6699999999999997E-3</v>
@@ -5943,31 +5939,31 @@
         <v>53</v>
       </c>
       <c r="C62" s="101" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D62" s="102" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E62" s="103" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F62" s="102" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G62" s="103" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="H62" s="102" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I62" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J62" s="102" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="K62" s="103" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="L62" s="102">
         <v>1</v>
@@ -5980,7 +5976,7 @@
         <v>100</v>
       </c>
       <c r="O62" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P62" s="95">
         <v>1.1999999999999999E-3</v>
@@ -5998,31 +5994,31 @@
         <v>54</v>
       </c>
       <c r="C63" s="105" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D63" s="106" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E63" s="107" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F63" s="106" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G63" s="107" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="H63" s="106" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="I63" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J63" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K63" s="107" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="L63" s="106">
         <v>1</v>
@@ -6035,7 +6031,7 @@
         <v>50</v>
       </c>
       <c r="O63" s="109" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="P63" s="108">
         <v>1.11E-2</v>
@@ -6053,31 +6049,31 @@
         <v>55</v>
       </c>
       <c r="C64" s="101" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D64" s="102" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E64" s="103" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F64" s="102" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G64" s="103" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H64" s="102" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I64" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J64" s="102" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="K64" s="103" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="L64" s="102">
         <v>1</v>
@@ -6090,7 +6086,7 @@
         <v>100</v>
       </c>
       <c r="O64" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P64" s="95">
         <v>2.0999999999999999E-3</v>
@@ -6108,31 +6104,31 @@
         <v>56</v>
       </c>
       <c r="C65" s="105" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D65" s="106" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E65" s="107" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F65" s="106" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G65" s="107" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="H65" s="106" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I65" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J65" s="106" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="K65" s="107" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="L65" s="106">
         <v>1</v>
@@ -6145,7 +6141,7 @@
         <v>100</v>
       </c>
       <c r="O65" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P65" s="108">
         <v>1.6000000000000001E-3</v>
@@ -6163,31 +6159,31 @@
         <v>57</v>
       </c>
       <c r="C66" s="101" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D66" s="102" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E66" s="103" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F66" s="102" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G66" s="118" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="H66" s="102" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I66" s="102" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="J66" s="102" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="K66" s="103" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="L66" s="102">
         <v>1</v>
@@ -6200,7 +6196,7 @@
         <v>50</v>
       </c>
       <c r="O66" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P66" s="95">
         <v>6.8999999999999999E-3</v>
@@ -6218,31 +6214,31 @@
         <v>58</v>
       </c>
       <c r="C67" s="105" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D67" s="106" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
       <c r="E67" s="107" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F67" s="106" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G67" s="107" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="H67" s="106" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I67" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J67" s="106" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="K67" s="107" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="L67" s="106">
         <v>2</v>
@@ -6255,7 +6251,7 @@
         <v>100</v>
       </c>
       <c r="O67" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P67" s="108">
         <v>1.1000000000000001E-3</v>
@@ -6273,31 +6269,31 @@
         <v>59</v>
       </c>
       <c r="C68" s="60" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D68" s="37" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E68" s="38" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F68" s="37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G68" s="38" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="H68" s="37" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I68" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J68" s="37" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="K68" s="38" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="L68" s="37">
         <v>2</v>
@@ -6310,7 +6306,7 @@
         <v>100</v>
       </c>
       <c r="O68" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P68" s="41">
         <v>1.5E-3</v>
@@ -6328,29 +6324,29 @@
         <v>60</v>
       </c>
       <c r="C69" s="59" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D69" s="86" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="E69" s="40" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F69" s="39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G69" s="40" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="H69" s="39" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I69" s="39"/>
       <c r="J69" s="39" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="K69" s="40" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="L69" s="39">
         <v>1</v>
@@ -6363,7 +6359,7 @@
         <v>100</v>
       </c>
       <c r="O69" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P69" s="42">
         <v>1.5E-3</v>
@@ -6381,31 +6377,31 @@
         <v>61</v>
       </c>
       <c r="C70" s="60" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D70" s="37" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E70" s="38" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F70" s="37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G70" s="38" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="H70" s="37" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I70" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J70" s="37" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="K70" s="38" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="L70" s="37">
         <v>2</v>
@@ -6418,7 +6414,7 @@
         <v>100</v>
       </c>
       <c r="O70" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P70" s="41">
         <v>1.5E-3</v>
@@ -6436,31 +6432,31 @@
         <v>62</v>
       </c>
       <c r="C71" s="59" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D71" s="39" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E71" s="40" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F71" s="39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G71" s="40" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="H71" s="39" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="I71" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J71" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K71" s="40" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="L71" s="39">
         <v>1</v>
@@ -6473,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="O71" s="64" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="P71" s="42">
         <v>8.5400000000000004E-2</v>
@@ -6491,31 +6487,31 @@
         <v>63</v>
       </c>
       <c r="C72" s="60" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D72" s="37" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E72" s="38" t="s">
-        <v>433</v>
+        <v>426</v>
       </c>
       <c r="F72" s="85" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G72" s="38" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
       <c r="H72" s="37" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="I72" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J72" s="37" t="s">
-        <v>434</v>
+        <v>427</v>
       </c>
       <c r="K72" s="38" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="L72" s="37">
         <v>1</v>
@@ -6528,7 +6524,7 @@
         <v>50</v>
       </c>
       <c r="O72" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P72" s="41">
         <v>3.8E-3</v>
@@ -6546,31 +6542,31 @@
         <v>64</v>
       </c>
       <c r="C73" s="59" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D73" s="39" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="E73" s="40" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F73" s="39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G73" s="40" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="H73" s="39" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I73" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J73" s="39" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="K73" s="40" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="L73" s="39">
         <v>6</v>
@@ -6583,7 +6579,7 @@
         <v>200</v>
       </c>
       <c r="O73" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P73" s="42">
         <v>1.1999999999999999E-3</v>
@@ -6601,31 +6597,31 @@
         <v>65</v>
       </c>
       <c r="C74" s="60" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D74" s="37" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E74" s="38" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="F74" s="37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G74" s="38" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="H74" s="37" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="I74" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J74" s="37" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="K74" s="38" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="L74" s="37">
         <v>1</v>
@@ -6638,7 +6634,7 @@
         <v>100</v>
       </c>
       <c r="O74" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P74" s="41">
         <v>1E-3</v>
@@ -6656,31 +6652,31 @@
         <v>66</v>
       </c>
       <c r="C75" s="59" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D75" s="39" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E75" s="40" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F75" s="39" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G75" s="40" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="H75" s="39" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="I75" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J75" s="39" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="K75" s="40" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="L75" s="39">
         <v>1</v>
@@ -6693,7 +6689,7 @@
         <v>50</v>
       </c>
       <c r="O75" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P75" s="42">
         <v>4.3E-3</v>
@@ -6711,31 +6707,31 @@
         <v>67</v>
       </c>
       <c r="C76" s="96" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D76" s="97" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E76" s="98" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F76" s="97" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G76" s="98" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="H76" s="97" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I76" s="97" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J76" s="97" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="K76" s="98" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="L76" s="97">
         <v>4</v>
@@ -6748,7 +6744,7 @@
         <v>100</v>
       </c>
       <c r="O76" s="99" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P76" s="65">
         <v>1.1999999999999999E-3</v>
@@ -6758,7 +6754,7 @@
         <v>0.12</v>
       </c>
       <c r="R76" s="65" t="s">
-        <v>451</v>
+        <v>443</v>
       </c>
     </row>
     <row r="77" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6768,31 +6764,31 @@
         <v>68</v>
       </c>
       <c r="C77" s="96" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D77" s="122" t="s">
-        <v>479</v>
+        <v>471</v>
       </c>
       <c r="E77" s="98" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F77" s="97" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="G77" s="98" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="H77" s="97" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I77" s="97" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J77" s="97" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K77" s="98" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L77" s="97">
         <v>11</v>
@@ -6812,7 +6808,7 @@
         <v>0</v>
       </c>
       <c r="R77" s="65" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="78" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6822,31 +6818,31 @@
         <v>69</v>
       </c>
       <c r="C78" s="101" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="D78" s="102" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E78" s="103" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F78" s="102" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="G78" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="H78" s="102" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="I78" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J78" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K78" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L78" s="102">
         <v>1</v>
@@ -6860,7 +6856,7 @@
         <v>22</v>
       </c>
       <c r="O78" s="104" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
       <c r="P78" s="95">
         <v>1.42</v>
@@ -6877,31 +6873,31 @@
         <v>70</v>
       </c>
       <c r="C79" s="105" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="D79" s="106" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E79" s="107" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F79" s="106" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G79" s="107">
         <v>750314597</v>
       </c>
       <c r="H79" s="106" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="I79" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J79" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K79" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L79" s="106">
         <v>1</v>
@@ -6914,7 +6910,7 @@
         <v>21</v>
       </c>
       <c r="O79" s="109" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="P79" s="108">
         <v>3.81</v>
@@ -6932,31 +6928,31 @@
         <v>71</v>
       </c>
       <c r="C80" s="101" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D80" s="102" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E80" s="103" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F80" s="102" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G80" s="103" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="H80" s="102" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="I80" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J80" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K80" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L80" s="102">
         <v>1</v>
@@ -6969,7 +6965,7 @@
         <v>21</v>
       </c>
       <c r="O80" s="104" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="P80" s="95">
         <v>2.48</v>
@@ -6987,31 +6983,31 @@
         <v>72</v>
       </c>
       <c r="C81" s="105" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D81" s="106" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E81" s="107" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F81" s="106" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="G81" s="119" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="H81" s="106" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="I81" s="106" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="J81" s="106" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="K81" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L81" s="106">
         <v>1</v>
@@ -7024,7 +7020,7 @@
         <v>21</v>
       </c>
       <c r="O81" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P81" s="108">
         <v>1.3939999999999999</v>
@@ -7042,31 +7038,31 @@
         <v>73</v>
       </c>
       <c r="C82" s="101" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D82" s="102" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E82" s="103" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="F82" s="102" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="G82" s="118" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="H82" s="102" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="I82" s="102" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="J82" s="102" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="K82" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L82" s="102">
         <v>1</v>
@@ -7079,7 +7075,7 @@
         <v>21</v>
       </c>
       <c r="O82" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P82" s="95">
         <v>0.69430000000000003</v>
@@ -7097,31 +7093,31 @@
         <v>74</v>
       </c>
       <c r="C83" s="105" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D83" s="106" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E83" s="107" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="F83" s="106" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="G83" s="107" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H83" s="106" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="I83" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J83" s="106" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K83" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L83" s="106">
         <v>1</v>
@@ -7134,7 +7130,7 @@
         <v>21</v>
       </c>
       <c r="O83" s="109" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="P83" s="108">
         <v>3.637</v>
@@ -7152,31 +7148,31 @@
         <v>75</v>
       </c>
       <c r="C84" s="101" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D84" s="102" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E84" s="103" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F84" s="102" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G84" s="103" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H84" s="102" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="I84" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J84" s="102" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="K84" s="103" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L84" s="102">
         <v>1</v>
@@ -7189,7 +7185,7 @@
         <v>21</v>
       </c>
       <c r="O84" s="104" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P84" s="95">
         <v>0.43280000000000002</v>
@@ -7207,31 +7203,31 @@
         <v>76</v>
       </c>
       <c r="C85" s="70" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D85" s="71" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E85" s="72" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F85" s="71" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="G85" s="72" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H85" s="71" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="I85" s="71" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J85" s="71" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
       <c r="K85" s="72" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L85" s="71">
         <v>1</v>
@@ -7244,7 +7240,7 @@
         <v>21</v>
       </c>
       <c r="O85" s="74" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P85" s="73">
         <v>7.4638</v>
@@ -7254,7 +7250,7 @@
         <v>156.7398</v>
       </c>
       <c r="R85" s="73" t="s">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="U85" s="114"/>
     </row>
@@ -7265,31 +7261,31 @@
         <v>77</v>
       </c>
       <c r="C86" s="101" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D86" s="102" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E86" s="103" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F86" s="102" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="G86" s="103" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="H86" s="102" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I86" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J86" s="102" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K86" s="112" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L86" s="102">
         <v>1</v>
@@ -7302,7 +7298,7 @@
         <v>21</v>
       </c>
       <c r="O86" s="104" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="P86" s="95">
         <v>2.6459999999999999</v>
@@ -7320,31 +7316,31 @@
         <v>78</v>
       </c>
       <c r="C87" s="105" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D87" s="106" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="E87" s="107" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F87" s="106" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G87" s="119" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="H87" s="106" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="I87" s="106" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="J87" s="106" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="K87" s="107" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L87" s="113">
         <v>2</v>
@@ -7357,7 +7353,7 @@
         <v>42</v>
       </c>
       <c r="O87" s="109" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P87" s="108">
         <v>2.2974000000000001</v>
@@ -7375,31 +7371,31 @@
         <v>79</v>
       </c>
       <c r="C88" s="60" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D88" s="37" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E88" s="38" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F88" s="37" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="G88" s="38" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H88" s="37" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="I88" s="62" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J88" s="62" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="K88" s="38" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L88" s="37">
         <v>1</v>
@@ -7412,7 +7408,7 @@
         <v>21</v>
       </c>
       <c r="O88" s="63" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P88" s="41">
         <v>0.39140000000000003</v>
@@ -7430,31 +7426,31 @@
         <v>80</v>
       </c>
       <c r="C89" s="59" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D89" s="39" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="E89" s="40" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="F89" s="39" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="G89" s="121" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="H89" s="39" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I89" s="39" t="s">
-        <v>417</v>
+        <v>410</v>
       </c>
       <c r="J89" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K89" s="40" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="L89" s="39">
         <v>1</v>
@@ -7467,7 +7463,7 @@
         <v>21</v>
       </c>
       <c r="O89" s="64" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="P89" s="42">
         <v>3.532</v>
@@ -7485,28 +7481,28 @@
         <v>81</v>
       </c>
       <c r="C90" s="59" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
       <c r="D90" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="E90" s="40" t="s">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="F90" s="39" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G90" s="40" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="H90" s="39" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="I90" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J90" s="39" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="K90" s="40"/>
       <c r="L90" s="39">
@@ -7520,7 +7516,7 @@
         <v>25</v>
       </c>
       <c r="O90" s="64" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="P90" s="42">
         <v>8.8999999999999996E-2</v>
@@ -7549,12 +7545,12 @@
       <c r="M91" s="36"/>
       <c r="N91" s="36"/>
       <c r="O91" s="68" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="P91" s="66"/>
       <c r="Q91" s="66">
         <f>SUM(Q10:Q90)</f>
-        <v>970.9928000000001</v>
+        <v>966.49730000000011</v>
       </c>
       <c r="R91" s="44"/>
     </row>
@@ -7576,12 +7572,12 @@
       <c r="M92" s="9"/>
       <c r="N92" s="9"/>
       <c r="O92" s="69" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="P92" s="67"/>
       <c r="Q92" s="67">
         <f>Q91/20</f>
-        <v>48.549640000000004</v>
+        <v>48.324865000000003</v>
       </c>
       <c r="R92" s="45"/>
     </row>
@@ -7591,84 +7587,84 @@
     <mergeCell ref="R3:R8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O11" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="O12" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="O13" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="O14" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="O15" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="O16" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="O17" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="O18" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="O19" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="O20" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="O21" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="O22" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="O23" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="O24" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="O25" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="O26" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="O27" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="O28" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="O29" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="O30" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="O31" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="O32" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="O33" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="O34" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="O35" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="O36" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="O37" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="O38" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="O39" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="O40" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="O41" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="O43" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="O44" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="O45" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="O46" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="O48" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="O51" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="O52" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="O53" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="O54" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="O55" r:id="rId41" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="O56" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="O57" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="O69" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="O59" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="O60" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="O61" r:id="rId47" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="O62" r:id="rId48" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="O63" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="O64" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="O65" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="O66" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="O67" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="O68" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="O70" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="O71" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="O72" r:id="rId57" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="O75" r:id="rId58" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="O76" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="O73" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="O79" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="O80" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="O81" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="O82" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="O83" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="O84" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="O85" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="O86" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="O87" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="O89" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="O88" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="O58" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="O47" r:id="rId73" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="O90" r:id="rId74" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="O42" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="O10" r:id="rId76" xr:uid="{5D88A11D-3624-47E9-BBD7-2366F8BA7980}"/>
-    <hyperlink ref="O50" r:id="rId77" xr:uid="{3AF3C69B-110E-4BD5-B2CB-21B12CDADF8A}"/>
-    <hyperlink ref="O78" r:id="rId78" xr:uid="{D0B601F1-C091-44E0-B215-033F4B4B50D1}"/>
+    <hyperlink ref="O11" r:id="rId1"/>
+    <hyperlink ref="O12" r:id="rId2"/>
+    <hyperlink ref="O13" r:id="rId3"/>
+    <hyperlink ref="O14" r:id="rId4"/>
+    <hyperlink ref="O15" r:id="rId5"/>
+    <hyperlink ref="O16" r:id="rId6"/>
+    <hyperlink ref="O17" r:id="rId7"/>
+    <hyperlink ref="O18" r:id="rId8"/>
+    <hyperlink ref="O19" r:id="rId9"/>
+    <hyperlink ref="O20" r:id="rId10"/>
+    <hyperlink ref="O21" r:id="rId11"/>
+    <hyperlink ref="O22" r:id="rId12"/>
+    <hyperlink ref="O23" r:id="rId13"/>
+    <hyperlink ref="O24" r:id="rId14"/>
+    <hyperlink ref="O25" r:id="rId15"/>
+    <hyperlink ref="O26" r:id="rId16"/>
+    <hyperlink ref="O27" r:id="rId17"/>
+    <hyperlink ref="O28" r:id="rId18"/>
+    <hyperlink ref="O29" r:id="rId19"/>
+    <hyperlink ref="O30" r:id="rId20"/>
+    <hyperlink ref="O31" r:id="rId21"/>
+    <hyperlink ref="O32" r:id="rId22"/>
+    <hyperlink ref="O33" r:id="rId23"/>
+    <hyperlink ref="O34" r:id="rId24"/>
+    <hyperlink ref="O35" r:id="rId25"/>
+    <hyperlink ref="O36" r:id="rId26"/>
+    <hyperlink ref="O37" r:id="rId27"/>
+    <hyperlink ref="O38" r:id="rId28"/>
+    <hyperlink ref="O39" r:id="rId29"/>
+    <hyperlink ref="O40" r:id="rId30"/>
+    <hyperlink ref="O41" r:id="rId31"/>
+    <hyperlink ref="O43" r:id="rId32"/>
+    <hyperlink ref="O44" r:id="rId33"/>
+    <hyperlink ref="O45" r:id="rId34"/>
+    <hyperlink ref="O46" r:id="rId35"/>
+    <hyperlink ref="O48" r:id="rId36"/>
+    <hyperlink ref="O51" r:id="rId37"/>
+    <hyperlink ref="O52" r:id="rId38"/>
+    <hyperlink ref="O53" r:id="rId39"/>
+    <hyperlink ref="O54" r:id="rId40"/>
+    <hyperlink ref="O55" r:id="rId41"/>
+    <hyperlink ref="O56" r:id="rId42"/>
+    <hyperlink ref="O69" r:id="rId43"/>
+    <hyperlink ref="O59" r:id="rId44"/>
+    <hyperlink ref="O60" r:id="rId45"/>
+    <hyperlink ref="O61" r:id="rId46"/>
+    <hyperlink ref="O62" r:id="rId47"/>
+    <hyperlink ref="O63" r:id="rId48"/>
+    <hyperlink ref="O64" r:id="rId49"/>
+    <hyperlink ref="O65" r:id="rId50"/>
+    <hyperlink ref="O66" r:id="rId51"/>
+    <hyperlink ref="O67" r:id="rId52"/>
+    <hyperlink ref="O68" r:id="rId53"/>
+    <hyperlink ref="O70" r:id="rId54"/>
+    <hyperlink ref="O71" r:id="rId55"/>
+    <hyperlink ref="O72" r:id="rId56"/>
+    <hyperlink ref="O75" r:id="rId57"/>
+    <hyperlink ref="O76" r:id="rId58"/>
+    <hyperlink ref="O73" r:id="rId59"/>
+    <hyperlink ref="O79" r:id="rId60"/>
+    <hyperlink ref="O80" r:id="rId61"/>
+    <hyperlink ref="O81" r:id="rId62"/>
+    <hyperlink ref="O82" r:id="rId63"/>
+    <hyperlink ref="O83" r:id="rId64"/>
+    <hyperlink ref="O84" r:id="rId65"/>
+    <hyperlink ref="O85" r:id="rId66"/>
+    <hyperlink ref="O86" r:id="rId67"/>
+    <hyperlink ref="O87" r:id="rId68"/>
+    <hyperlink ref="O89" r:id="rId69"/>
+    <hyperlink ref="O88" r:id="rId70"/>
+    <hyperlink ref="O58" r:id="rId71"/>
+    <hyperlink ref="O47" r:id="rId72"/>
+    <hyperlink ref="O90" r:id="rId73"/>
+    <hyperlink ref="O42" r:id="rId74"/>
+    <hyperlink ref="O10" r:id="rId75"/>
+    <hyperlink ref="O50" r:id="rId76"/>
+    <hyperlink ref="O78" r:id="rId77"/>
+    <hyperlink ref="O57" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId79"/>

</xml_diff>